<commit_message>
vault backup: 2026-04-28 14:46:45
</commit_message>
<xml_diff>
--- a/Knowledge/Model Outputs/CELH/CELH_model.xlsx
+++ b/Knowledge/Model Outputs/CELH/CELH_model.xlsx
@@ -29857,67 +29857,67 @@
         <v/>
       </c>
       <c r="R2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!Q2,'QTR P&amp;L'!N2)*(1+'IS DRIVERS'!R2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!Q2,'QTR P&amp;L'!N2)*(1+'IS DRIVERS'!S2)</f>
         <v/>
       </c>
       <c r="S2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!R2,'QTR P&amp;L'!O2)*(1+'IS DRIVERS'!S2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!R2,'QTR P&amp;L'!O2)*(1+'IS DRIVERS'!T2)</f>
         <v/>
       </c>
       <c r="T2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!S2,'QTR P&amp;L'!P2)*(1+'IS DRIVERS'!T2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!S2,'QTR P&amp;L'!P2)*(1+'IS DRIVERS'!U2)</f>
         <v/>
       </c>
       <c r="U2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!T2,'QTR P&amp;L'!Q2)*(1+'IS DRIVERS'!U2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!T2,'QTR P&amp;L'!Q2)*(1+'IS DRIVERS'!V2)</f>
         <v/>
       </c>
       <c r="V2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!U2,'QTR P&amp;L'!R2)*(1+'IS DRIVERS'!V2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!U2,'QTR P&amp;L'!R2)*(1+'IS DRIVERS'!W2)</f>
         <v/>
       </c>
       <c r="W2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!V2,'QTR P&amp;L'!S2)*(1+'IS DRIVERS'!W2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!V2,'QTR P&amp;L'!S2)*(1+'IS DRIVERS'!X2)</f>
         <v/>
       </c>
       <c r="X2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!W2,'QTR P&amp;L'!T2)*(1+'IS DRIVERS'!X2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!W2,'QTR P&amp;L'!T2)*(1+'IS DRIVERS'!Y2)</f>
         <v/>
       </c>
       <c r="Y2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!X2,'QTR P&amp;L'!U2)*(1+'IS DRIVERS'!Y2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!X2,'QTR P&amp;L'!U2)*(1+'IS DRIVERS'!Z2)</f>
         <v/>
       </c>
       <c r="Z2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!Y2,'QTR P&amp;L'!V2)*(1+'IS DRIVERS'!Z2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!Y2,'QTR P&amp;L'!V2)*(1+'IS DRIVERS'!AA2)</f>
         <v/>
       </c>
       <c r="AA2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!Z2,'QTR P&amp;L'!W2)*(1+'IS DRIVERS'!AA2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!Z2,'QTR P&amp;L'!W2)*(1+'IS DRIVERS'!AB2)</f>
         <v/>
       </c>
       <c r="AB2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!AA2,'QTR P&amp;L'!X2)*(1+'IS DRIVERS'!AB2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!AA2,'QTR P&amp;L'!X2)*(1+'IS DRIVERS'!AC2)</f>
         <v/>
       </c>
       <c r="AC2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!AB2,'QTR P&amp;L'!Y2)*(1+'IS DRIVERS'!AC2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!AB2,'QTR P&amp;L'!Y2)*(1+'IS DRIVERS'!AD2)</f>
         <v/>
       </c>
       <c r="AD2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!AC2,'QTR P&amp;L'!Z2)*(1+'IS DRIVERS'!AD2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!AC2,'QTR P&amp;L'!Z2)*(1+'IS DRIVERS'!AE2)</f>
         <v/>
       </c>
       <c r="AE2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!AD2,'QTR P&amp;L'!AA2)*(1+'IS DRIVERS'!AE2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!AD2,'QTR P&amp;L'!AA2)*(1+'IS DRIVERS'!AF2)</f>
         <v/>
       </c>
       <c r="AF2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!AE2,'QTR P&amp;L'!AB2)*(1+'IS DRIVERS'!AF2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!AE2,'QTR P&amp;L'!AB2)*(1+'IS DRIVERS'!AG2)</f>
         <v/>
       </c>
       <c r="AG2" s="9">
-        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!AF2,'QTR P&amp;L'!AC2)*(1+'IS DRIVERS'!AG2)</f>
+        <f>IF('IS DRIVERS'!$B2="QoQ",'QTR P&amp;L'!AF2,'QTR P&amp;L'!AC2)*(1+'IS DRIVERS'!AH2)</f>
         <v/>
       </c>
     </row>
@@ -29992,67 +29992,67 @@
         <v/>
       </c>
       <c r="R3" s="9">
-        <f>'QTR P&amp;L'!R2*'IS DRIVERS'!R3</f>
+        <f>'QTR P&amp;L'!R2*'IS DRIVERS'!S3</f>
         <v/>
       </c>
       <c r="S3" s="9">
-        <f>'QTR P&amp;L'!S2*'IS DRIVERS'!S3</f>
+        <f>'QTR P&amp;L'!S2*'IS DRIVERS'!T3</f>
         <v/>
       </c>
       <c r="T3" s="9">
-        <f>'QTR P&amp;L'!T2*'IS DRIVERS'!T3</f>
+        <f>'QTR P&amp;L'!T2*'IS DRIVERS'!U3</f>
         <v/>
       </c>
       <c r="U3" s="9">
-        <f>'QTR P&amp;L'!U2*'IS DRIVERS'!U3</f>
+        <f>'QTR P&amp;L'!U2*'IS DRIVERS'!V3</f>
         <v/>
       </c>
       <c r="V3" s="9">
-        <f>'QTR P&amp;L'!V2*'IS DRIVERS'!V3</f>
+        <f>'QTR P&amp;L'!V2*'IS DRIVERS'!W3</f>
         <v/>
       </c>
       <c r="W3" s="9">
-        <f>'QTR P&amp;L'!W2*'IS DRIVERS'!W3</f>
+        <f>'QTR P&amp;L'!W2*'IS DRIVERS'!X3</f>
         <v/>
       </c>
       <c r="X3" s="9">
-        <f>'QTR P&amp;L'!X2*'IS DRIVERS'!X3</f>
+        <f>'QTR P&amp;L'!X2*'IS DRIVERS'!Y3</f>
         <v/>
       </c>
       <c r="Y3" s="9">
-        <f>'QTR P&amp;L'!Y2*'IS DRIVERS'!Y3</f>
+        <f>'QTR P&amp;L'!Y2*'IS DRIVERS'!Z3</f>
         <v/>
       </c>
       <c r="Z3" s="9">
-        <f>'QTR P&amp;L'!Z2*'IS DRIVERS'!Z3</f>
+        <f>'QTR P&amp;L'!Z2*'IS DRIVERS'!AA3</f>
         <v/>
       </c>
       <c r="AA3" s="9">
-        <f>'QTR P&amp;L'!AA2*'IS DRIVERS'!AA3</f>
+        <f>'QTR P&amp;L'!AA2*'IS DRIVERS'!AB3</f>
         <v/>
       </c>
       <c r="AB3" s="9">
-        <f>'QTR P&amp;L'!AB2*'IS DRIVERS'!AB3</f>
+        <f>'QTR P&amp;L'!AB2*'IS DRIVERS'!AC3</f>
         <v/>
       </c>
       <c r="AC3" s="9">
-        <f>'QTR P&amp;L'!AC2*'IS DRIVERS'!AC3</f>
+        <f>'QTR P&amp;L'!AC2*'IS DRIVERS'!AD3</f>
         <v/>
       </c>
       <c r="AD3" s="9">
-        <f>'QTR P&amp;L'!AD2*'IS DRIVERS'!AD3</f>
+        <f>'QTR P&amp;L'!AD2*'IS DRIVERS'!AE3</f>
         <v/>
       </c>
       <c r="AE3" s="9">
-        <f>'QTR P&amp;L'!AE2*'IS DRIVERS'!AE3</f>
+        <f>'QTR P&amp;L'!AE2*'IS DRIVERS'!AF3</f>
         <v/>
       </c>
       <c r="AF3" s="9">
-        <f>'QTR P&amp;L'!AF2*'IS DRIVERS'!AF3</f>
+        <f>'QTR P&amp;L'!AF2*'IS DRIVERS'!AG3</f>
         <v/>
       </c>
       <c r="AG3" s="9">
-        <f>'QTR P&amp;L'!AG2*'IS DRIVERS'!AG3</f>
+        <f>'QTR P&amp;L'!AG2*'IS DRIVERS'!AH3</f>
         <v/>
       </c>
     </row>
@@ -30262,67 +30262,67 @@
         <v/>
       </c>
       <c r="R5" s="9">
-        <f>'QTR P&amp;L'!R2*'IS DRIVERS'!R4</f>
+        <f>'QTR P&amp;L'!R2*'IS DRIVERS'!S4</f>
         <v/>
       </c>
       <c r="S5" s="9">
-        <f>'QTR P&amp;L'!S2*'IS DRIVERS'!S4</f>
+        <f>'QTR P&amp;L'!S2*'IS DRIVERS'!T4</f>
         <v/>
       </c>
       <c r="T5" s="9">
-        <f>'QTR P&amp;L'!T2*'IS DRIVERS'!T4</f>
+        <f>'QTR P&amp;L'!T2*'IS DRIVERS'!U4</f>
         <v/>
       </c>
       <c r="U5" s="9">
-        <f>'QTR P&amp;L'!U2*'IS DRIVERS'!U4</f>
+        <f>'QTR P&amp;L'!U2*'IS DRIVERS'!V4</f>
         <v/>
       </c>
       <c r="V5" s="9">
-        <f>'QTR P&amp;L'!V2*'IS DRIVERS'!V4</f>
+        <f>'QTR P&amp;L'!V2*'IS DRIVERS'!W4</f>
         <v/>
       </c>
       <c r="W5" s="9">
-        <f>'QTR P&amp;L'!W2*'IS DRIVERS'!W4</f>
+        <f>'QTR P&amp;L'!W2*'IS DRIVERS'!X4</f>
         <v/>
       </c>
       <c r="X5" s="9">
-        <f>'QTR P&amp;L'!X2*'IS DRIVERS'!X4</f>
+        <f>'QTR P&amp;L'!X2*'IS DRIVERS'!Y4</f>
         <v/>
       </c>
       <c r="Y5" s="9">
-        <f>'QTR P&amp;L'!Y2*'IS DRIVERS'!Y4</f>
+        <f>'QTR P&amp;L'!Y2*'IS DRIVERS'!Z4</f>
         <v/>
       </c>
       <c r="Z5" s="9">
-        <f>'QTR P&amp;L'!Z2*'IS DRIVERS'!Z4</f>
+        <f>'QTR P&amp;L'!Z2*'IS DRIVERS'!AA4</f>
         <v/>
       </c>
       <c r="AA5" s="9">
-        <f>'QTR P&amp;L'!AA2*'IS DRIVERS'!AA4</f>
+        <f>'QTR P&amp;L'!AA2*'IS DRIVERS'!AB4</f>
         <v/>
       </c>
       <c r="AB5" s="9">
-        <f>'QTR P&amp;L'!AB2*'IS DRIVERS'!AB4</f>
+        <f>'QTR P&amp;L'!AB2*'IS DRIVERS'!AC4</f>
         <v/>
       </c>
       <c r="AC5" s="9">
-        <f>'QTR P&amp;L'!AC2*'IS DRIVERS'!AC4</f>
+        <f>'QTR P&amp;L'!AC2*'IS DRIVERS'!AD4</f>
         <v/>
       </c>
       <c r="AD5" s="9">
-        <f>'QTR P&amp;L'!AD2*'IS DRIVERS'!AD4</f>
+        <f>'QTR P&amp;L'!AD2*'IS DRIVERS'!AE4</f>
         <v/>
       </c>
       <c r="AE5" s="9">
-        <f>'QTR P&amp;L'!AE2*'IS DRIVERS'!AE4</f>
+        <f>'QTR P&amp;L'!AE2*'IS DRIVERS'!AF4</f>
         <v/>
       </c>
       <c r="AF5" s="9">
-        <f>'QTR P&amp;L'!AF2*'IS DRIVERS'!AF4</f>
+        <f>'QTR P&amp;L'!AF2*'IS DRIVERS'!AG4</f>
         <v/>
       </c>
       <c r="AG5" s="9">
-        <f>'QTR P&amp;L'!AG2*'IS DRIVERS'!AG4</f>
+        <f>'QTR P&amp;L'!AG2*'IS DRIVERS'!AH4</f>
         <v/>
       </c>
     </row>
@@ -30397,67 +30397,67 @@
         <v/>
       </c>
       <c r="R6" s="9">
-        <f>'IS DRIVERS'!R5</f>
+        <f>'IS DRIVERS'!S5</f>
         <v/>
       </c>
       <c r="S6" s="9">
-        <f>'IS DRIVERS'!S5</f>
+        <f>'IS DRIVERS'!T5</f>
         <v/>
       </c>
       <c r="T6" s="9">
-        <f>'IS DRIVERS'!T5</f>
+        <f>'IS DRIVERS'!U5</f>
         <v/>
       </c>
       <c r="U6" s="9">
-        <f>'IS DRIVERS'!U5</f>
+        <f>'IS DRIVERS'!V5</f>
         <v/>
       </c>
       <c r="V6" s="9">
-        <f>'IS DRIVERS'!V5</f>
+        <f>'IS DRIVERS'!W5</f>
         <v/>
       </c>
       <c r="W6" s="9">
-        <f>'IS DRIVERS'!W5</f>
+        <f>'IS DRIVERS'!X5</f>
         <v/>
       </c>
       <c r="X6" s="9">
-        <f>'IS DRIVERS'!X5</f>
+        <f>'IS DRIVERS'!Y5</f>
         <v/>
       </c>
       <c r="Y6" s="9">
-        <f>'IS DRIVERS'!Y5</f>
+        <f>'IS DRIVERS'!Z5</f>
         <v/>
       </c>
       <c r="Z6" s="9">
-        <f>'IS DRIVERS'!Z5</f>
+        <f>'IS DRIVERS'!AA5</f>
         <v/>
       </c>
       <c r="AA6" s="9">
-        <f>'IS DRIVERS'!AA5</f>
+        <f>'IS DRIVERS'!AB5</f>
         <v/>
       </c>
       <c r="AB6" s="9">
-        <f>'IS DRIVERS'!AB5</f>
+        <f>'IS DRIVERS'!AC5</f>
         <v/>
       </c>
       <c r="AC6" s="9">
-        <f>'IS DRIVERS'!AC5</f>
+        <f>'IS DRIVERS'!AD5</f>
         <v/>
       </c>
       <c r="AD6" s="9">
-        <f>'IS DRIVERS'!AD5</f>
+        <f>'IS DRIVERS'!AE5</f>
         <v/>
       </c>
       <c r="AE6" s="9">
-        <f>'IS DRIVERS'!AE5</f>
+        <f>'IS DRIVERS'!AF5</f>
         <v/>
       </c>
       <c r="AF6" s="9">
-        <f>'IS DRIVERS'!AF5</f>
+        <f>'IS DRIVERS'!AG5</f>
         <v/>
       </c>
       <c r="AG6" s="9">
-        <f>'IS DRIVERS'!AG5</f>
+        <f>'IS DRIVERS'!AH5</f>
         <v/>
       </c>
     </row>
@@ -30667,67 +30667,67 @@
         <v/>
       </c>
       <c r="R8" s="9">
-        <f>'IS DRIVERS'!R6</f>
+        <f>'IS DRIVERS'!S6</f>
         <v/>
       </c>
       <c r="S8" s="9">
-        <f>'IS DRIVERS'!S6</f>
+        <f>'IS DRIVERS'!T6</f>
         <v/>
       </c>
       <c r="T8" s="9">
-        <f>'IS DRIVERS'!T6</f>
+        <f>'IS DRIVERS'!U6</f>
         <v/>
       </c>
       <c r="U8" s="9">
-        <f>'IS DRIVERS'!U6</f>
+        <f>'IS DRIVERS'!V6</f>
         <v/>
       </c>
       <c r="V8" s="9">
-        <f>'IS DRIVERS'!V6</f>
+        <f>'IS DRIVERS'!W6</f>
         <v/>
       </c>
       <c r="W8" s="9">
-        <f>'IS DRIVERS'!W6</f>
+        <f>'IS DRIVERS'!X6</f>
         <v/>
       </c>
       <c r="X8" s="9">
-        <f>'IS DRIVERS'!X6</f>
+        <f>'IS DRIVERS'!Y6</f>
         <v/>
       </c>
       <c r="Y8" s="9">
-        <f>'IS DRIVERS'!Y6</f>
+        <f>'IS DRIVERS'!Z6</f>
         <v/>
       </c>
       <c r="Z8" s="9">
-        <f>'IS DRIVERS'!Z6</f>
+        <f>'IS DRIVERS'!AA6</f>
         <v/>
       </c>
       <c r="AA8" s="9">
-        <f>'IS DRIVERS'!AA6</f>
+        <f>'IS DRIVERS'!AB6</f>
         <v/>
       </c>
       <c r="AB8" s="9">
-        <f>'IS DRIVERS'!AB6</f>
+        <f>'IS DRIVERS'!AC6</f>
         <v/>
       </c>
       <c r="AC8" s="9">
-        <f>'IS DRIVERS'!AC6</f>
+        <f>'IS DRIVERS'!AD6</f>
         <v/>
       </c>
       <c r="AD8" s="9">
-        <f>'IS DRIVERS'!AD6</f>
+        <f>'IS DRIVERS'!AE6</f>
         <v/>
       </c>
       <c r="AE8" s="9">
-        <f>'IS DRIVERS'!AE6</f>
+        <f>'IS DRIVERS'!AF6</f>
         <v/>
       </c>
       <c r="AF8" s="9">
-        <f>'IS DRIVERS'!AF6</f>
+        <f>'IS DRIVERS'!AG6</f>
         <v/>
       </c>
       <c r="AG8" s="9">
-        <f>'IS DRIVERS'!AG6</f>
+        <f>'IS DRIVERS'!AH6</f>
         <v/>
       </c>
     </row>
@@ -30802,67 +30802,67 @@
         <v/>
       </c>
       <c r="R9" s="9">
-        <f>'IS DRIVERS'!R7</f>
+        <f>'IS DRIVERS'!S7</f>
         <v/>
       </c>
       <c r="S9" s="9">
-        <f>'IS DRIVERS'!S7</f>
+        <f>'IS DRIVERS'!T7</f>
         <v/>
       </c>
       <c r="T9" s="9">
-        <f>'IS DRIVERS'!T7</f>
+        <f>'IS DRIVERS'!U7</f>
         <v/>
       </c>
       <c r="U9" s="9">
-        <f>'IS DRIVERS'!U7</f>
+        <f>'IS DRIVERS'!V7</f>
         <v/>
       </c>
       <c r="V9" s="9">
-        <f>'IS DRIVERS'!V7</f>
+        <f>'IS DRIVERS'!W7</f>
         <v/>
       </c>
       <c r="W9" s="9">
-        <f>'IS DRIVERS'!W7</f>
+        <f>'IS DRIVERS'!X7</f>
         <v/>
       </c>
       <c r="X9" s="9">
-        <f>'IS DRIVERS'!X7</f>
+        <f>'IS DRIVERS'!Y7</f>
         <v/>
       </c>
       <c r="Y9" s="9">
-        <f>'IS DRIVERS'!Y7</f>
+        <f>'IS DRIVERS'!Z7</f>
         <v/>
       </c>
       <c r="Z9" s="9">
-        <f>'IS DRIVERS'!Z7</f>
+        <f>'IS DRIVERS'!AA7</f>
         <v/>
       </c>
       <c r="AA9" s="9">
-        <f>'IS DRIVERS'!AA7</f>
+        <f>'IS DRIVERS'!AB7</f>
         <v/>
       </c>
       <c r="AB9" s="9">
-        <f>'IS DRIVERS'!AB7</f>
+        <f>'IS DRIVERS'!AC7</f>
         <v/>
       </c>
       <c r="AC9" s="9">
-        <f>'IS DRIVERS'!AC7</f>
+        <f>'IS DRIVERS'!AD7</f>
         <v/>
       </c>
       <c r="AD9" s="9">
-        <f>'IS DRIVERS'!AD7</f>
+        <f>'IS DRIVERS'!AE7</f>
         <v/>
       </c>
       <c r="AE9" s="9">
-        <f>'IS DRIVERS'!AE7</f>
+        <f>'IS DRIVERS'!AF7</f>
         <v/>
       </c>
       <c r="AF9" s="9">
-        <f>'IS DRIVERS'!AF7</f>
+        <f>'IS DRIVERS'!AG7</f>
         <v/>
       </c>
       <c r="AG9" s="9">
-        <f>'IS DRIVERS'!AG7</f>
+        <f>'IS DRIVERS'!AH7</f>
         <v/>
       </c>
     </row>
@@ -30937,67 +30937,67 @@
         <v/>
       </c>
       <c r="R10" s="9">
-        <f>'IS DRIVERS'!R8</f>
+        <f>'IS DRIVERS'!S8</f>
         <v/>
       </c>
       <c r="S10" s="9">
-        <f>'IS DRIVERS'!S8</f>
+        <f>'IS DRIVERS'!T8</f>
         <v/>
       </c>
       <c r="T10" s="9">
-        <f>'IS DRIVERS'!T8</f>
+        <f>'IS DRIVERS'!U8</f>
         <v/>
       </c>
       <c r="U10" s="9">
-        <f>'IS DRIVERS'!U8</f>
+        <f>'IS DRIVERS'!V8</f>
         <v/>
       </c>
       <c r="V10" s="9">
-        <f>'IS DRIVERS'!V8</f>
+        <f>'IS DRIVERS'!W8</f>
         <v/>
       </c>
       <c r="W10" s="9">
-        <f>'IS DRIVERS'!W8</f>
+        <f>'IS DRIVERS'!X8</f>
         <v/>
       </c>
       <c r="X10" s="9">
-        <f>'IS DRIVERS'!X8</f>
+        <f>'IS DRIVERS'!Y8</f>
         <v/>
       </c>
       <c r="Y10" s="9">
-        <f>'IS DRIVERS'!Y8</f>
+        <f>'IS DRIVERS'!Z8</f>
         <v/>
       </c>
       <c r="Z10" s="9">
-        <f>'IS DRIVERS'!Z8</f>
+        <f>'IS DRIVERS'!AA8</f>
         <v/>
       </c>
       <c r="AA10" s="9">
-        <f>'IS DRIVERS'!AA8</f>
+        <f>'IS DRIVERS'!AB8</f>
         <v/>
       </c>
       <c r="AB10" s="9">
-        <f>'IS DRIVERS'!AB8</f>
+        <f>'IS DRIVERS'!AC8</f>
         <v/>
       </c>
       <c r="AC10" s="9">
-        <f>'IS DRIVERS'!AC8</f>
+        <f>'IS DRIVERS'!AD8</f>
         <v/>
       </c>
       <c r="AD10" s="9">
-        <f>'IS DRIVERS'!AD8</f>
+        <f>'IS DRIVERS'!AE8</f>
         <v/>
       </c>
       <c r="AE10" s="9">
-        <f>'IS DRIVERS'!AE8</f>
+        <f>'IS DRIVERS'!AF8</f>
         <v/>
       </c>
       <c r="AF10" s="9">
-        <f>'IS DRIVERS'!AF8</f>
+        <f>'IS DRIVERS'!AG8</f>
         <v/>
       </c>
       <c r="AG10" s="9">
-        <f>'IS DRIVERS'!AG8</f>
+        <f>'IS DRIVERS'!AH8</f>
         <v/>
       </c>
     </row>
@@ -31207,67 +31207,67 @@
         <v/>
       </c>
       <c r="R12" s="9">
-        <f>'QTR P&amp;L'!R11*'IS DRIVERS'!R9</f>
+        <f>'QTR P&amp;L'!R11*'IS DRIVERS'!S9</f>
         <v/>
       </c>
       <c r="S12" s="9">
-        <f>'QTR P&amp;L'!S11*'IS DRIVERS'!S9</f>
+        <f>'QTR P&amp;L'!S11*'IS DRIVERS'!T9</f>
         <v/>
       </c>
       <c r="T12" s="9">
-        <f>'QTR P&amp;L'!T11*'IS DRIVERS'!T9</f>
+        <f>'QTR P&amp;L'!T11*'IS DRIVERS'!U9</f>
         <v/>
       </c>
       <c r="U12" s="9">
-        <f>'QTR P&amp;L'!U11*'IS DRIVERS'!U9</f>
+        <f>'QTR P&amp;L'!U11*'IS DRIVERS'!V9</f>
         <v/>
       </c>
       <c r="V12" s="9">
-        <f>'QTR P&amp;L'!V11*'IS DRIVERS'!V9</f>
+        <f>'QTR P&amp;L'!V11*'IS DRIVERS'!W9</f>
         <v/>
       </c>
       <c r="W12" s="9">
-        <f>'QTR P&amp;L'!W11*'IS DRIVERS'!W9</f>
+        <f>'QTR P&amp;L'!W11*'IS DRIVERS'!X9</f>
         <v/>
       </c>
       <c r="X12" s="9">
-        <f>'QTR P&amp;L'!X11*'IS DRIVERS'!X9</f>
+        <f>'QTR P&amp;L'!X11*'IS DRIVERS'!Y9</f>
         <v/>
       </c>
       <c r="Y12" s="9">
-        <f>'QTR P&amp;L'!Y11*'IS DRIVERS'!Y9</f>
+        <f>'QTR P&amp;L'!Y11*'IS DRIVERS'!Z9</f>
         <v/>
       </c>
       <c r="Z12" s="9">
-        <f>'QTR P&amp;L'!Z11*'IS DRIVERS'!Z9</f>
+        <f>'QTR P&amp;L'!Z11*'IS DRIVERS'!AA9</f>
         <v/>
       </c>
       <c r="AA12" s="9">
-        <f>'QTR P&amp;L'!AA11*'IS DRIVERS'!AA9</f>
+        <f>'QTR P&amp;L'!AA11*'IS DRIVERS'!AB9</f>
         <v/>
       </c>
       <c r="AB12" s="9">
-        <f>'QTR P&amp;L'!AB11*'IS DRIVERS'!AB9</f>
+        <f>'QTR P&amp;L'!AB11*'IS DRIVERS'!AC9</f>
         <v/>
       </c>
       <c r="AC12" s="9">
-        <f>'QTR P&amp;L'!AC11*'IS DRIVERS'!AC9</f>
+        <f>'QTR P&amp;L'!AC11*'IS DRIVERS'!AD9</f>
         <v/>
       </c>
       <c r="AD12" s="9">
-        <f>'QTR P&amp;L'!AD11*'IS DRIVERS'!AD9</f>
+        <f>'QTR P&amp;L'!AD11*'IS DRIVERS'!AE9</f>
         <v/>
       </c>
       <c r="AE12" s="9">
-        <f>'QTR P&amp;L'!AE11*'IS DRIVERS'!AE9</f>
+        <f>'QTR P&amp;L'!AE11*'IS DRIVERS'!AF9</f>
         <v/>
       </c>
       <c r="AF12" s="9">
-        <f>'QTR P&amp;L'!AF11*'IS DRIVERS'!AF9</f>
+        <f>'QTR P&amp;L'!AF11*'IS DRIVERS'!AG9</f>
         <v/>
       </c>
       <c r="AG12" s="9">
-        <f>'QTR P&amp;L'!AG11*'IS DRIVERS'!AG9</f>
+        <f>'QTR P&amp;L'!AG11*'IS DRIVERS'!AH9</f>
         <v/>
       </c>
     </row>
@@ -31651,67 +31651,67 @@
         <v/>
       </c>
       <c r="R16" s="9">
-        <f>'QTR P&amp;L'!R2*'IS DRIVERS'!R10</f>
+        <f>'QTR P&amp;L'!R2*'IS DRIVERS'!S10</f>
         <v/>
       </c>
       <c r="S16" s="9">
-        <f>'QTR P&amp;L'!S2*'IS DRIVERS'!S10</f>
+        <f>'QTR P&amp;L'!S2*'IS DRIVERS'!T10</f>
         <v/>
       </c>
       <c r="T16" s="9">
-        <f>'QTR P&amp;L'!T2*'IS DRIVERS'!T10</f>
+        <f>'QTR P&amp;L'!T2*'IS DRIVERS'!U10</f>
         <v/>
       </c>
       <c r="U16" s="9">
-        <f>'QTR P&amp;L'!U2*'IS DRIVERS'!U10</f>
+        <f>'QTR P&amp;L'!U2*'IS DRIVERS'!V10</f>
         <v/>
       </c>
       <c r="V16" s="9">
-        <f>'QTR P&amp;L'!V2*'IS DRIVERS'!V10</f>
+        <f>'QTR P&amp;L'!V2*'IS DRIVERS'!W10</f>
         <v/>
       </c>
       <c r="W16" s="9">
-        <f>'QTR P&amp;L'!W2*'IS DRIVERS'!W10</f>
+        <f>'QTR P&amp;L'!W2*'IS DRIVERS'!X10</f>
         <v/>
       </c>
       <c r="X16" s="9">
-        <f>'QTR P&amp;L'!X2*'IS DRIVERS'!X10</f>
+        <f>'QTR P&amp;L'!X2*'IS DRIVERS'!Y10</f>
         <v/>
       </c>
       <c r="Y16" s="9">
-        <f>'QTR P&amp;L'!Y2*'IS DRIVERS'!Y10</f>
+        <f>'QTR P&amp;L'!Y2*'IS DRIVERS'!Z10</f>
         <v/>
       </c>
       <c r="Z16" s="9">
-        <f>'QTR P&amp;L'!Z2*'IS DRIVERS'!Z10</f>
+        <f>'QTR P&amp;L'!Z2*'IS DRIVERS'!AA10</f>
         <v/>
       </c>
       <c r="AA16" s="9">
-        <f>'QTR P&amp;L'!AA2*'IS DRIVERS'!AA10</f>
+        <f>'QTR P&amp;L'!AA2*'IS DRIVERS'!AB10</f>
         <v/>
       </c>
       <c r="AB16" s="9">
-        <f>'QTR P&amp;L'!AB2*'IS DRIVERS'!AB10</f>
+        <f>'QTR P&amp;L'!AB2*'IS DRIVERS'!AC10</f>
         <v/>
       </c>
       <c r="AC16" s="9">
-        <f>'QTR P&amp;L'!AC2*'IS DRIVERS'!AC10</f>
+        <f>'QTR P&amp;L'!AC2*'IS DRIVERS'!AD10</f>
         <v/>
       </c>
       <c r="AD16" s="9">
-        <f>'QTR P&amp;L'!AD2*'IS DRIVERS'!AD10</f>
+        <f>'QTR P&amp;L'!AD2*'IS DRIVERS'!AE10</f>
         <v/>
       </c>
       <c r="AE16" s="9">
-        <f>'QTR P&amp;L'!AE2*'IS DRIVERS'!AE10</f>
+        <f>'QTR P&amp;L'!AE2*'IS DRIVERS'!AF10</f>
         <v/>
       </c>
       <c r="AF16" s="9">
-        <f>'QTR P&amp;L'!AF2*'IS DRIVERS'!AF10</f>
+        <f>'QTR P&amp;L'!AF2*'IS DRIVERS'!AG10</f>
         <v/>
       </c>
       <c r="AG16" s="9">
-        <f>'QTR P&amp;L'!AG2*'IS DRIVERS'!AG10</f>
+        <f>'QTR P&amp;L'!AG2*'IS DRIVERS'!AH10</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-04-28 15:12:23
</commit_message>
<xml_diff>
--- a/Knowledge/Model Outputs/CELH/CELH_model.xlsx
+++ b/Knowledge/Model Outputs/CELH/CELH_model.xlsx
@@ -9382,55 +9382,55 @@
         </is>
       </c>
       <c r="B4" s="14">
-        <f>IFERROR('QTR BS'!B4/'QTR P&amp;L'!B2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!B4/'QTR P&amp;L'!E2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="C4" s="14">
-        <f>IFERROR('QTR BS'!C4/'QTR P&amp;L'!C2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!C4/'QTR P&amp;L'!F2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="D4" s="14">
-        <f>IFERROR('QTR BS'!D4/'QTR P&amp;L'!D2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!D4/'QTR P&amp;L'!G2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="E4" s="14">
-        <f>IFERROR('QTR BS'!E4/'QTR P&amp;L'!E2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!E4/'QTR P&amp;L'!H2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="F4" s="14">
-        <f>IFERROR('QTR BS'!F4/'QTR P&amp;L'!F2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!F4/'QTR P&amp;L'!I2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="G4" s="14">
-        <f>IFERROR('QTR BS'!G4/'QTR P&amp;L'!G2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!G4/'QTR P&amp;L'!J2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="H4" s="14">
-        <f>IFERROR('QTR BS'!H4/'QTR P&amp;L'!H2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!H4/'QTR P&amp;L'!K2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="I4" s="14">
-        <f>IFERROR('QTR BS'!I4/'QTR P&amp;L'!I2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!I4/'QTR P&amp;L'!L2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="J4" s="14">
-        <f>IFERROR('QTR BS'!J4/'QTR P&amp;L'!J2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!J4/'QTR P&amp;L'!M2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="K4" s="14">
-        <f>IFERROR('QTR BS'!K4/'QTR P&amp;L'!K2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!K4/'QTR P&amp;L'!N2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="L4" s="14">
-        <f>IFERROR('QTR BS'!L4/'QTR P&amp;L'!L2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!L4/'QTR P&amp;L'!O2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="M4" s="14">
-        <f>IFERROR('QTR BS'!M4/'QTR P&amp;L'!M2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!M4/'QTR P&amp;L'!P2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="N4" s="14">
-        <f>IFERROR('QTR BS'!N4/'QTR P&amp;L'!N2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!N4/'QTR P&amp;L'!Q2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="O4" s="15">
@@ -9505,55 +9505,55 @@
         </is>
       </c>
       <c r="B5" s="14">
-        <f>IFERROR('QTR BS'!B5/'QTR P&amp;L'!B2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!B5/'QTR P&amp;L'!E2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="C5" s="14">
-        <f>IFERROR('QTR BS'!C5/'QTR P&amp;L'!C2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!C5/'QTR P&amp;L'!F2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="D5" s="14">
-        <f>IFERROR('QTR BS'!D5/'QTR P&amp;L'!D2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!D5/'QTR P&amp;L'!G2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="E5" s="14">
-        <f>IFERROR('QTR BS'!E5/'QTR P&amp;L'!E2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!E5/'QTR P&amp;L'!H2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="F5" s="14">
-        <f>IFERROR('QTR BS'!F5/'QTR P&amp;L'!F2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!F5/'QTR P&amp;L'!I2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="G5" s="14">
-        <f>IFERROR('QTR BS'!G5/'QTR P&amp;L'!G2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!G5/'QTR P&amp;L'!J2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="H5" s="14">
-        <f>IFERROR('QTR BS'!H5/'QTR P&amp;L'!H2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!H5/'QTR P&amp;L'!K2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="I5" s="14">
-        <f>IFERROR('QTR BS'!I5/'QTR P&amp;L'!I2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!I5/'QTR P&amp;L'!L2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="J5" s="14">
-        <f>IFERROR('QTR BS'!J5/'QTR P&amp;L'!J2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!J5/'QTR P&amp;L'!M2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="K5" s="14">
-        <f>IFERROR('QTR BS'!K5/'QTR P&amp;L'!K2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!K5/'QTR P&amp;L'!N2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="L5" s="14">
-        <f>IFERROR('QTR BS'!L5/'QTR P&amp;L'!L2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!L5/'QTR P&amp;L'!O2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="M5" s="14">
-        <f>IFERROR('QTR BS'!M5/'QTR P&amp;L'!M2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!M5/'QTR P&amp;L'!P2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="N5" s="14">
-        <f>IFERROR('QTR BS'!N5/'QTR P&amp;L'!N2*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!N5/'QTR P&amp;L'!Q2*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="O5" s="15">
@@ -9628,55 +9628,55 @@
         </is>
       </c>
       <c r="B6" s="14">
-        <f>IFERROR('QTR BS'!B6/'QTR P&amp;L'!B3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!B6/'QTR P&amp;L'!E3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="C6" s="14">
-        <f>IFERROR('QTR BS'!C6/'QTR P&amp;L'!C3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!C6/'QTR P&amp;L'!F3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="D6" s="14">
-        <f>IFERROR('QTR BS'!D6/'QTR P&amp;L'!D3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!D6/'QTR P&amp;L'!G3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="E6" s="14">
-        <f>IFERROR('QTR BS'!E6/'QTR P&amp;L'!E3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!E6/'QTR P&amp;L'!H3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="F6" s="14">
-        <f>IFERROR('QTR BS'!F6/'QTR P&amp;L'!F3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!F6/'QTR P&amp;L'!I3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="G6" s="14">
-        <f>IFERROR('QTR BS'!G6/'QTR P&amp;L'!G3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!G6/'QTR P&amp;L'!J3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="H6" s="14">
-        <f>IFERROR('QTR BS'!H6/'QTR P&amp;L'!H3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!H6/'QTR P&amp;L'!K3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="I6" s="14">
-        <f>IFERROR('QTR BS'!I6/'QTR P&amp;L'!I3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!I6/'QTR P&amp;L'!L3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="J6" s="14">
-        <f>IFERROR('QTR BS'!J6/'QTR P&amp;L'!J3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!J6/'QTR P&amp;L'!M3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="K6" s="14">
-        <f>IFERROR('QTR BS'!K6/'QTR P&amp;L'!K3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!K6/'QTR P&amp;L'!N3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="L6" s="14">
-        <f>IFERROR('QTR BS'!L6/'QTR P&amp;L'!L3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!L6/'QTR P&amp;L'!O3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="M6" s="14">
-        <f>IFERROR('QTR BS'!M6/'QTR P&amp;L'!M3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!M6/'QTR P&amp;L'!P3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="N6" s="14">
-        <f>IFERROR('QTR BS'!N6/'QTR P&amp;L'!N3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!N6/'QTR P&amp;L'!Q3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="O6" s="15">
@@ -9751,55 +9751,55 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>IFERROR('QTR BS'!B7/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B7/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C7" s="11">
-        <f>IFERROR('QTR BS'!C7/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C7/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>IFERROR('QTR BS'!D7/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D7/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E7" s="11">
-        <f>IFERROR('QTR BS'!E7/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E7/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F7" s="11">
-        <f>IFERROR('QTR BS'!F7/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F7/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G7" s="11">
-        <f>IFERROR('QTR BS'!G7/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G7/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H7" s="11">
-        <f>IFERROR('QTR BS'!H7/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H7/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I7" s="11">
-        <f>IFERROR('QTR BS'!I7/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I7/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J7" s="11">
-        <f>IFERROR('QTR BS'!J7/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J7/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K7" s="11">
-        <f>IFERROR('QTR BS'!K7/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K7/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L7" s="11">
-        <f>IFERROR('QTR BS'!L7/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L7/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M7" s="11">
-        <f>IFERROR('QTR BS'!M7/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M7/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N7" s="11">
-        <f>IFERROR('QTR BS'!N7/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N7/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O7" s="12">
@@ -9874,55 +9874,55 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>IFERROR('QTR BS'!B8/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B8/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C8" s="11">
-        <f>IFERROR('QTR BS'!C8/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C8/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>IFERROR('QTR BS'!D8/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D8/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E8" s="11">
-        <f>IFERROR('QTR BS'!E8/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E8/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F8" s="11">
-        <f>IFERROR('QTR BS'!F8/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F8/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G8" s="11">
-        <f>IFERROR('QTR BS'!G8/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G8/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H8" s="11">
-        <f>IFERROR('QTR BS'!H8/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H8/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I8" s="11">
-        <f>IFERROR('QTR BS'!I8/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I8/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J8" s="11">
-        <f>IFERROR('QTR BS'!J8/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J8/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K8" s="11">
-        <f>IFERROR('QTR BS'!K8/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K8/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L8" s="11">
-        <f>IFERROR('QTR BS'!L8/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L8/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M8" s="11">
-        <f>IFERROR('QTR BS'!M8/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M8/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N8" s="11">
-        <f>IFERROR('QTR BS'!N8/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N8/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O8" s="12">
@@ -9997,55 +9997,55 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>IFERROR('QTR BS'!B10/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B10/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C9" s="11">
-        <f>IFERROR('QTR BS'!C10/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C10/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D9" s="11">
-        <f>IFERROR('QTR BS'!D10/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D10/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E9" s="11">
-        <f>IFERROR('QTR BS'!E10/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E10/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F9" s="11">
-        <f>IFERROR('QTR BS'!F10/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F10/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G9" s="11">
-        <f>IFERROR('QTR BS'!G10/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G10/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H9" s="11">
-        <f>IFERROR('QTR BS'!H10/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H10/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I9" s="11">
-        <f>IFERROR('QTR BS'!I10/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I10/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J9" s="11">
-        <f>IFERROR('QTR BS'!J10/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J10/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K9" s="11">
-        <f>IFERROR('QTR BS'!K10/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K10/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L9" s="11">
-        <f>IFERROR('QTR BS'!L10/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L10/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M9" s="11">
-        <f>IFERROR('QTR BS'!M10/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M10/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N9" s="11">
-        <f>IFERROR('QTR BS'!N10/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N10/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O9" s="12">
@@ -10243,55 +10243,55 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>IFERROR('QTR BS'!B12/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B12/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C11" s="11">
-        <f>IFERROR('QTR BS'!C12/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C12/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D11" s="11">
-        <f>IFERROR('QTR BS'!D12/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D12/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E11" s="11">
-        <f>IFERROR('QTR BS'!E12/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E12/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F11" s="11">
-        <f>IFERROR('QTR BS'!F12/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F12/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G11" s="11">
-        <f>IFERROR('QTR BS'!G12/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G12/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H11" s="11">
-        <f>IFERROR('QTR BS'!H12/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H12/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I11" s="11">
-        <f>IFERROR('QTR BS'!I12/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I12/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J11" s="11">
-        <f>IFERROR('QTR BS'!J12/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J12/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K11" s="11">
-        <f>IFERROR('QTR BS'!K12/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K12/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L11" s="11">
-        <f>IFERROR('QTR BS'!L12/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L12/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M11" s="11">
-        <f>IFERROR('QTR BS'!M12/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M12/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N11" s="11">
-        <f>IFERROR('QTR BS'!N12/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N12/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O11" s="12">
@@ -10612,55 +10612,55 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>IFERROR('QTR BS'!B15/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B15/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C14" s="11">
-        <f>IFERROR('QTR BS'!C15/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C15/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D14" s="11">
-        <f>IFERROR('QTR BS'!D15/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D15/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E14" s="11">
-        <f>IFERROR('QTR BS'!E15/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E15/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F14" s="11">
-        <f>IFERROR('QTR BS'!F15/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F15/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G14" s="11">
-        <f>IFERROR('QTR BS'!G15/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G15/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H14" s="11">
-        <f>IFERROR('QTR BS'!H15/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H15/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I14" s="11">
-        <f>IFERROR('QTR BS'!I15/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I15/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J14" s="11">
-        <f>IFERROR('QTR BS'!J15/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J15/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K14" s="11">
-        <f>IFERROR('QTR BS'!K15/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K15/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L14" s="11">
-        <f>IFERROR('QTR BS'!L15/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L15/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M14" s="11">
-        <f>IFERROR('QTR BS'!M15/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M15/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N14" s="11">
-        <f>IFERROR('QTR BS'!N15/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N15/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O14" s="12">
@@ -10858,55 +10858,55 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>IFERROR('QTR BS'!B17/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B17/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C16" s="11">
-        <f>IFERROR('QTR BS'!C17/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C17/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D16" s="11">
-        <f>IFERROR('QTR BS'!D17/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D17/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E16" s="11">
-        <f>IFERROR('QTR BS'!E17/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E17/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F16" s="11">
-        <f>IFERROR('QTR BS'!F17/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F17/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G16" s="11">
-        <f>IFERROR('QTR BS'!G17/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G17/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H16" s="11">
-        <f>IFERROR('QTR BS'!H17/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H17/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I16" s="11">
-        <f>IFERROR('QTR BS'!I17/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I17/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J16" s="11">
-        <f>IFERROR('QTR BS'!J17/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J17/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K16" s="11">
-        <f>IFERROR('QTR BS'!K17/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K17/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L16" s="11">
-        <f>IFERROR('QTR BS'!L17/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L17/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M16" s="11">
-        <f>IFERROR('QTR BS'!M17/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M17/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N16" s="11">
-        <f>IFERROR('QTR BS'!N17/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N17/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O16" s="12">
@@ -10981,55 +10981,55 @@
         </is>
       </c>
       <c r="B17" s="11">
-        <f>IFERROR('QTR BS'!B18/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B18/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C17" s="11">
-        <f>IFERROR('QTR BS'!C18/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C18/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D17" s="11">
-        <f>IFERROR('QTR BS'!D18/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D18/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E17" s="11">
-        <f>IFERROR('QTR BS'!E18/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E18/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F17" s="11">
-        <f>IFERROR('QTR BS'!F18/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F18/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G17" s="11">
-        <f>IFERROR('QTR BS'!G18/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G18/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H17" s="11">
-        <f>IFERROR('QTR BS'!H18/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H18/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I17" s="11">
-        <f>IFERROR('QTR BS'!I18/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I18/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J17" s="11">
-        <f>IFERROR('QTR BS'!J18/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J18/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K17" s="11">
-        <f>IFERROR('QTR BS'!K18/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K18/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L17" s="11">
-        <f>IFERROR('QTR BS'!L18/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L18/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M17" s="11">
-        <f>IFERROR('QTR BS'!M18/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M18/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N17" s="11">
-        <f>IFERROR('QTR BS'!N18/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N18/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O17" s="12">
@@ -11104,55 +11104,55 @@
         </is>
       </c>
       <c r="B18" s="14">
-        <f>IFERROR('QTR BS'!B20/'QTR P&amp;L'!B3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!B20/'QTR P&amp;L'!E3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="C18" s="14">
-        <f>IFERROR('QTR BS'!C20/'QTR P&amp;L'!C3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!C20/'QTR P&amp;L'!F3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="D18" s="14">
-        <f>IFERROR('QTR BS'!D20/'QTR P&amp;L'!D3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!D20/'QTR P&amp;L'!G3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="E18" s="14">
-        <f>IFERROR('QTR BS'!E20/'QTR P&amp;L'!E3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!E20/'QTR P&amp;L'!H3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="F18" s="14">
-        <f>IFERROR('QTR BS'!F20/'QTR P&amp;L'!F3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!F20/'QTR P&amp;L'!I3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="G18" s="14">
-        <f>IFERROR('QTR BS'!G20/'QTR P&amp;L'!G3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!G20/'QTR P&amp;L'!J3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="H18" s="14">
-        <f>IFERROR('QTR BS'!H20/'QTR P&amp;L'!H3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!H20/'QTR P&amp;L'!K3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="I18" s="14">
-        <f>IFERROR('QTR BS'!I20/'QTR P&amp;L'!I3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!I20/'QTR P&amp;L'!L3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="J18" s="14">
-        <f>IFERROR('QTR BS'!J20/'QTR P&amp;L'!J3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!J20/'QTR P&amp;L'!M3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="K18" s="14">
-        <f>IFERROR('QTR BS'!K20/'QTR P&amp;L'!K3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!K20/'QTR P&amp;L'!N3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="L18" s="14">
-        <f>IFERROR('QTR BS'!L20/'QTR P&amp;L'!L3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!L20/'QTR P&amp;L'!O3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="M18" s="14">
-        <f>IFERROR('QTR BS'!M20/'QTR P&amp;L'!M3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!M20/'QTR P&amp;L'!P3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="N18" s="14">
-        <f>IFERROR('QTR BS'!N20/'QTR P&amp;L'!N3*ASSUMPTIONS!$B$2,"")</f>
+        <f>IFERROR('QTR BS'!N20/'QTR P&amp;L'!Q3*ASSUMPTIONS!$B$2,"")</f>
         <v/>
       </c>
       <c r="O18" s="15">
@@ -11227,55 +11227,55 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>IFERROR('QTR BS'!B21/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B21/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C19" s="11">
-        <f>IFERROR('QTR BS'!C21/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C21/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D19" s="11">
-        <f>IFERROR('QTR BS'!D21/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D21/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E19" s="11">
-        <f>IFERROR('QTR BS'!E21/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E21/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F19" s="11">
-        <f>IFERROR('QTR BS'!F21/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F21/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G19" s="11">
-        <f>IFERROR('QTR BS'!G21/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G21/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H19" s="11">
-        <f>IFERROR('QTR BS'!H21/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H21/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I19" s="11">
-        <f>IFERROR('QTR BS'!I21/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I21/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J19" s="11">
-        <f>IFERROR('QTR BS'!J21/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J21/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K19" s="11">
-        <f>IFERROR('QTR BS'!K21/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K21/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L19" s="11">
-        <f>IFERROR('QTR BS'!L21/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L21/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M19" s="11">
-        <f>IFERROR('QTR BS'!M21/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M21/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N19" s="11">
-        <f>IFERROR('QTR BS'!N21/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N21/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O19" s="12">
@@ -11350,55 +11350,55 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>IFERROR('QTR BS'!B22/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B22/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C20" s="11">
-        <f>IFERROR('QTR BS'!C22/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C22/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D20" s="11">
-        <f>IFERROR('QTR BS'!D22/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D22/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E20" s="11">
-        <f>IFERROR('QTR BS'!E22/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E22/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F20" s="11">
-        <f>IFERROR('QTR BS'!F22/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F22/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G20" s="11">
-        <f>IFERROR('QTR BS'!G22/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G22/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H20" s="11">
-        <f>IFERROR('QTR BS'!H22/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H22/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I20" s="11">
-        <f>IFERROR('QTR BS'!I22/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I22/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J20" s="11">
-        <f>IFERROR('QTR BS'!J22/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J22/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K20" s="11">
-        <f>IFERROR('QTR BS'!K22/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K22/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L20" s="11">
-        <f>IFERROR('QTR BS'!L22/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L22/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M20" s="11">
-        <f>IFERROR('QTR BS'!M22/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M22/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N20" s="11">
-        <f>IFERROR('QTR BS'!N22/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N22/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O20" s="12">
@@ -11580,55 +11580,55 @@
         </is>
       </c>
       <c r="B22" s="11">
-        <f>IFERROR('QTR BS'!B24/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B24/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C22" s="11">
-        <f>IFERROR('QTR BS'!C24/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C24/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D22" s="11">
-        <f>IFERROR('QTR BS'!D24/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D24/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E22" s="11">
-        <f>IFERROR('QTR BS'!E24/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E24/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F22" s="11">
-        <f>IFERROR('QTR BS'!F24/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F24/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G22" s="11">
-        <f>IFERROR('QTR BS'!G24/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G24/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H22" s="11">
-        <f>IFERROR('QTR BS'!H24/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H24/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I22" s="11">
-        <f>IFERROR('QTR BS'!I24/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I24/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J22" s="11">
-        <f>IFERROR('QTR BS'!J24/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J24/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K22" s="11">
-        <f>IFERROR('QTR BS'!K24/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K24/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L22" s="11">
-        <f>IFERROR('QTR BS'!L24/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L24/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M22" s="11">
-        <f>IFERROR('QTR BS'!M24/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M24/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N22" s="11">
-        <f>IFERROR('QTR BS'!N24/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N24/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O22" s="12">
@@ -11703,55 +11703,55 @@
         </is>
       </c>
       <c r="B23" s="11">
-        <f>IFERROR('QTR BS'!B25/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B25/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C23" s="11">
-        <f>IFERROR('QTR BS'!C25/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C25/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D23" s="11">
-        <f>IFERROR('QTR BS'!D25/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D25/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E23" s="11">
-        <f>IFERROR('QTR BS'!E25/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E25/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F23" s="11">
-        <f>IFERROR('QTR BS'!F25/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F25/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G23" s="11">
-        <f>IFERROR('QTR BS'!G25/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G25/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H23" s="11">
-        <f>IFERROR('QTR BS'!H25/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H25/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I23" s="11">
-        <f>IFERROR('QTR BS'!I25/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I25/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J23" s="11">
-        <f>IFERROR('QTR BS'!J25/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J25/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K23" s="11">
-        <f>IFERROR('QTR BS'!K25/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K25/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L23" s="11">
-        <f>IFERROR('QTR BS'!L25/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L25/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M23" s="11">
-        <f>IFERROR('QTR BS'!M25/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M25/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N23" s="11">
-        <f>IFERROR('QTR BS'!N25/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N25/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O23" s="12">
@@ -11826,55 +11826,55 @@
         </is>
       </c>
       <c r="B24" s="11">
-        <f>IFERROR('QTR BS'!B26/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B26/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C24" s="11">
-        <f>IFERROR('QTR BS'!C26/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C26/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D24" s="11">
-        <f>IFERROR('QTR BS'!D26/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D26/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E24" s="11">
-        <f>IFERROR('QTR BS'!E26/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E26/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F24" s="11">
-        <f>IFERROR('QTR BS'!F26/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F26/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G24" s="11">
-        <f>IFERROR('QTR BS'!G26/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G26/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H24" s="11">
-        <f>IFERROR('QTR BS'!H26/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H26/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I24" s="11">
-        <f>IFERROR('QTR BS'!I26/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I26/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J24" s="11">
-        <f>IFERROR('QTR BS'!J26/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J26/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K24" s="11">
-        <f>IFERROR('QTR BS'!K26/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K26/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L24" s="11">
-        <f>IFERROR('QTR BS'!L26/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L26/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M24" s="11">
-        <f>IFERROR('QTR BS'!M26/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M26/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N24" s="11">
-        <f>IFERROR('QTR BS'!N26/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N26/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O24" s="12">
@@ -11949,55 +11949,55 @@
         </is>
       </c>
       <c r="B25" s="11">
-        <f>IFERROR('QTR BS'!B27/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B27/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C25" s="11">
-        <f>IFERROR('QTR BS'!C27/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C27/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D25" s="11">
-        <f>IFERROR('QTR BS'!D27/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D27/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E25" s="11">
-        <f>IFERROR('QTR BS'!E27/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E27/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F25" s="11">
-        <f>IFERROR('QTR BS'!F27/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F27/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G25" s="11">
-        <f>IFERROR('QTR BS'!G27/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G27/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H25" s="11">
-        <f>IFERROR('QTR BS'!H27/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H27/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I25" s="11">
-        <f>IFERROR('QTR BS'!I27/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I27/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J25" s="11">
-        <f>IFERROR('QTR BS'!J27/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J27/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K25" s="11">
-        <f>IFERROR('QTR BS'!K27/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K27/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L25" s="11">
-        <f>IFERROR('QTR BS'!L27/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L27/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M25" s="11">
-        <f>IFERROR('QTR BS'!M27/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M27/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N25" s="11">
-        <f>IFERROR('QTR BS'!N27/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N27/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O25" s="12">
@@ -12072,55 +12072,55 @@
         </is>
       </c>
       <c r="B26" s="11">
-        <f>IFERROR('QTR BS'!B28/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B28/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C26" s="11">
-        <f>IFERROR('QTR BS'!C28/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C28/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D26" s="11">
-        <f>IFERROR('QTR BS'!D28/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D28/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E26" s="11">
-        <f>IFERROR('QTR BS'!E28/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E28/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F26" s="11">
-        <f>IFERROR('QTR BS'!F28/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F28/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G26" s="11">
-        <f>IFERROR('QTR BS'!G28/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G28/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H26" s="11">
-        <f>IFERROR('QTR BS'!H28/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H28/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I26" s="11">
-        <f>IFERROR('QTR BS'!I28/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I28/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J26" s="11">
-        <f>IFERROR('QTR BS'!J28/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J28/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K26" s="11">
-        <f>IFERROR('QTR BS'!K28/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K28/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L26" s="11">
-        <f>IFERROR('QTR BS'!L28/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L28/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M26" s="11">
-        <f>IFERROR('QTR BS'!M28/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M28/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N26" s="11">
-        <f>IFERROR('QTR BS'!N28/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N28/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O26" s="12">
@@ -12195,55 +12195,55 @@
         </is>
       </c>
       <c r="B27" s="11">
-        <f>IFERROR('QTR BS'!B29/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B29/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C27" s="11">
-        <f>IFERROR('QTR BS'!C29/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C29/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D27" s="11">
-        <f>IFERROR('QTR BS'!D29/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D29/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E27" s="11">
-        <f>IFERROR('QTR BS'!E29/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E29/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F27" s="11">
-        <f>IFERROR('QTR BS'!F29/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F29/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G27" s="11">
-        <f>IFERROR('QTR BS'!G29/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G29/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H27" s="11">
-        <f>IFERROR('QTR BS'!H29/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H29/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I27" s="11">
-        <f>IFERROR('QTR BS'!I29/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I29/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J27" s="11">
-        <f>IFERROR('QTR BS'!J29/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J29/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K27" s="11">
-        <f>IFERROR('QTR BS'!K29/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K29/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L27" s="11">
-        <f>IFERROR('QTR BS'!L29/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L29/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M27" s="11">
-        <f>IFERROR('QTR BS'!M29/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M29/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N27" s="11">
-        <f>IFERROR('QTR BS'!N29/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N29/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O27" s="12">
@@ -12318,55 +12318,55 @@
         </is>
       </c>
       <c r="B28" s="11">
-        <f>IFERROR('QTR BS'!B31/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B31/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C28" s="11">
-        <f>IFERROR('QTR BS'!C31/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C31/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D28" s="11">
-        <f>IFERROR('QTR BS'!D31/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D31/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E28" s="11">
-        <f>IFERROR('QTR BS'!E31/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E31/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F28" s="11">
-        <f>IFERROR('QTR BS'!F31/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F31/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G28" s="11">
-        <f>IFERROR('QTR BS'!G31/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G31/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H28" s="11">
-        <f>IFERROR('QTR BS'!H31/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H31/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I28" s="11">
-        <f>IFERROR('QTR BS'!I31/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I31/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J28" s="11">
-        <f>IFERROR('QTR BS'!J31/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J31/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K28" s="11">
-        <f>IFERROR('QTR BS'!K31/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K31/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L28" s="11">
-        <f>IFERROR('QTR BS'!L31/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L31/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M28" s="11">
-        <f>IFERROR('QTR BS'!M31/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M31/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N28" s="11">
-        <f>IFERROR('QTR BS'!N31/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N31/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O28" s="12">
@@ -12441,55 +12441,55 @@
         </is>
       </c>
       <c r="B29" s="11">
-        <f>IFERROR('QTR BS'!B32/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B32/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C29" s="11">
-        <f>IFERROR('QTR BS'!C32/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C32/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D29" s="11">
-        <f>IFERROR('QTR BS'!D32/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D32/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E29" s="11">
-        <f>IFERROR('QTR BS'!E32/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E32/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F29" s="11">
-        <f>IFERROR('QTR BS'!F32/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F32/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G29" s="11">
-        <f>IFERROR('QTR BS'!G32/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G32/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H29" s="11">
-        <f>IFERROR('QTR BS'!H32/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H32/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I29" s="11">
-        <f>IFERROR('QTR BS'!I32/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I32/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J29" s="11">
-        <f>IFERROR('QTR BS'!J32/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J32/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K29" s="11">
-        <f>IFERROR('QTR BS'!K32/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K32/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L29" s="11">
-        <f>IFERROR('QTR BS'!L32/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L32/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M29" s="11">
-        <f>IFERROR('QTR BS'!M32/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M32/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N29" s="11">
-        <f>IFERROR('QTR BS'!N32/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N32/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O29" s="12">
@@ -12810,55 +12810,55 @@
         </is>
       </c>
       <c r="B32" s="11">
-        <f>IFERROR('QTR BS'!B35/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B35/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C32" s="11">
-        <f>IFERROR('QTR BS'!C35/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C35/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D32" s="11">
-        <f>IFERROR('QTR BS'!D35/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D35/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E32" s="11">
-        <f>IFERROR('QTR BS'!E35/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E35/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F32" s="11">
-        <f>IFERROR('QTR BS'!F35/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F35/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G32" s="11">
-        <f>IFERROR('QTR BS'!G35/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G35/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H32" s="11">
-        <f>IFERROR('QTR BS'!H35/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H35/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I32" s="11">
-        <f>IFERROR('QTR BS'!I35/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I35/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J32" s="11">
-        <f>IFERROR('QTR BS'!J35/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J35/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K32" s="11">
-        <f>IFERROR('QTR BS'!K35/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K35/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L32" s="11">
-        <f>IFERROR('QTR BS'!L35/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L35/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M32" s="11">
-        <f>IFERROR('QTR BS'!M35/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M35/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N32" s="11">
-        <f>IFERROR('QTR BS'!N35/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N35/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O32" s="12">
@@ -12933,55 +12933,55 @@
         </is>
       </c>
       <c r="B33" s="11">
-        <f>IFERROR('QTR BS'!B36/'QTR P&amp;L'!B2,"")</f>
+        <f>IFERROR('QTR BS'!B36/'QTR P&amp;L'!E2,"")</f>
         <v/>
       </c>
       <c r="C33" s="11">
-        <f>IFERROR('QTR BS'!C36/'QTR P&amp;L'!C2,"")</f>
+        <f>IFERROR('QTR BS'!C36/'QTR P&amp;L'!F2,"")</f>
         <v/>
       </c>
       <c r="D33" s="11">
-        <f>IFERROR('QTR BS'!D36/'QTR P&amp;L'!D2,"")</f>
+        <f>IFERROR('QTR BS'!D36/'QTR P&amp;L'!G2,"")</f>
         <v/>
       </c>
       <c r="E33" s="11">
-        <f>IFERROR('QTR BS'!E36/'QTR P&amp;L'!E2,"")</f>
+        <f>IFERROR('QTR BS'!E36/'QTR P&amp;L'!H2,"")</f>
         <v/>
       </c>
       <c r="F33" s="11">
-        <f>IFERROR('QTR BS'!F36/'QTR P&amp;L'!F2,"")</f>
+        <f>IFERROR('QTR BS'!F36/'QTR P&amp;L'!I2,"")</f>
         <v/>
       </c>
       <c r="G33" s="11">
-        <f>IFERROR('QTR BS'!G36/'QTR P&amp;L'!G2,"")</f>
+        <f>IFERROR('QTR BS'!G36/'QTR P&amp;L'!J2,"")</f>
         <v/>
       </c>
       <c r="H33" s="11">
-        <f>IFERROR('QTR BS'!H36/'QTR P&amp;L'!H2,"")</f>
+        <f>IFERROR('QTR BS'!H36/'QTR P&amp;L'!K2,"")</f>
         <v/>
       </c>
       <c r="I33" s="11">
-        <f>IFERROR('QTR BS'!I36/'QTR P&amp;L'!I2,"")</f>
+        <f>IFERROR('QTR BS'!I36/'QTR P&amp;L'!L2,"")</f>
         <v/>
       </c>
       <c r="J33" s="11">
-        <f>IFERROR('QTR BS'!J36/'QTR P&amp;L'!J2,"")</f>
+        <f>IFERROR('QTR BS'!J36/'QTR P&amp;L'!M2,"")</f>
         <v/>
       </c>
       <c r="K33" s="11">
-        <f>IFERROR('QTR BS'!K36/'QTR P&amp;L'!K2,"")</f>
+        <f>IFERROR('QTR BS'!K36/'QTR P&amp;L'!N2,"")</f>
         <v/>
       </c>
       <c r="L33" s="11">
-        <f>IFERROR('QTR BS'!L36/'QTR P&amp;L'!L2,"")</f>
+        <f>IFERROR('QTR BS'!L36/'QTR P&amp;L'!O2,"")</f>
         <v/>
       </c>
       <c r="M33" s="11">
-        <f>IFERROR('QTR BS'!M36/'QTR P&amp;L'!M2,"")</f>
+        <f>IFERROR('QTR BS'!M36/'QTR P&amp;L'!P2,"")</f>
         <v/>
       </c>
       <c r="N33" s="11">
-        <f>IFERROR('QTR BS'!N36/'QTR P&amp;L'!N2,"")</f>
+        <f>IFERROR('QTR BS'!N36/'QTR P&amp;L'!Q2,"")</f>
         <v/>
       </c>
       <c r="O33" s="12">

</xml_diff>

<commit_message>
vault backup: 2026-04-28 15:27:53
</commit_message>
<xml_diff>
--- a/Knowledge/Model Outputs/CELH/CELH_model.xlsx
+++ b/Knowledge/Model Outputs/CELH/CELH_model.xlsx
@@ -8666,79 +8666,79 @@
         <v/>
       </c>
       <c r="T2" s="12">
-        <f>R2</f>
+        <f>S2</f>
         <v/>
       </c>
       <c r="U2" s="12">
-        <f>R2</f>
+        <f>T2</f>
         <v/>
       </c>
       <c r="V2" s="12">
-        <f>R2</f>
+        <f>U2</f>
         <v/>
       </c>
       <c r="W2" s="12">
-        <f>R2</f>
+        <f>V2</f>
         <v/>
       </c>
       <c r="X2" s="12">
-        <f>R2</f>
+        <f>W2</f>
         <v/>
       </c>
       <c r="Y2" s="12">
-        <f>R2</f>
+        <f>X2</f>
         <v/>
       </c>
       <c r="Z2" s="12">
-        <f>R2</f>
+        <f>Y2</f>
         <v/>
       </c>
       <c r="AA2" s="12">
-        <f>R2</f>
+        <f>Z2</f>
         <v/>
       </c>
       <c r="AB2" s="12">
-        <f>R2</f>
+        <f>AA2</f>
         <v/>
       </c>
       <c r="AC2" s="12">
-        <f>R2</f>
+        <f>AB2</f>
         <v/>
       </c>
       <c r="AD2" s="12">
-        <f>R2</f>
+        <f>AC2</f>
         <v/>
       </c>
       <c r="AE2" s="12">
-        <f>R2</f>
+        <f>AD2</f>
         <v/>
       </c>
       <c r="AF2" s="12">
-        <f>R2</f>
+        <f>AE2</f>
         <v/>
       </c>
       <c r="AG2" s="12">
-        <f>R2</f>
+        <f>AF2</f>
         <v/>
       </c>
       <c r="AH2" s="12">
-        <f>R2</f>
+        <f>AG2</f>
         <v/>
       </c>
       <c r="AI2" s="12">
-        <f>R2</f>
+        <f>AH2</f>
         <v/>
       </c>
       <c r="AJ2" s="12">
-        <f>R2</f>
+        <f>AI2</f>
         <v/>
       </c>
       <c r="AK2" s="12">
-        <f>R2</f>
+        <f>AJ2</f>
         <v/>
       </c>
       <c r="AL2" s="12">
-        <f>R2</f>
+        <f>AK2</f>
         <v/>
       </c>
     </row>
@@ -8817,79 +8817,79 @@
         <v/>
       </c>
       <c r="T3" s="12">
-        <f>R3</f>
+        <f>S3</f>
         <v/>
       </c>
       <c r="U3" s="12">
-        <f>R3</f>
+        <f>T3</f>
         <v/>
       </c>
       <c r="V3" s="12">
-        <f>R3</f>
+        <f>U3</f>
         <v/>
       </c>
       <c r="W3" s="12">
-        <f>R3</f>
+        <f>V3</f>
         <v/>
       </c>
       <c r="X3" s="12">
-        <f>R3</f>
+        <f>W3</f>
         <v/>
       </c>
       <c r="Y3" s="12">
-        <f>R3</f>
+        <f>X3</f>
         <v/>
       </c>
       <c r="Z3" s="12">
-        <f>R3</f>
+        <f>Y3</f>
         <v/>
       </c>
       <c r="AA3" s="12">
-        <f>R3</f>
+        <f>Z3</f>
         <v/>
       </c>
       <c r="AB3" s="12">
-        <f>R3</f>
+        <f>AA3</f>
         <v/>
       </c>
       <c r="AC3" s="12">
-        <f>R3</f>
+        <f>AB3</f>
         <v/>
       </c>
       <c r="AD3" s="12">
-        <f>R3</f>
+        <f>AC3</f>
         <v/>
       </c>
       <c r="AE3" s="12">
-        <f>R3</f>
+        <f>AD3</f>
         <v/>
       </c>
       <c r="AF3" s="12">
-        <f>R3</f>
+        <f>AE3</f>
         <v/>
       </c>
       <c r="AG3" s="12">
-        <f>R3</f>
+        <f>AF3</f>
         <v/>
       </c>
       <c r="AH3" s="12">
-        <f>R3</f>
+        <f>AG3</f>
         <v/>
       </c>
       <c r="AI3" s="12">
-        <f>R3</f>
+        <f>AH3</f>
         <v/>
       </c>
       <c r="AJ3" s="12">
-        <f>R3</f>
+        <f>AI3</f>
         <v/>
       </c>
       <c r="AK3" s="12">
-        <f>R3</f>
+        <f>AJ3</f>
         <v/>
       </c>
       <c r="AL3" s="12">
-        <f>R3</f>
+        <f>AK3</f>
         <v/>
       </c>
     </row>
@@ -8968,79 +8968,79 @@
         <v/>
       </c>
       <c r="T4" s="12">
-        <f>R4</f>
+        <f>S4</f>
         <v/>
       </c>
       <c r="U4" s="12">
-        <f>R4</f>
+        <f>T4</f>
         <v/>
       </c>
       <c r="V4" s="12">
-        <f>R4</f>
+        <f>U4</f>
         <v/>
       </c>
       <c r="W4" s="12">
-        <f>R4</f>
+        <f>V4</f>
         <v/>
       </c>
       <c r="X4" s="12">
-        <f>R4</f>
+        <f>W4</f>
         <v/>
       </c>
       <c r="Y4" s="12">
-        <f>R4</f>
+        <f>X4</f>
         <v/>
       </c>
       <c r="Z4" s="12">
-        <f>R4</f>
+        <f>Y4</f>
         <v/>
       </c>
       <c r="AA4" s="12">
-        <f>R4</f>
+        <f>Z4</f>
         <v/>
       </c>
       <c r="AB4" s="12">
-        <f>R4</f>
+        <f>AA4</f>
         <v/>
       </c>
       <c r="AC4" s="12">
-        <f>R4</f>
+        <f>AB4</f>
         <v/>
       </c>
       <c r="AD4" s="12">
-        <f>R4</f>
+        <f>AC4</f>
         <v/>
       </c>
       <c r="AE4" s="12">
-        <f>R4</f>
+        <f>AD4</f>
         <v/>
       </c>
       <c r="AF4" s="12">
-        <f>R4</f>
+        <f>AE4</f>
         <v/>
       </c>
       <c r="AG4" s="12">
-        <f>R4</f>
+        <f>AF4</f>
         <v/>
       </c>
       <c r="AH4" s="12">
-        <f>R4</f>
+        <f>AG4</f>
         <v/>
       </c>
       <c r="AI4" s="12">
-        <f>R4</f>
+        <f>AH4</f>
         <v/>
       </c>
       <c r="AJ4" s="12">
-        <f>R4</f>
+        <f>AI4</f>
         <v/>
       </c>
       <c r="AK4" s="12">
-        <f>R4</f>
+        <f>AJ4</f>
         <v/>
       </c>
       <c r="AL4" s="12">
-        <f>R4</f>
+        <f>AK4</f>
         <v/>
       </c>
     </row>
@@ -9250,79 +9250,79 @@
         <v/>
       </c>
       <c r="T6" s="13">
-        <f>R6</f>
+        <f>S6</f>
         <v/>
       </c>
       <c r="U6" s="13">
-        <f>R6</f>
+        <f>T6</f>
         <v/>
       </c>
       <c r="V6" s="13">
-        <f>R6</f>
+        <f>U6</f>
         <v/>
       </c>
       <c r="W6" s="13">
-        <f>R6</f>
+        <f>V6</f>
         <v/>
       </c>
       <c r="X6" s="13">
-        <f>R6</f>
+        <f>W6</f>
         <v/>
       </c>
       <c r="Y6" s="13">
-        <f>R6</f>
+        <f>X6</f>
         <v/>
       </c>
       <c r="Z6" s="13">
-        <f>R6</f>
+        <f>Y6</f>
         <v/>
       </c>
       <c r="AA6" s="13">
-        <f>R6</f>
+        <f>Z6</f>
         <v/>
       </c>
       <c r="AB6" s="13">
-        <f>R6</f>
+        <f>AA6</f>
         <v/>
       </c>
       <c r="AC6" s="13">
-        <f>R6</f>
+        <f>AB6</f>
         <v/>
       </c>
       <c r="AD6" s="13">
-        <f>R6</f>
+        <f>AC6</f>
         <v/>
       </c>
       <c r="AE6" s="13">
-        <f>R6</f>
+        <f>AD6</f>
         <v/>
       </c>
       <c r="AF6" s="13">
-        <f>R6</f>
+        <f>AE6</f>
         <v/>
       </c>
       <c r="AG6" s="13">
-        <f>R6</f>
+        <f>AF6</f>
         <v/>
       </c>
       <c r="AH6" s="13">
-        <f>R6</f>
+        <f>AG6</f>
         <v/>
       </c>
       <c r="AI6" s="13">
-        <f>R6</f>
+        <f>AH6</f>
         <v/>
       </c>
       <c r="AJ6" s="13">
-        <f>R6</f>
+        <f>AI6</f>
         <v/>
       </c>
       <c r="AK6" s="13">
-        <f>R6</f>
+        <f>AJ6</f>
         <v/>
       </c>
       <c r="AL6" s="13">
-        <f>R6</f>
+        <f>AK6</f>
         <v/>
       </c>
     </row>
@@ -9401,79 +9401,79 @@
         <v/>
       </c>
       <c r="T7" s="13">
-        <f>R7</f>
+        <f>S7</f>
         <v/>
       </c>
       <c r="U7" s="13">
-        <f>R7</f>
+        <f>T7</f>
         <v/>
       </c>
       <c r="V7" s="13">
-        <f>R7</f>
+        <f>U7</f>
         <v/>
       </c>
       <c r="W7" s="13">
-        <f>R7</f>
+        <f>V7</f>
         <v/>
       </c>
       <c r="X7" s="13">
-        <f>R7</f>
+        <f>W7</f>
         <v/>
       </c>
       <c r="Y7" s="13">
-        <f>R7</f>
+        <f>X7</f>
         <v/>
       </c>
       <c r="Z7" s="13">
-        <f>R7</f>
+        <f>Y7</f>
         <v/>
       </c>
       <c r="AA7" s="13">
-        <f>R7</f>
+        <f>Z7</f>
         <v/>
       </c>
       <c r="AB7" s="13">
-        <f>R7</f>
+        <f>AA7</f>
         <v/>
       </c>
       <c r="AC7" s="13">
-        <f>R7</f>
+        <f>AB7</f>
         <v/>
       </c>
       <c r="AD7" s="13">
-        <f>R7</f>
+        <f>AC7</f>
         <v/>
       </c>
       <c r="AE7" s="13">
-        <f>R7</f>
+        <f>AD7</f>
         <v/>
       </c>
       <c r="AF7" s="13">
-        <f>R7</f>
+        <f>AE7</f>
         <v/>
       </c>
       <c r="AG7" s="13">
-        <f>R7</f>
+        <f>AF7</f>
         <v/>
       </c>
       <c r="AH7" s="13">
-        <f>R7</f>
+        <f>AG7</f>
         <v/>
       </c>
       <c r="AI7" s="13">
-        <f>R7</f>
+        <f>AH7</f>
         <v/>
       </c>
       <c r="AJ7" s="13">
-        <f>R7</f>
+        <f>AI7</f>
         <v/>
       </c>
       <c r="AK7" s="13">
-        <f>R7</f>
+        <f>AJ7</f>
         <v/>
       </c>
       <c r="AL7" s="13">
-        <f>R7</f>
+        <f>AK7</f>
         <v/>
       </c>
     </row>
@@ -9552,79 +9552,79 @@
         <v/>
       </c>
       <c r="T8" s="13">
-        <f>R8</f>
+        <f>S8</f>
         <v/>
       </c>
       <c r="U8" s="13">
-        <f>R8</f>
+        <f>T8</f>
         <v/>
       </c>
       <c r="V8" s="13">
-        <f>R8</f>
+        <f>U8</f>
         <v/>
       </c>
       <c r="W8" s="13">
-        <f>R8</f>
+        <f>V8</f>
         <v/>
       </c>
       <c r="X8" s="13">
-        <f>R8</f>
+        <f>W8</f>
         <v/>
       </c>
       <c r="Y8" s="13">
-        <f>R8</f>
+        <f>X8</f>
         <v/>
       </c>
       <c r="Z8" s="13">
-        <f>R8</f>
+        <f>Y8</f>
         <v/>
       </c>
       <c r="AA8" s="13">
-        <f>R8</f>
+        <f>Z8</f>
         <v/>
       </c>
       <c r="AB8" s="13">
-        <f>R8</f>
+        <f>AA8</f>
         <v/>
       </c>
       <c r="AC8" s="13">
-        <f>R8</f>
+        <f>AB8</f>
         <v/>
       </c>
       <c r="AD8" s="13">
-        <f>R8</f>
+        <f>AC8</f>
         <v/>
       </c>
       <c r="AE8" s="13">
-        <f>R8</f>
+        <f>AD8</f>
         <v/>
       </c>
       <c r="AF8" s="13">
-        <f>R8</f>
+        <f>AE8</f>
         <v/>
       </c>
       <c r="AG8" s="13">
-        <f>R8</f>
+        <f>AF8</f>
         <v/>
       </c>
       <c r="AH8" s="13">
-        <f>R8</f>
+        <f>AG8</f>
         <v/>
       </c>
       <c r="AI8" s="13">
-        <f>R8</f>
+        <f>AH8</f>
         <v/>
       </c>
       <c r="AJ8" s="13">
-        <f>R8</f>
+        <f>AI8</f>
         <v/>
       </c>
       <c r="AK8" s="13">
-        <f>R8</f>
+        <f>AJ8</f>
         <v/>
       </c>
       <c r="AL8" s="13">
-        <f>R8</f>
+        <f>AK8</f>
         <v/>
       </c>
     </row>
@@ -9703,79 +9703,79 @@
         <v/>
       </c>
       <c r="T9" s="12">
-        <f>R9</f>
+        <f>S9</f>
         <v/>
       </c>
       <c r="U9" s="12">
-        <f>R9</f>
+        <f>T9</f>
         <v/>
       </c>
       <c r="V9" s="12">
-        <f>R9</f>
+        <f>U9</f>
         <v/>
       </c>
       <c r="W9" s="12">
-        <f>R9</f>
+        <f>V9</f>
         <v/>
       </c>
       <c r="X9" s="12">
-        <f>R9</f>
+        <f>W9</f>
         <v/>
       </c>
       <c r="Y9" s="12">
-        <f>R9</f>
+        <f>X9</f>
         <v/>
       </c>
       <c r="Z9" s="12">
-        <f>R9</f>
+        <f>Y9</f>
         <v/>
       </c>
       <c r="AA9" s="12">
-        <f>R9</f>
+        <f>Z9</f>
         <v/>
       </c>
       <c r="AB9" s="12">
-        <f>R9</f>
+        <f>AA9</f>
         <v/>
       </c>
       <c r="AC9" s="12">
-        <f>R9</f>
+        <f>AB9</f>
         <v/>
       </c>
       <c r="AD9" s="12">
-        <f>R9</f>
+        <f>AC9</f>
         <v/>
       </c>
       <c r="AE9" s="12">
-        <f>R9</f>
+        <f>AD9</f>
         <v/>
       </c>
       <c r="AF9" s="12">
-        <f>R9</f>
+        <f>AE9</f>
         <v/>
       </c>
       <c r="AG9" s="12">
-        <f>R9</f>
+        <f>AF9</f>
         <v/>
       </c>
       <c r="AH9" s="12">
-        <f>R9</f>
+        <f>AG9</f>
         <v/>
       </c>
       <c r="AI9" s="12">
-        <f>R9</f>
+        <f>AH9</f>
         <v/>
       </c>
       <c r="AJ9" s="12">
-        <f>R9</f>
+        <f>AI9</f>
         <v/>
       </c>
       <c r="AK9" s="12">
-        <f>R9</f>
+        <f>AJ9</f>
         <v/>
       </c>
       <c r="AL9" s="12">
-        <f>R9</f>
+        <f>AK9</f>
         <v/>
       </c>
     </row>
@@ -9854,79 +9854,79 @@
         <v/>
       </c>
       <c r="T10" s="12">
-        <f>R10</f>
+        <f>S10</f>
         <v/>
       </c>
       <c r="U10" s="12">
-        <f>R10</f>
+        <f>T10</f>
         <v/>
       </c>
       <c r="V10" s="12">
-        <f>R10</f>
+        <f>U10</f>
         <v/>
       </c>
       <c r="W10" s="12">
-        <f>R10</f>
+        <f>V10</f>
         <v/>
       </c>
       <c r="X10" s="12">
-        <f>R10</f>
+        <f>W10</f>
         <v/>
       </c>
       <c r="Y10" s="12">
-        <f>R10</f>
+        <f>X10</f>
         <v/>
       </c>
       <c r="Z10" s="12">
-        <f>R10</f>
+        <f>Y10</f>
         <v/>
       </c>
       <c r="AA10" s="12">
-        <f>R10</f>
+        <f>Z10</f>
         <v/>
       </c>
       <c r="AB10" s="12">
-        <f>R10</f>
+        <f>AA10</f>
         <v/>
       </c>
       <c r="AC10" s="12">
-        <f>R10</f>
+        <f>AB10</f>
         <v/>
       </c>
       <c r="AD10" s="12">
-        <f>R10</f>
+        <f>AC10</f>
         <v/>
       </c>
       <c r="AE10" s="12">
-        <f>R10</f>
+        <f>AD10</f>
         <v/>
       </c>
       <c r="AF10" s="12">
-        <f>R10</f>
+        <f>AE10</f>
         <v/>
       </c>
       <c r="AG10" s="12">
-        <f>R10</f>
+        <f>AF10</f>
         <v/>
       </c>
       <c r="AH10" s="12">
-        <f>R10</f>
+        <f>AG10</f>
         <v/>
       </c>
       <c r="AI10" s="12">
-        <f>R10</f>
+        <f>AH10</f>
         <v/>
       </c>
       <c r="AJ10" s="12">
-        <f>R10</f>
+        <f>AI10</f>
         <v/>
       </c>
       <c r="AK10" s="12">
-        <f>R10</f>
+        <f>AJ10</f>
         <v/>
       </c>
       <c r="AL10" s="12">
-        <f>R10</f>
+        <f>AK10</f>
         <v/>
       </c>
     </row>
@@ -10359,79 +10359,79 @@
         <v/>
       </c>
       <c r="P3" s="13">
-        <f>N3</f>
+        <f>O3</f>
         <v/>
       </c>
       <c r="Q3" s="13">
-        <f>N3</f>
+        <f>P3</f>
         <v/>
       </c>
       <c r="R3" s="13">
-        <f>N3</f>
+        <f>Q3</f>
         <v/>
       </c>
       <c r="S3" s="13">
-        <f>N3</f>
+        <f>R3</f>
         <v/>
       </c>
       <c r="T3" s="13">
-        <f>N3</f>
+        <f>S3</f>
         <v/>
       </c>
       <c r="U3" s="13">
-        <f>N3</f>
+        <f>T3</f>
         <v/>
       </c>
       <c r="V3" s="13">
-        <f>N3</f>
+        <f>U3</f>
         <v/>
       </c>
       <c r="W3" s="13">
-        <f>N3</f>
+        <f>V3</f>
         <v/>
       </c>
       <c r="X3" s="13">
-        <f>N3</f>
+        <f>W3</f>
         <v/>
       </c>
       <c r="Y3" s="13">
-        <f>N3</f>
+        <f>X3</f>
         <v/>
       </c>
       <c r="Z3" s="13">
-        <f>N3</f>
+        <f>Y3</f>
         <v/>
       </c>
       <c r="AA3" s="13">
-        <f>N3</f>
+        <f>Z3</f>
         <v/>
       </c>
       <c r="AB3" s="13">
-        <f>N3</f>
+        <f>AA3</f>
         <v/>
       </c>
       <c r="AC3" s="13">
-        <f>N3</f>
+        <f>AB3</f>
         <v/>
       </c>
       <c r="AD3" s="13">
-        <f>N3</f>
+        <f>AC3</f>
         <v/>
       </c>
       <c r="AE3" s="13">
-        <f>N3</f>
+        <f>AD3</f>
         <v/>
       </c>
       <c r="AF3" s="13">
-        <f>N3</f>
+        <f>AE3</f>
         <v/>
       </c>
       <c r="AG3" s="13">
-        <f>N3</f>
+        <f>AF3</f>
         <v/>
       </c>
       <c r="AH3" s="13">
-        <f>N3</f>
+        <f>AG3</f>
         <v/>
       </c>
     </row>
@@ -10498,79 +10498,79 @@
         <v/>
       </c>
       <c r="P4" s="15">
-        <f>N4</f>
+        <f>O4</f>
         <v/>
       </c>
       <c r="Q4" s="15">
-        <f>N4</f>
+        <f>P4</f>
         <v/>
       </c>
       <c r="R4" s="15">
-        <f>N4</f>
+        <f>Q4</f>
         <v/>
       </c>
       <c r="S4" s="15">
-        <f>N4</f>
+        <f>R4</f>
         <v/>
       </c>
       <c r="T4" s="15">
-        <f>N4</f>
+        <f>S4</f>
         <v/>
       </c>
       <c r="U4" s="15">
-        <f>N4</f>
+        <f>T4</f>
         <v/>
       </c>
       <c r="V4" s="15">
-        <f>N4</f>
+        <f>U4</f>
         <v/>
       </c>
       <c r="W4" s="15">
-        <f>N4</f>
+        <f>V4</f>
         <v/>
       </c>
       <c r="X4" s="15">
-        <f>N4</f>
+        <f>W4</f>
         <v/>
       </c>
       <c r="Y4" s="15">
-        <f>N4</f>
+        <f>X4</f>
         <v/>
       </c>
       <c r="Z4" s="15">
-        <f>N4</f>
+        <f>Y4</f>
         <v/>
       </c>
       <c r="AA4" s="15">
-        <f>N4</f>
+        <f>Z4</f>
         <v/>
       </c>
       <c r="AB4" s="15">
-        <f>N4</f>
+        <f>AA4</f>
         <v/>
       </c>
       <c r="AC4" s="15">
-        <f>N4</f>
+        <f>AB4</f>
         <v/>
       </c>
       <c r="AD4" s="15">
-        <f>N4</f>
+        <f>AC4</f>
         <v/>
       </c>
       <c r="AE4" s="15">
-        <f>N4</f>
+        <f>AD4</f>
         <v/>
       </c>
       <c r="AF4" s="15">
-        <f>N4</f>
+        <f>AE4</f>
         <v/>
       </c>
       <c r="AG4" s="15">
-        <f>N4</f>
+        <f>AF4</f>
         <v/>
       </c>
       <c r="AH4" s="15">
-        <f>N4</f>
+        <f>AG4</f>
         <v/>
       </c>
     </row>
@@ -10637,79 +10637,79 @@
         <v/>
       </c>
       <c r="P5" s="15">
-        <f>N5</f>
+        <f>O5</f>
         <v/>
       </c>
       <c r="Q5" s="15">
-        <f>N5</f>
+        <f>P5</f>
         <v/>
       </c>
       <c r="R5" s="15">
-        <f>N5</f>
+        <f>Q5</f>
         <v/>
       </c>
       <c r="S5" s="15">
-        <f>N5</f>
+        <f>R5</f>
         <v/>
       </c>
       <c r="T5" s="15">
-        <f>N5</f>
+        <f>S5</f>
         <v/>
       </c>
       <c r="U5" s="15">
-        <f>N5</f>
+        <f>T5</f>
         <v/>
       </c>
       <c r="V5" s="15">
-        <f>N5</f>
+        <f>U5</f>
         <v/>
       </c>
       <c r="W5" s="15">
-        <f>N5</f>
+        <f>V5</f>
         <v/>
       </c>
       <c r="X5" s="15">
-        <f>N5</f>
+        <f>W5</f>
         <v/>
       </c>
       <c r="Y5" s="15">
-        <f>N5</f>
+        <f>X5</f>
         <v/>
       </c>
       <c r="Z5" s="15">
-        <f>N5</f>
+        <f>Y5</f>
         <v/>
       </c>
       <c r="AA5" s="15">
-        <f>N5</f>
+        <f>Z5</f>
         <v/>
       </c>
       <c r="AB5" s="15">
-        <f>N5</f>
+        <f>AA5</f>
         <v/>
       </c>
       <c r="AC5" s="15">
-        <f>N5</f>
+        <f>AB5</f>
         <v/>
       </c>
       <c r="AD5" s="15">
-        <f>N5</f>
+        <f>AC5</f>
         <v/>
       </c>
       <c r="AE5" s="15">
-        <f>N5</f>
+        <f>AD5</f>
         <v/>
       </c>
       <c r="AF5" s="15">
-        <f>N5</f>
+        <f>AE5</f>
         <v/>
       </c>
       <c r="AG5" s="15">
-        <f>N5</f>
+        <f>AF5</f>
         <v/>
       </c>
       <c r="AH5" s="15">
-        <f>N5</f>
+        <f>AG5</f>
         <v/>
       </c>
     </row>
@@ -10776,79 +10776,79 @@
         <v/>
       </c>
       <c r="P6" s="15">
-        <f>N6</f>
+        <f>O6</f>
         <v/>
       </c>
       <c r="Q6" s="15">
-        <f>N6</f>
+        <f>P6</f>
         <v/>
       </c>
       <c r="R6" s="15">
-        <f>N6</f>
+        <f>Q6</f>
         <v/>
       </c>
       <c r="S6" s="15">
-        <f>N6</f>
+        <f>R6</f>
         <v/>
       </c>
       <c r="T6" s="15">
-        <f>N6</f>
+        <f>S6</f>
         <v/>
       </c>
       <c r="U6" s="15">
-        <f>N6</f>
+        <f>T6</f>
         <v/>
       </c>
       <c r="V6" s="15">
-        <f>N6</f>
+        <f>U6</f>
         <v/>
       </c>
       <c r="W6" s="15">
-        <f>N6</f>
+        <f>V6</f>
         <v/>
       </c>
       <c r="X6" s="15">
-        <f>N6</f>
+        <f>W6</f>
         <v/>
       </c>
       <c r="Y6" s="15">
-        <f>N6</f>
+        <f>X6</f>
         <v/>
       </c>
       <c r="Z6" s="15">
-        <f>N6</f>
+        <f>Y6</f>
         <v/>
       </c>
       <c r="AA6" s="15">
-        <f>N6</f>
+        <f>Z6</f>
         <v/>
       </c>
       <c r="AB6" s="15">
-        <f>N6</f>
+        <f>AA6</f>
         <v/>
       </c>
       <c r="AC6" s="15">
-        <f>N6</f>
+        <f>AB6</f>
         <v/>
       </c>
       <c r="AD6" s="15">
-        <f>N6</f>
+        <f>AC6</f>
         <v/>
       </c>
       <c r="AE6" s="15">
-        <f>N6</f>
+        <f>AD6</f>
         <v/>
       </c>
       <c r="AF6" s="15">
-        <f>N6</f>
+        <f>AE6</f>
         <v/>
       </c>
       <c r="AG6" s="15">
-        <f>N6</f>
+        <f>AF6</f>
         <v/>
       </c>
       <c r="AH6" s="15">
-        <f>N6</f>
+        <f>AG6</f>
         <v/>
       </c>
     </row>
@@ -10915,79 +10915,79 @@
         <v/>
       </c>
       <c r="P7" s="12">
-        <f>N7</f>
+        <f>O7</f>
         <v/>
       </c>
       <c r="Q7" s="12">
-        <f>N7</f>
+        <f>P7</f>
         <v/>
       </c>
       <c r="R7" s="12">
-        <f>N7</f>
+        <f>Q7</f>
         <v/>
       </c>
       <c r="S7" s="12">
-        <f>N7</f>
+        <f>R7</f>
         <v/>
       </c>
       <c r="T7" s="12">
-        <f>N7</f>
+        <f>S7</f>
         <v/>
       </c>
       <c r="U7" s="12">
-        <f>N7</f>
+        <f>T7</f>
         <v/>
       </c>
       <c r="V7" s="12">
-        <f>N7</f>
+        <f>U7</f>
         <v/>
       </c>
       <c r="W7" s="12">
-        <f>N7</f>
+        <f>V7</f>
         <v/>
       </c>
       <c r="X7" s="12">
-        <f>N7</f>
+        <f>W7</f>
         <v/>
       </c>
       <c r="Y7" s="12">
-        <f>N7</f>
+        <f>X7</f>
         <v/>
       </c>
       <c r="Z7" s="12">
-        <f>N7</f>
+        <f>Y7</f>
         <v/>
       </c>
       <c r="AA7" s="12">
-        <f>N7</f>
+        <f>Z7</f>
         <v/>
       </c>
       <c r="AB7" s="12">
-        <f>N7</f>
+        <f>AA7</f>
         <v/>
       </c>
       <c r="AC7" s="12">
-        <f>N7</f>
+        <f>AB7</f>
         <v/>
       </c>
       <c r="AD7" s="12">
-        <f>N7</f>
+        <f>AC7</f>
         <v/>
       </c>
       <c r="AE7" s="12">
-        <f>N7</f>
+        <f>AD7</f>
         <v/>
       </c>
       <c r="AF7" s="12">
-        <f>N7</f>
+        <f>AE7</f>
         <v/>
       </c>
       <c r="AG7" s="12">
-        <f>N7</f>
+        <f>AF7</f>
         <v/>
       </c>
       <c r="AH7" s="12">
-        <f>N7</f>
+        <f>AG7</f>
         <v/>
       </c>
     </row>
@@ -11054,79 +11054,79 @@
         <v/>
       </c>
       <c r="P8" s="12">
-        <f>N8</f>
+        <f>O8</f>
         <v/>
       </c>
       <c r="Q8" s="12">
-        <f>N8</f>
+        <f>P8</f>
         <v/>
       </c>
       <c r="R8" s="12">
-        <f>N8</f>
+        <f>Q8</f>
         <v/>
       </c>
       <c r="S8" s="12">
-        <f>N8</f>
+        <f>R8</f>
         <v/>
       </c>
       <c r="T8" s="12">
-        <f>N8</f>
+        <f>S8</f>
         <v/>
       </c>
       <c r="U8" s="12">
-        <f>N8</f>
+        <f>T8</f>
         <v/>
       </c>
       <c r="V8" s="12">
-        <f>N8</f>
+        <f>U8</f>
         <v/>
       </c>
       <c r="W8" s="12">
-        <f>N8</f>
+        <f>V8</f>
         <v/>
       </c>
       <c r="X8" s="12">
-        <f>N8</f>
+        <f>W8</f>
         <v/>
       </c>
       <c r="Y8" s="12">
-        <f>N8</f>
+        <f>X8</f>
         <v/>
       </c>
       <c r="Z8" s="12">
-        <f>N8</f>
+        <f>Y8</f>
         <v/>
       </c>
       <c r="AA8" s="12">
-        <f>N8</f>
+        <f>Z8</f>
         <v/>
       </c>
       <c r="AB8" s="12">
-        <f>N8</f>
+        <f>AA8</f>
         <v/>
       </c>
       <c r="AC8" s="12">
-        <f>N8</f>
+        <f>AB8</f>
         <v/>
       </c>
       <c r="AD8" s="12">
-        <f>N8</f>
+        <f>AC8</f>
         <v/>
       </c>
       <c r="AE8" s="12">
-        <f>N8</f>
+        <f>AD8</f>
         <v/>
       </c>
       <c r="AF8" s="12">
-        <f>N8</f>
+        <f>AE8</f>
         <v/>
       </c>
       <c r="AG8" s="12">
-        <f>N8</f>
+        <f>AF8</f>
         <v/>
       </c>
       <c r="AH8" s="12">
-        <f>N8</f>
+        <f>AG8</f>
         <v/>
       </c>
     </row>
@@ -11193,79 +11193,79 @@
         <v/>
       </c>
       <c r="P9" s="12">
-        <f>N9</f>
+        <f>O9</f>
         <v/>
       </c>
       <c r="Q9" s="12">
-        <f>N9</f>
+        <f>P9</f>
         <v/>
       </c>
       <c r="R9" s="12">
-        <f>N9</f>
+        <f>Q9</f>
         <v/>
       </c>
       <c r="S9" s="12">
-        <f>N9</f>
+        <f>R9</f>
         <v/>
       </c>
       <c r="T9" s="12">
-        <f>N9</f>
+        <f>S9</f>
         <v/>
       </c>
       <c r="U9" s="12">
-        <f>N9</f>
+        <f>T9</f>
         <v/>
       </c>
       <c r="V9" s="12">
-        <f>N9</f>
+        <f>U9</f>
         <v/>
       </c>
       <c r="W9" s="12">
-        <f>N9</f>
+        <f>V9</f>
         <v/>
       </c>
       <c r="X9" s="12">
-        <f>N9</f>
+        <f>W9</f>
         <v/>
       </c>
       <c r="Y9" s="12">
-        <f>N9</f>
+        <f>X9</f>
         <v/>
       </c>
       <c r="Z9" s="12">
-        <f>N9</f>
+        <f>Y9</f>
         <v/>
       </c>
       <c r="AA9" s="12">
-        <f>N9</f>
+        <f>Z9</f>
         <v/>
       </c>
       <c r="AB9" s="12">
-        <f>N9</f>
+        <f>AA9</f>
         <v/>
       </c>
       <c r="AC9" s="12">
-        <f>N9</f>
+        <f>AB9</f>
         <v/>
       </c>
       <c r="AD9" s="12">
-        <f>N9</f>
+        <f>AC9</f>
         <v/>
       </c>
       <c r="AE9" s="12">
-        <f>N9</f>
+        <f>AD9</f>
         <v/>
       </c>
       <c r="AF9" s="12">
-        <f>N9</f>
+        <f>AE9</f>
         <v/>
       </c>
       <c r="AG9" s="12">
-        <f>N9</f>
+        <f>AF9</f>
         <v/>
       </c>
       <c r="AH9" s="12">
-        <f>N9</f>
+        <f>AG9</f>
         <v/>
       </c>
     </row>
@@ -11471,79 +11471,79 @@
         <v/>
       </c>
       <c r="P11" s="12">
-        <f>N11</f>
+        <f>O11</f>
         <v/>
       </c>
       <c r="Q11" s="12">
-        <f>N11</f>
+        <f>P11</f>
         <v/>
       </c>
       <c r="R11" s="12">
-        <f>N11</f>
+        <f>Q11</f>
         <v/>
       </c>
       <c r="S11" s="12">
-        <f>N11</f>
+        <f>R11</f>
         <v/>
       </c>
       <c r="T11" s="12">
-        <f>N11</f>
+        <f>S11</f>
         <v/>
       </c>
       <c r="U11" s="12">
-        <f>N11</f>
+        <f>T11</f>
         <v/>
       </c>
       <c r="V11" s="12">
-        <f>N11</f>
+        <f>U11</f>
         <v/>
       </c>
       <c r="W11" s="12">
-        <f>N11</f>
+        <f>V11</f>
         <v/>
       </c>
       <c r="X11" s="12">
-        <f>N11</f>
+        <f>W11</f>
         <v/>
       </c>
       <c r="Y11" s="12">
-        <f>N11</f>
+        <f>X11</f>
         <v/>
       </c>
       <c r="Z11" s="12">
-        <f>N11</f>
+        <f>Y11</f>
         <v/>
       </c>
       <c r="AA11" s="12">
-        <f>N11</f>
+        <f>Z11</f>
         <v/>
       </c>
       <c r="AB11" s="12">
-        <f>N11</f>
+        <f>AA11</f>
         <v/>
       </c>
       <c r="AC11" s="12">
-        <f>N11</f>
+        <f>AB11</f>
         <v/>
       </c>
       <c r="AD11" s="12">
-        <f>N11</f>
+        <f>AC11</f>
         <v/>
       </c>
       <c r="AE11" s="12">
-        <f>N11</f>
+        <f>AD11</f>
         <v/>
       </c>
       <c r="AF11" s="12">
-        <f>N11</f>
+        <f>AE11</f>
         <v/>
       </c>
       <c r="AG11" s="12">
-        <f>N11</f>
+        <f>AF11</f>
         <v/>
       </c>
       <c r="AH11" s="12">
-        <f>N11</f>
+        <f>AG11</f>
         <v/>
       </c>
     </row>
@@ -11610,79 +11610,79 @@
         <v/>
       </c>
       <c r="P12" s="13">
-        <f>N12</f>
+        <f>O12</f>
         <v/>
       </c>
       <c r="Q12" s="13">
-        <f>N12</f>
+        <f>P12</f>
         <v/>
       </c>
       <c r="R12" s="13">
-        <f>N12</f>
+        <f>Q12</f>
         <v/>
       </c>
       <c r="S12" s="13">
-        <f>N12</f>
+        <f>R12</f>
         <v/>
       </c>
       <c r="T12" s="13">
-        <f>N12</f>
+        <f>S12</f>
         <v/>
       </c>
       <c r="U12" s="13">
-        <f>N12</f>
+        <f>T12</f>
         <v/>
       </c>
       <c r="V12" s="13">
-        <f>N12</f>
+        <f>U12</f>
         <v/>
       </c>
       <c r="W12" s="13">
-        <f>N12</f>
+        <f>V12</f>
         <v/>
       </c>
       <c r="X12" s="13">
-        <f>N12</f>
+        <f>W12</f>
         <v/>
       </c>
       <c r="Y12" s="13">
-        <f>N12</f>
+        <f>X12</f>
         <v/>
       </c>
       <c r="Z12" s="13">
-        <f>N12</f>
+        <f>Y12</f>
         <v/>
       </c>
       <c r="AA12" s="13">
-        <f>N12</f>
+        <f>Z12</f>
         <v/>
       </c>
       <c r="AB12" s="13">
-        <f>N12</f>
+        <f>AA12</f>
         <v/>
       </c>
       <c r="AC12" s="13">
-        <f>N12</f>
+        <f>AB12</f>
         <v/>
       </c>
       <c r="AD12" s="13">
-        <f>N12</f>
+        <f>AC12</f>
         <v/>
       </c>
       <c r="AE12" s="13">
-        <f>N12</f>
+        <f>AD12</f>
         <v/>
       </c>
       <c r="AF12" s="13">
-        <f>N12</f>
+        <f>AE12</f>
         <v/>
       </c>
       <c r="AG12" s="13">
-        <f>N12</f>
+        <f>AF12</f>
         <v/>
       </c>
       <c r="AH12" s="13">
-        <f>N12</f>
+        <f>AG12</f>
         <v/>
       </c>
     </row>
@@ -11749,79 +11749,79 @@
         <v/>
       </c>
       <c r="P13" s="13">
-        <f>N13</f>
+        <f>O13</f>
         <v/>
       </c>
       <c r="Q13" s="13">
-        <f>N13</f>
+        <f>P13</f>
         <v/>
       </c>
       <c r="R13" s="13">
-        <f>N13</f>
+        <f>Q13</f>
         <v/>
       </c>
       <c r="S13" s="13">
-        <f>N13</f>
+        <f>R13</f>
         <v/>
       </c>
       <c r="T13" s="13">
-        <f>N13</f>
+        <f>S13</f>
         <v/>
       </c>
       <c r="U13" s="13">
-        <f>N13</f>
+        <f>T13</f>
         <v/>
       </c>
       <c r="V13" s="13">
-        <f>N13</f>
+        <f>U13</f>
         <v/>
       </c>
       <c r="W13" s="13">
-        <f>N13</f>
+        <f>V13</f>
         <v/>
       </c>
       <c r="X13" s="13">
-        <f>N13</f>
+        <f>W13</f>
         <v/>
       </c>
       <c r="Y13" s="13">
-        <f>N13</f>
+        <f>X13</f>
         <v/>
       </c>
       <c r="Z13" s="13">
-        <f>N13</f>
+        <f>Y13</f>
         <v/>
       </c>
       <c r="AA13" s="13">
-        <f>N13</f>
+        <f>Z13</f>
         <v/>
       </c>
       <c r="AB13" s="13">
-        <f>N13</f>
+        <f>AA13</f>
         <v/>
       </c>
       <c r="AC13" s="13">
-        <f>N13</f>
+        <f>AB13</f>
         <v/>
       </c>
       <c r="AD13" s="13">
-        <f>N13</f>
+        <f>AC13</f>
         <v/>
       </c>
       <c r="AE13" s="13">
-        <f>N13</f>
+        <f>AD13</f>
         <v/>
       </c>
       <c r="AF13" s="13">
-        <f>N13</f>
+        <f>AE13</f>
         <v/>
       </c>
       <c r="AG13" s="13">
-        <f>N13</f>
+        <f>AF13</f>
         <v/>
       </c>
       <c r="AH13" s="13">
-        <f>N13</f>
+        <f>AG13</f>
         <v/>
       </c>
     </row>
@@ -11888,79 +11888,79 @@
         <v/>
       </c>
       <c r="P14" s="12">
-        <f>N14</f>
+        <f>O14</f>
         <v/>
       </c>
       <c r="Q14" s="12">
-        <f>N14</f>
+        <f>P14</f>
         <v/>
       </c>
       <c r="R14" s="12">
-        <f>N14</f>
+        <f>Q14</f>
         <v/>
       </c>
       <c r="S14" s="12">
-        <f>N14</f>
+        <f>R14</f>
         <v/>
       </c>
       <c r="T14" s="12">
-        <f>N14</f>
+        <f>S14</f>
         <v/>
       </c>
       <c r="U14" s="12">
-        <f>N14</f>
+        <f>T14</f>
         <v/>
       </c>
       <c r="V14" s="12">
-        <f>N14</f>
+        <f>U14</f>
         <v/>
       </c>
       <c r="W14" s="12">
-        <f>N14</f>
+        <f>V14</f>
         <v/>
       </c>
       <c r="X14" s="12">
-        <f>N14</f>
+        <f>W14</f>
         <v/>
       </c>
       <c r="Y14" s="12">
-        <f>N14</f>
+        <f>X14</f>
         <v/>
       </c>
       <c r="Z14" s="12">
-        <f>N14</f>
+        <f>Y14</f>
         <v/>
       </c>
       <c r="AA14" s="12">
-        <f>N14</f>
+        <f>Z14</f>
         <v/>
       </c>
       <c r="AB14" s="12">
-        <f>N14</f>
+        <f>AA14</f>
         <v/>
       </c>
       <c r="AC14" s="12">
-        <f>N14</f>
+        <f>AB14</f>
         <v/>
       </c>
       <c r="AD14" s="12">
-        <f>N14</f>
+        <f>AC14</f>
         <v/>
       </c>
       <c r="AE14" s="12">
-        <f>N14</f>
+        <f>AD14</f>
         <v/>
       </c>
       <c r="AF14" s="12">
-        <f>N14</f>
+        <f>AE14</f>
         <v/>
       </c>
       <c r="AG14" s="12">
-        <f>N14</f>
+        <f>AF14</f>
         <v/>
       </c>
       <c r="AH14" s="12">
-        <f>N14</f>
+        <f>AG14</f>
         <v/>
       </c>
     </row>
@@ -12166,79 +12166,79 @@
         <v/>
       </c>
       <c r="P16" s="12">
-        <f>N16</f>
+        <f>O16</f>
         <v/>
       </c>
       <c r="Q16" s="12">
-        <f>N16</f>
+        <f>P16</f>
         <v/>
       </c>
       <c r="R16" s="12">
-        <f>N16</f>
+        <f>Q16</f>
         <v/>
       </c>
       <c r="S16" s="12">
-        <f>N16</f>
+        <f>R16</f>
         <v/>
       </c>
       <c r="T16" s="12">
-        <f>N16</f>
+        <f>S16</f>
         <v/>
       </c>
       <c r="U16" s="12">
-        <f>N16</f>
+        <f>T16</f>
         <v/>
       </c>
       <c r="V16" s="12">
-        <f>N16</f>
+        <f>U16</f>
         <v/>
       </c>
       <c r="W16" s="12">
-        <f>N16</f>
+        <f>V16</f>
         <v/>
       </c>
       <c r="X16" s="12">
-        <f>N16</f>
+        <f>W16</f>
         <v/>
       </c>
       <c r="Y16" s="12">
-        <f>N16</f>
+        <f>X16</f>
         <v/>
       </c>
       <c r="Z16" s="12">
-        <f>N16</f>
+        <f>Y16</f>
         <v/>
       </c>
       <c r="AA16" s="12">
-        <f>N16</f>
+        <f>Z16</f>
         <v/>
       </c>
       <c r="AB16" s="12">
-        <f>N16</f>
+        <f>AA16</f>
         <v/>
       </c>
       <c r="AC16" s="12">
-        <f>N16</f>
+        <f>AB16</f>
         <v/>
       </c>
       <c r="AD16" s="12">
-        <f>N16</f>
+        <f>AC16</f>
         <v/>
       </c>
       <c r="AE16" s="12">
-        <f>N16</f>
+        <f>AD16</f>
         <v/>
       </c>
       <c r="AF16" s="12">
-        <f>N16</f>
+        <f>AE16</f>
         <v/>
       </c>
       <c r="AG16" s="12">
-        <f>N16</f>
+        <f>AF16</f>
         <v/>
       </c>
       <c r="AH16" s="12">
-        <f>N16</f>
+        <f>AG16</f>
         <v/>
       </c>
     </row>
@@ -12305,79 +12305,79 @@
         <v/>
       </c>
       <c r="P17" s="12">
-        <f>N17</f>
+        <f>O17</f>
         <v/>
       </c>
       <c r="Q17" s="12">
-        <f>N17</f>
+        <f>P17</f>
         <v/>
       </c>
       <c r="R17" s="12">
-        <f>N17</f>
+        <f>Q17</f>
         <v/>
       </c>
       <c r="S17" s="12">
-        <f>N17</f>
+        <f>R17</f>
         <v/>
       </c>
       <c r="T17" s="12">
-        <f>N17</f>
+        <f>S17</f>
         <v/>
       </c>
       <c r="U17" s="12">
-        <f>N17</f>
+        <f>T17</f>
         <v/>
       </c>
       <c r="V17" s="12">
-        <f>N17</f>
+        <f>U17</f>
         <v/>
       </c>
       <c r="W17" s="12">
-        <f>N17</f>
+        <f>V17</f>
         <v/>
       </c>
       <c r="X17" s="12">
-        <f>N17</f>
+        <f>W17</f>
         <v/>
       </c>
       <c r="Y17" s="12">
-        <f>N17</f>
+        <f>X17</f>
         <v/>
       </c>
       <c r="Z17" s="12">
-        <f>N17</f>
+        <f>Y17</f>
         <v/>
       </c>
       <c r="AA17" s="12">
-        <f>N17</f>
+        <f>Z17</f>
         <v/>
       </c>
       <c r="AB17" s="12">
-        <f>N17</f>
+        <f>AA17</f>
         <v/>
       </c>
       <c r="AC17" s="12">
-        <f>N17</f>
+        <f>AB17</f>
         <v/>
       </c>
       <c r="AD17" s="12">
-        <f>N17</f>
+        <f>AC17</f>
         <v/>
       </c>
       <c r="AE17" s="12">
-        <f>N17</f>
+        <f>AD17</f>
         <v/>
       </c>
       <c r="AF17" s="12">
-        <f>N17</f>
+        <f>AE17</f>
         <v/>
       </c>
       <c r="AG17" s="12">
-        <f>N17</f>
+        <f>AF17</f>
         <v/>
       </c>
       <c r="AH17" s="12">
-        <f>N17</f>
+        <f>AG17</f>
         <v/>
       </c>
     </row>
@@ -12444,79 +12444,79 @@
         <v/>
       </c>
       <c r="P18" s="15">
-        <f>N18</f>
+        <f>O18</f>
         <v/>
       </c>
       <c r="Q18" s="15">
-        <f>N18</f>
+        <f>P18</f>
         <v/>
       </c>
       <c r="R18" s="15">
-        <f>N18</f>
+        <f>Q18</f>
         <v/>
       </c>
       <c r="S18" s="15">
-        <f>N18</f>
+        <f>R18</f>
         <v/>
       </c>
       <c r="T18" s="15">
-        <f>N18</f>
+        <f>S18</f>
         <v/>
       </c>
       <c r="U18" s="15">
-        <f>N18</f>
+        <f>T18</f>
         <v/>
       </c>
       <c r="V18" s="15">
-        <f>N18</f>
+        <f>U18</f>
         <v/>
       </c>
       <c r="W18" s="15">
-        <f>N18</f>
+        <f>V18</f>
         <v/>
       </c>
       <c r="X18" s="15">
-        <f>N18</f>
+        <f>W18</f>
         <v/>
       </c>
       <c r="Y18" s="15">
-        <f>N18</f>
+        <f>X18</f>
         <v/>
       </c>
       <c r="Z18" s="15">
-        <f>N18</f>
+        <f>Y18</f>
         <v/>
       </c>
       <c r="AA18" s="15">
-        <f>N18</f>
+        <f>Z18</f>
         <v/>
       </c>
       <c r="AB18" s="15">
-        <f>N18</f>
+        <f>AA18</f>
         <v/>
       </c>
       <c r="AC18" s="15">
-        <f>N18</f>
+        <f>AB18</f>
         <v/>
       </c>
       <c r="AD18" s="15">
-        <f>N18</f>
+        <f>AC18</f>
         <v/>
       </c>
       <c r="AE18" s="15">
-        <f>N18</f>
+        <f>AD18</f>
         <v/>
       </c>
       <c r="AF18" s="15">
-        <f>N18</f>
+        <f>AE18</f>
         <v/>
       </c>
       <c r="AG18" s="15">
-        <f>N18</f>
+        <f>AF18</f>
         <v/>
       </c>
       <c r="AH18" s="15">
-        <f>N18</f>
+        <f>AG18</f>
         <v/>
       </c>
     </row>
@@ -12583,79 +12583,79 @@
         <v/>
       </c>
       <c r="P19" s="12">
-        <f>N19</f>
+        <f>O19</f>
         <v/>
       </c>
       <c r="Q19" s="12">
-        <f>N19</f>
+        <f>P19</f>
         <v/>
       </c>
       <c r="R19" s="12">
-        <f>N19</f>
+        <f>Q19</f>
         <v/>
       </c>
       <c r="S19" s="12">
-        <f>N19</f>
+        <f>R19</f>
         <v/>
       </c>
       <c r="T19" s="12">
-        <f>N19</f>
+        <f>S19</f>
         <v/>
       </c>
       <c r="U19" s="12">
-        <f>N19</f>
+        <f>T19</f>
         <v/>
       </c>
       <c r="V19" s="12">
-        <f>N19</f>
+        <f>U19</f>
         <v/>
       </c>
       <c r="W19" s="12">
-        <f>N19</f>
+        <f>V19</f>
         <v/>
       </c>
       <c r="X19" s="12">
-        <f>N19</f>
+        <f>W19</f>
         <v/>
       </c>
       <c r="Y19" s="12">
-        <f>N19</f>
+        <f>X19</f>
         <v/>
       </c>
       <c r="Z19" s="12">
-        <f>N19</f>
+        <f>Y19</f>
         <v/>
       </c>
       <c r="AA19" s="12">
-        <f>N19</f>
+        <f>Z19</f>
         <v/>
       </c>
       <c r="AB19" s="12">
-        <f>N19</f>
+        <f>AA19</f>
         <v/>
       </c>
       <c r="AC19" s="12">
-        <f>N19</f>
+        <f>AB19</f>
         <v/>
       </c>
       <c r="AD19" s="12">
-        <f>N19</f>
+        <f>AC19</f>
         <v/>
       </c>
       <c r="AE19" s="12">
-        <f>N19</f>
+        <f>AD19</f>
         <v/>
       </c>
       <c r="AF19" s="12">
-        <f>N19</f>
+        <f>AE19</f>
         <v/>
       </c>
       <c r="AG19" s="12">
-        <f>N19</f>
+        <f>AF19</f>
         <v/>
       </c>
       <c r="AH19" s="12">
-        <f>N19</f>
+        <f>AG19</f>
         <v/>
       </c>
     </row>
@@ -12722,79 +12722,79 @@
         <v/>
       </c>
       <c r="P20" s="12">
-        <f>N20</f>
+        <f>O20</f>
         <v/>
       </c>
       <c r="Q20" s="12">
-        <f>N20</f>
+        <f>P20</f>
         <v/>
       </c>
       <c r="R20" s="12">
-        <f>N20</f>
+        <f>Q20</f>
         <v/>
       </c>
       <c r="S20" s="12">
-        <f>N20</f>
+        <f>R20</f>
         <v/>
       </c>
       <c r="T20" s="12">
-        <f>N20</f>
+        <f>S20</f>
         <v/>
       </c>
       <c r="U20" s="12">
-        <f>N20</f>
+        <f>T20</f>
         <v/>
       </c>
       <c r="V20" s="12">
-        <f>N20</f>
+        <f>U20</f>
         <v/>
       </c>
       <c r="W20" s="12">
-        <f>N20</f>
+        <f>V20</f>
         <v/>
       </c>
       <c r="X20" s="12">
-        <f>N20</f>
+        <f>W20</f>
         <v/>
       </c>
       <c r="Y20" s="12">
-        <f>N20</f>
+        <f>X20</f>
         <v/>
       </c>
       <c r="Z20" s="12">
-        <f>N20</f>
+        <f>Y20</f>
         <v/>
       </c>
       <c r="AA20" s="12">
-        <f>N20</f>
+        <f>Z20</f>
         <v/>
       </c>
       <c r="AB20" s="12">
-        <f>N20</f>
+        <f>AA20</f>
         <v/>
       </c>
       <c r="AC20" s="12">
-        <f>N20</f>
+        <f>AB20</f>
         <v/>
       </c>
       <c r="AD20" s="12">
-        <f>N20</f>
+        <f>AC20</f>
         <v/>
       </c>
       <c r="AE20" s="12">
-        <f>N20</f>
+        <f>AD20</f>
         <v/>
       </c>
       <c r="AF20" s="12">
-        <f>N20</f>
+        <f>AE20</f>
         <v/>
       </c>
       <c r="AG20" s="12">
-        <f>N20</f>
+        <f>AF20</f>
         <v/>
       </c>
       <c r="AH20" s="12">
-        <f>N20</f>
+        <f>AG20</f>
         <v/>
       </c>
     </row>
@@ -12980,79 +12980,79 @@
         <v/>
       </c>
       <c r="P22" s="12">
-        <f>N22</f>
+        <f>O22</f>
         <v/>
       </c>
       <c r="Q22" s="12">
-        <f>N22</f>
+        <f>P22</f>
         <v/>
       </c>
       <c r="R22" s="12">
-        <f>N22</f>
+        <f>Q22</f>
         <v/>
       </c>
       <c r="S22" s="12">
-        <f>N22</f>
+        <f>R22</f>
         <v/>
       </c>
       <c r="T22" s="12">
-        <f>N22</f>
+        <f>S22</f>
         <v/>
       </c>
       <c r="U22" s="12">
-        <f>N22</f>
+        <f>T22</f>
         <v/>
       </c>
       <c r="V22" s="12">
-        <f>N22</f>
+        <f>U22</f>
         <v/>
       </c>
       <c r="W22" s="12">
-        <f>N22</f>
+        <f>V22</f>
         <v/>
       </c>
       <c r="X22" s="12">
-        <f>N22</f>
+        <f>W22</f>
         <v/>
       </c>
       <c r="Y22" s="12">
-        <f>N22</f>
+        <f>X22</f>
         <v/>
       </c>
       <c r="Z22" s="12">
-        <f>N22</f>
+        <f>Y22</f>
         <v/>
       </c>
       <c r="AA22" s="12">
-        <f>N22</f>
+        <f>Z22</f>
         <v/>
       </c>
       <c r="AB22" s="12">
-        <f>N22</f>
+        <f>AA22</f>
         <v/>
       </c>
       <c r="AC22" s="12">
-        <f>N22</f>
+        <f>AB22</f>
         <v/>
       </c>
       <c r="AD22" s="12">
-        <f>N22</f>
+        <f>AC22</f>
         <v/>
       </c>
       <c r="AE22" s="12">
-        <f>N22</f>
+        <f>AD22</f>
         <v/>
       </c>
       <c r="AF22" s="12">
-        <f>N22</f>
+        <f>AE22</f>
         <v/>
       </c>
       <c r="AG22" s="12">
-        <f>N22</f>
+        <f>AF22</f>
         <v/>
       </c>
       <c r="AH22" s="12">
-        <f>N22</f>
+        <f>AG22</f>
         <v/>
       </c>
     </row>
@@ -13119,79 +13119,79 @@
         <v/>
       </c>
       <c r="P23" s="12">
-        <f>N23</f>
+        <f>O23</f>
         <v/>
       </c>
       <c r="Q23" s="12">
-        <f>N23</f>
+        <f>P23</f>
         <v/>
       </c>
       <c r="R23" s="12">
-        <f>N23</f>
+        <f>Q23</f>
         <v/>
       </c>
       <c r="S23" s="12">
-        <f>N23</f>
+        <f>R23</f>
         <v/>
       </c>
       <c r="T23" s="12">
-        <f>N23</f>
+        <f>S23</f>
         <v/>
       </c>
       <c r="U23" s="12">
-        <f>N23</f>
+        <f>T23</f>
         <v/>
       </c>
       <c r="V23" s="12">
-        <f>N23</f>
+        <f>U23</f>
         <v/>
       </c>
       <c r="W23" s="12">
-        <f>N23</f>
+        <f>V23</f>
         <v/>
       </c>
       <c r="X23" s="12">
-        <f>N23</f>
+        <f>W23</f>
         <v/>
       </c>
       <c r="Y23" s="12">
-        <f>N23</f>
+        <f>X23</f>
         <v/>
       </c>
       <c r="Z23" s="12">
-        <f>N23</f>
+        <f>Y23</f>
         <v/>
       </c>
       <c r="AA23" s="12">
-        <f>N23</f>
+        <f>Z23</f>
         <v/>
       </c>
       <c r="AB23" s="12">
-        <f>N23</f>
+        <f>AA23</f>
         <v/>
       </c>
       <c r="AC23" s="12">
-        <f>N23</f>
+        <f>AB23</f>
         <v/>
       </c>
       <c r="AD23" s="12">
-        <f>N23</f>
+        <f>AC23</f>
         <v/>
       </c>
       <c r="AE23" s="12">
-        <f>N23</f>
+        <f>AD23</f>
         <v/>
       </c>
       <c r="AF23" s="12">
-        <f>N23</f>
+        <f>AE23</f>
         <v/>
       </c>
       <c r="AG23" s="12">
-        <f>N23</f>
+        <f>AF23</f>
         <v/>
       </c>
       <c r="AH23" s="12">
-        <f>N23</f>
+        <f>AG23</f>
         <v/>
       </c>
     </row>
@@ -13258,79 +13258,79 @@
         <v/>
       </c>
       <c r="P24" s="12">
-        <f>N24</f>
+        <f>O24</f>
         <v/>
       </c>
       <c r="Q24" s="12">
-        <f>N24</f>
+        <f>P24</f>
         <v/>
       </c>
       <c r="R24" s="12">
-        <f>N24</f>
+        <f>Q24</f>
         <v/>
       </c>
       <c r="S24" s="12">
-        <f>N24</f>
+        <f>R24</f>
         <v/>
       </c>
       <c r="T24" s="12">
-        <f>N24</f>
+        <f>S24</f>
         <v/>
       </c>
       <c r="U24" s="12">
-        <f>N24</f>
+        <f>T24</f>
         <v/>
       </c>
       <c r="V24" s="12">
-        <f>N24</f>
+        <f>U24</f>
         <v/>
       </c>
       <c r="W24" s="12">
-        <f>N24</f>
+        <f>V24</f>
         <v/>
       </c>
       <c r="X24" s="12">
-        <f>N24</f>
+        <f>W24</f>
         <v/>
       </c>
       <c r="Y24" s="12">
-        <f>N24</f>
+        <f>X24</f>
         <v/>
       </c>
       <c r="Z24" s="12">
-        <f>N24</f>
+        <f>Y24</f>
         <v/>
       </c>
       <c r="AA24" s="12">
-        <f>N24</f>
+        <f>Z24</f>
         <v/>
       </c>
       <c r="AB24" s="12">
-        <f>N24</f>
+        <f>AA24</f>
         <v/>
       </c>
       <c r="AC24" s="12">
-        <f>N24</f>
+        <f>AB24</f>
         <v/>
       </c>
       <c r="AD24" s="12">
-        <f>N24</f>
+        <f>AC24</f>
         <v/>
       </c>
       <c r="AE24" s="12">
-        <f>N24</f>
+        <f>AD24</f>
         <v/>
       </c>
       <c r="AF24" s="12">
-        <f>N24</f>
+        <f>AE24</f>
         <v/>
       </c>
       <c r="AG24" s="12">
-        <f>N24</f>
+        <f>AF24</f>
         <v/>
       </c>
       <c r="AH24" s="12">
-        <f>N24</f>
+        <f>AG24</f>
         <v/>
       </c>
     </row>
@@ -13397,79 +13397,79 @@
         <v/>
       </c>
       <c r="P25" s="12">
-        <f>N25</f>
+        <f>O25</f>
         <v/>
       </c>
       <c r="Q25" s="12">
-        <f>N25</f>
+        <f>P25</f>
         <v/>
       </c>
       <c r="R25" s="12">
-        <f>N25</f>
+        <f>Q25</f>
         <v/>
       </c>
       <c r="S25" s="12">
-        <f>N25</f>
+        <f>R25</f>
         <v/>
       </c>
       <c r="T25" s="12">
-        <f>N25</f>
+        <f>S25</f>
         <v/>
       </c>
       <c r="U25" s="12">
-        <f>N25</f>
+        <f>T25</f>
         <v/>
       </c>
       <c r="V25" s="12">
-        <f>N25</f>
+        <f>U25</f>
         <v/>
       </c>
       <c r="W25" s="12">
-        <f>N25</f>
+        <f>V25</f>
         <v/>
       </c>
       <c r="X25" s="12">
-        <f>N25</f>
+        <f>W25</f>
         <v/>
       </c>
       <c r="Y25" s="12">
-        <f>N25</f>
+        <f>X25</f>
         <v/>
       </c>
       <c r="Z25" s="12">
-        <f>N25</f>
+        <f>Y25</f>
         <v/>
       </c>
       <c r="AA25" s="12">
-        <f>N25</f>
+        <f>Z25</f>
         <v/>
       </c>
       <c r="AB25" s="12">
-        <f>N25</f>
+        <f>AA25</f>
         <v/>
       </c>
       <c r="AC25" s="12">
-        <f>N25</f>
+        <f>AB25</f>
         <v/>
       </c>
       <c r="AD25" s="12">
-        <f>N25</f>
+        <f>AC25</f>
         <v/>
       </c>
       <c r="AE25" s="12">
-        <f>N25</f>
+        <f>AD25</f>
         <v/>
       </c>
       <c r="AF25" s="12">
-        <f>N25</f>
+        <f>AE25</f>
         <v/>
       </c>
       <c r="AG25" s="12">
-        <f>N25</f>
+        <f>AF25</f>
         <v/>
       </c>
       <c r="AH25" s="12">
-        <f>N25</f>
+        <f>AG25</f>
         <v/>
       </c>
     </row>
@@ -13536,79 +13536,79 @@
         <v/>
       </c>
       <c r="P26" s="12">
-        <f>N26</f>
+        <f>O26</f>
         <v/>
       </c>
       <c r="Q26" s="12">
-        <f>N26</f>
+        <f>P26</f>
         <v/>
       </c>
       <c r="R26" s="12">
-        <f>N26</f>
+        <f>Q26</f>
         <v/>
       </c>
       <c r="S26" s="12">
-        <f>N26</f>
+        <f>R26</f>
         <v/>
       </c>
       <c r="T26" s="12">
-        <f>N26</f>
+        <f>S26</f>
         <v/>
       </c>
       <c r="U26" s="12">
-        <f>N26</f>
+        <f>T26</f>
         <v/>
       </c>
       <c r="V26" s="12">
-        <f>N26</f>
+        <f>U26</f>
         <v/>
       </c>
       <c r="W26" s="12">
-        <f>N26</f>
+        <f>V26</f>
         <v/>
       </c>
       <c r="X26" s="12">
-        <f>N26</f>
+        <f>W26</f>
         <v/>
       </c>
       <c r="Y26" s="12">
-        <f>N26</f>
+        <f>X26</f>
         <v/>
       </c>
       <c r="Z26" s="12">
-        <f>N26</f>
+        <f>Y26</f>
         <v/>
       </c>
       <c r="AA26" s="12">
-        <f>N26</f>
+        <f>Z26</f>
         <v/>
       </c>
       <c r="AB26" s="12">
-        <f>N26</f>
+        <f>AA26</f>
         <v/>
       </c>
       <c r="AC26" s="12">
-        <f>N26</f>
+        <f>AB26</f>
         <v/>
       </c>
       <c r="AD26" s="12">
-        <f>N26</f>
+        <f>AC26</f>
         <v/>
       </c>
       <c r="AE26" s="12">
-        <f>N26</f>
+        <f>AD26</f>
         <v/>
       </c>
       <c r="AF26" s="12">
-        <f>N26</f>
+        <f>AE26</f>
         <v/>
       </c>
       <c r="AG26" s="12">
-        <f>N26</f>
+        <f>AF26</f>
         <v/>
       </c>
       <c r="AH26" s="12">
-        <f>N26</f>
+        <f>AG26</f>
         <v/>
       </c>
     </row>
@@ -13675,79 +13675,79 @@
         <v/>
       </c>
       <c r="P27" s="12">
-        <f>N27</f>
+        <f>O27</f>
         <v/>
       </c>
       <c r="Q27" s="12">
-        <f>N27</f>
+        <f>P27</f>
         <v/>
       </c>
       <c r="R27" s="12">
-        <f>N27</f>
+        <f>Q27</f>
         <v/>
       </c>
       <c r="S27" s="12">
-        <f>N27</f>
+        <f>R27</f>
         <v/>
       </c>
       <c r="T27" s="12">
-        <f>N27</f>
+        <f>S27</f>
         <v/>
       </c>
       <c r="U27" s="12">
-        <f>N27</f>
+        <f>T27</f>
         <v/>
       </c>
       <c r="V27" s="12">
-        <f>N27</f>
+        <f>U27</f>
         <v/>
       </c>
       <c r="W27" s="12">
-        <f>N27</f>
+        <f>V27</f>
         <v/>
       </c>
       <c r="X27" s="12">
-        <f>N27</f>
+        <f>W27</f>
         <v/>
       </c>
       <c r="Y27" s="12">
-        <f>N27</f>
+        <f>X27</f>
         <v/>
       </c>
       <c r="Z27" s="12">
-        <f>N27</f>
+        <f>Y27</f>
         <v/>
       </c>
       <c r="AA27" s="12">
-        <f>N27</f>
+        <f>Z27</f>
         <v/>
       </c>
       <c r="AB27" s="12">
-        <f>N27</f>
+        <f>AA27</f>
         <v/>
       </c>
       <c r="AC27" s="12">
-        <f>N27</f>
+        <f>AB27</f>
         <v/>
       </c>
       <c r="AD27" s="12">
-        <f>N27</f>
+        <f>AC27</f>
         <v/>
       </c>
       <c r="AE27" s="12">
-        <f>N27</f>
+        <f>AD27</f>
         <v/>
       </c>
       <c r="AF27" s="12">
-        <f>N27</f>
+        <f>AE27</f>
         <v/>
       </c>
       <c r="AG27" s="12">
-        <f>N27</f>
+        <f>AF27</f>
         <v/>
       </c>
       <c r="AH27" s="12">
-        <f>N27</f>
+        <f>AG27</f>
         <v/>
       </c>
     </row>
@@ -13814,79 +13814,79 @@
         <v/>
       </c>
       <c r="P28" s="12">
-        <f>N28</f>
+        <f>O28</f>
         <v/>
       </c>
       <c r="Q28" s="12">
-        <f>N28</f>
+        <f>P28</f>
         <v/>
       </c>
       <c r="R28" s="12">
-        <f>N28</f>
+        <f>Q28</f>
         <v/>
       </c>
       <c r="S28" s="12">
-        <f>N28</f>
+        <f>R28</f>
         <v/>
       </c>
       <c r="T28" s="12">
-        <f>N28</f>
+        <f>S28</f>
         <v/>
       </c>
       <c r="U28" s="12">
-        <f>N28</f>
+        <f>T28</f>
         <v/>
       </c>
       <c r="V28" s="12">
-        <f>N28</f>
+        <f>U28</f>
         <v/>
       </c>
       <c r="W28" s="12">
-        <f>N28</f>
+        <f>V28</f>
         <v/>
       </c>
       <c r="X28" s="12">
-        <f>N28</f>
+        <f>W28</f>
         <v/>
       </c>
       <c r="Y28" s="12">
-        <f>N28</f>
+        <f>X28</f>
         <v/>
       </c>
       <c r="Z28" s="12">
-        <f>N28</f>
+        <f>Y28</f>
         <v/>
       </c>
       <c r="AA28" s="12">
-        <f>N28</f>
+        <f>Z28</f>
         <v/>
       </c>
       <c r="AB28" s="12">
-        <f>N28</f>
+        <f>AA28</f>
         <v/>
       </c>
       <c r="AC28" s="12">
-        <f>N28</f>
+        <f>AB28</f>
         <v/>
       </c>
       <c r="AD28" s="12">
-        <f>N28</f>
+        <f>AC28</f>
         <v/>
       </c>
       <c r="AE28" s="12">
-        <f>N28</f>
+        <f>AD28</f>
         <v/>
       </c>
       <c r="AF28" s="12">
-        <f>N28</f>
+        <f>AE28</f>
         <v/>
       </c>
       <c r="AG28" s="12">
-        <f>N28</f>
+        <f>AF28</f>
         <v/>
       </c>
       <c r="AH28" s="12">
-        <f>N28</f>
+        <f>AG28</f>
         <v/>
       </c>
     </row>
@@ -13953,79 +13953,79 @@
         <v/>
       </c>
       <c r="P29" s="12">
-        <f>N29</f>
+        <f>O29</f>
         <v/>
       </c>
       <c r="Q29" s="12">
-        <f>N29</f>
+        <f>P29</f>
         <v/>
       </c>
       <c r="R29" s="12">
-        <f>N29</f>
+        <f>Q29</f>
         <v/>
       </c>
       <c r="S29" s="12">
-        <f>N29</f>
+        <f>R29</f>
         <v/>
       </c>
       <c r="T29" s="12">
-        <f>N29</f>
+        <f>S29</f>
         <v/>
       </c>
       <c r="U29" s="12">
-        <f>N29</f>
+        <f>T29</f>
         <v/>
       </c>
       <c r="V29" s="12">
-        <f>N29</f>
+        <f>U29</f>
         <v/>
       </c>
       <c r="W29" s="12">
-        <f>N29</f>
+        <f>V29</f>
         <v/>
       </c>
       <c r="X29" s="12">
-        <f>N29</f>
+        <f>W29</f>
         <v/>
       </c>
       <c r="Y29" s="12">
-        <f>N29</f>
+        <f>X29</f>
         <v/>
       </c>
       <c r="Z29" s="12">
-        <f>N29</f>
+        <f>Y29</f>
         <v/>
       </c>
       <c r="AA29" s="12">
-        <f>N29</f>
+        <f>Z29</f>
         <v/>
       </c>
       <c r="AB29" s="12">
-        <f>N29</f>
+        <f>AA29</f>
         <v/>
       </c>
       <c r="AC29" s="12">
-        <f>N29</f>
+        <f>AB29</f>
         <v/>
       </c>
       <c r="AD29" s="12">
-        <f>N29</f>
+        <f>AC29</f>
         <v/>
       </c>
       <c r="AE29" s="12">
-        <f>N29</f>
+        <f>AD29</f>
         <v/>
       </c>
       <c r="AF29" s="12">
-        <f>N29</f>
+        <f>AE29</f>
         <v/>
       </c>
       <c r="AG29" s="12">
-        <f>N29</f>
+        <f>AF29</f>
         <v/>
       </c>
       <c r="AH29" s="12">
-        <f>N29</f>
+        <f>AG29</f>
         <v/>
       </c>
     </row>
@@ -14092,79 +14092,79 @@
         <v/>
       </c>
       <c r="P30" s="13">
-        <f>N30</f>
+        <f>O30</f>
         <v/>
       </c>
       <c r="Q30" s="13">
-        <f>N30</f>
+        <f>P30</f>
         <v/>
       </c>
       <c r="R30" s="13">
-        <f>N30</f>
+        <f>Q30</f>
         <v/>
       </c>
       <c r="S30" s="13">
-        <f>N30</f>
+        <f>R30</f>
         <v/>
       </c>
       <c r="T30" s="13">
-        <f>N30</f>
+        <f>S30</f>
         <v/>
       </c>
       <c r="U30" s="13">
-        <f>N30</f>
+        <f>T30</f>
         <v/>
       </c>
       <c r="V30" s="13">
-        <f>N30</f>
+        <f>U30</f>
         <v/>
       </c>
       <c r="W30" s="13">
-        <f>N30</f>
+        <f>V30</f>
         <v/>
       </c>
       <c r="X30" s="13">
-        <f>N30</f>
+        <f>W30</f>
         <v/>
       </c>
       <c r="Y30" s="13">
-        <f>N30</f>
+        <f>X30</f>
         <v/>
       </c>
       <c r="Z30" s="13">
-        <f>N30</f>
+        <f>Y30</f>
         <v/>
       </c>
       <c r="AA30" s="13">
-        <f>N30</f>
+        <f>Z30</f>
         <v/>
       </c>
       <c r="AB30" s="13">
-        <f>N30</f>
+        <f>AA30</f>
         <v/>
       </c>
       <c r="AC30" s="13">
-        <f>N30</f>
+        <f>AB30</f>
         <v/>
       </c>
       <c r="AD30" s="13">
-        <f>N30</f>
+        <f>AC30</f>
         <v/>
       </c>
       <c r="AE30" s="13">
-        <f>N30</f>
+        <f>AD30</f>
         <v/>
       </c>
       <c r="AF30" s="13">
-        <f>N30</f>
+        <f>AE30</f>
         <v/>
       </c>
       <c r="AG30" s="13">
-        <f>N30</f>
+        <f>AF30</f>
         <v/>
       </c>
       <c r="AH30" s="13">
-        <f>N30</f>
+        <f>AG30</f>
         <v/>
       </c>
     </row>
@@ -14231,79 +14231,79 @@
         <v/>
       </c>
       <c r="P31" s="13">
-        <f>N31</f>
+        <f>O31</f>
         <v/>
       </c>
       <c r="Q31" s="13">
-        <f>N31</f>
+        <f>P31</f>
         <v/>
       </c>
       <c r="R31" s="13">
-        <f>N31</f>
+        <f>Q31</f>
         <v/>
       </c>
       <c r="S31" s="13">
-        <f>N31</f>
+        <f>R31</f>
         <v/>
       </c>
       <c r="T31" s="13">
-        <f>N31</f>
+        <f>S31</f>
         <v/>
       </c>
       <c r="U31" s="13">
-        <f>N31</f>
+        <f>T31</f>
         <v/>
       </c>
       <c r="V31" s="13">
-        <f>N31</f>
+        <f>U31</f>
         <v/>
       </c>
       <c r="W31" s="13">
-        <f>N31</f>
+        <f>V31</f>
         <v/>
       </c>
       <c r="X31" s="13">
-        <f>N31</f>
+        <f>W31</f>
         <v/>
       </c>
       <c r="Y31" s="13">
-        <f>N31</f>
+        <f>X31</f>
         <v/>
       </c>
       <c r="Z31" s="13">
-        <f>N31</f>
+        <f>Y31</f>
         <v/>
       </c>
       <c r="AA31" s="13">
-        <f>N31</f>
+        <f>Z31</f>
         <v/>
       </c>
       <c r="AB31" s="13">
-        <f>N31</f>
+        <f>AA31</f>
         <v/>
       </c>
       <c r="AC31" s="13">
-        <f>N31</f>
+        <f>AB31</f>
         <v/>
       </c>
       <c r="AD31" s="13">
-        <f>N31</f>
+        <f>AC31</f>
         <v/>
       </c>
       <c r="AE31" s="13">
-        <f>N31</f>
+        <f>AD31</f>
         <v/>
       </c>
       <c r="AF31" s="13">
-        <f>N31</f>
+        <f>AE31</f>
         <v/>
       </c>
       <c r="AG31" s="13">
-        <f>N31</f>
+        <f>AF31</f>
         <v/>
       </c>
       <c r="AH31" s="13">
-        <f>N31</f>
+        <f>AG31</f>
         <v/>
       </c>
     </row>
@@ -14370,79 +14370,79 @@
         <v/>
       </c>
       <c r="P32" s="12">
-        <f>N32</f>
+        <f>O32</f>
         <v/>
       </c>
       <c r="Q32" s="12">
-        <f>N32</f>
+        <f>P32</f>
         <v/>
       </c>
       <c r="R32" s="12">
-        <f>N32</f>
+        <f>Q32</f>
         <v/>
       </c>
       <c r="S32" s="12">
-        <f>N32</f>
+        <f>R32</f>
         <v/>
       </c>
       <c r="T32" s="12">
-        <f>N32</f>
+        <f>S32</f>
         <v/>
       </c>
       <c r="U32" s="12">
-        <f>N32</f>
+        <f>T32</f>
         <v/>
       </c>
       <c r="V32" s="12">
-        <f>N32</f>
+        <f>U32</f>
         <v/>
       </c>
       <c r="W32" s="12">
-        <f>N32</f>
+        <f>V32</f>
         <v/>
       </c>
       <c r="X32" s="12">
-        <f>N32</f>
+        <f>W32</f>
         <v/>
       </c>
       <c r="Y32" s="12">
-        <f>N32</f>
+        <f>X32</f>
         <v/>
       </c>
       <c r="Z32" s="12">
-        <f>N32</f>
+        <f>Y32</f>
         <v/>
       </c>
       <c r="AA32" s="12">
-        <f>N32</f>
+        <f>Z32</f>
         <v/>
       </c>
       <c r="AB32" s="12">
-        <f>N32</f>
+        <f>AA32</f>
         <v/>
       </c>
       <c r="AC32" s="12">
-        <f>N32</f>
+        <f>AB32</f>
         <v/>
       </c>
       <c r="AD32" s="12">
-        <f>N32</f>
+        <f>AC32</f>
         <v/>
       </c>
       <c r="AE32" s="12">
-        <f>N32</f>
+        <f>AD32</f>
         <v/>
       </c>
       <c r="AF32" s="12">
-        <f>N32</f>
+        <f>AE32</f>
         <v/>
       </c>
       <c r="AG32" s="12">
-        <f>N32</f>
+        <f>AF32</f>
         <v/>
       </c>
       <c r="AH32" s="12">
-        <f>N32</f>
+        <f>AG32</f>
         <v/>
       </c>
     </row>
@@ -14509,79 +14509,79 @@
         <v/>
       </c>
       <c r="P33" s="12">
-        <f>N33</f>
+        <f>O33</f>
         <v/>
       </c>
       <c r="Q33" s="12">
-        <f>N33</f>
+        <f>P33</f>
         <v/>
       </c>
       <c r="R33" s="12">
-        <f>N33</f>
+        <f>Q33</f>
         <v/>
       </c>
       <c r="S33" s="12">
-        <f>N33</f>
+        <f>R33</f>
         <v/>
       </c>
       <c r="T33" s="12">
-        <f>N33</f>
+        <f>S33</f>
         <v/>
       </c>
       <c r="U33" s="12">
-        <f>N33</f>
+        <f>T33</f>
         <v/>
       </c>
       <c r="V33" s="12">
-        <f>N33</f>
+        <f>U33</f>
         <v/>
       </c>
       <c r="W33" s="12">
-        <f>N33</f>
+        <f>V33</f>
         <v/>
       </c>
       <c r="X33" s="12">
-        <f>N33</f>
+        <f>W33</f>
         <v/>
       </c>
       <c r="Y33" s="12">
-        <f>N33</f>
+        <f>X33</f>
         <v/>
       </c>
       <c r="Z33" s="12">
-        <f>N33</f>
+        <f>Y33</f>
         <v/>
       </c>
       <c r="AA33" s="12">
-        <f>N33</f>
+        <f>Z33</f>
         <v/>
       </c>
       <c r="AB33" s="12">
-        <f>N33</f>
+        <f>AA33</f>
         <v/>
       </c>
       <c r="AC33" s="12">
-        <f>N33</f>
+        <f>AB33</f>
         <v/>
       </c>
       <c r="AD33" s="12">
-        <f>N33</f>
+        <f>AC33</f>
         <v/>
       </c>
       <c r="AE33" s="12">
-        <f>N33</f>
+        <f>AD33</f>
         <v/>
       </c>
       <c r="AF33" s="12">
-        <f>N33</f>
+        <f>AE33</f>
         <v/>
       </c>
       <c r="AG33" s="12">
-        <f>N33</f>
+        <f>AF33</f>
         <v/>
       </c>
       <c r="AH33" s="12">
-        <f>N33</f>
+        <f>AG33</f>
         <v/>
       </c>
     </row>
@@ -14648,79 +14648,79 @@
         <v/>
       </c>
       <c r="P34" s="13">
-        <f>N34</f>
+        <f>O34</f>
         <v/>
       </c>
       <c r="Q34" s="13">
-        <f>N34</f>
+        <f>P34</f>
         <v/>
       </c>
       <c r="R34" s="13">
-        <f>N34</f>
+        <f>Q34</f>
         <v/>
       </c>
       <c r="S34" s="13">
-        <f>N34</f>
+        <f>R34</f>
         <v/>
       </c>
       <c r="T34" s="13">
-        <f>N34</f>
+        <f>S34</f>
         <v/>
       </c>
       <c r="U34" s="13">
-        <f>N34</f>
+        <f>T34</f>
         <v/>
       </c>
       <c r="V34" s="13">
-        <f>N34</f>
+        <f>U34</f>
         <v/>
       </c>
       <c r="W34" s="13">
-        <f>N34</f>
+        <f>V34</f>
         <v/>
       </c>
       <c r="X34" s="13">
-        <f>N34</f>
+        <f>W34</f>
         <v/>
       </c>
       <c r="Y34" s="13">
-        <f>N34</f>
+        <f>X34</f>
         <v/>
       </c>
       <c r="Z34" s="13">
-        <f>N34</f>
+        <f>Y34</f>
         <v/>
       </c>
       <c r="AA34" s="13">
-        <f>N34</f>
+        <f>Z34</f>
         <v/>
       </c>
       <c r="AB34" s="13">
-        <f>N34</f>
+        <f>AA34</f>
         <v/>
       </c>
       <c r="AC34" s="13">
-        <f>N34</f>
+        <f>AB34</f>
         <v/>
       </c>
       <c r="AD34" s="13">
-        <f>N34</f>
+        <f>AC34</f>
         <v/>
       </c>
       <c r="AE34" s="13">
-        <f>N34</f>
+        <f>AD34</f>
         <v/>
       </c>
       <c r="AF34" s="13">
-        <f>N34</f>
+        <f>AE34</f>
         <v/>
       </c>
       <c r="AG34" s="13">
-        <f>N34</f>
+        <f>AF34</f>
         <v/>
       </c>
       <c r="AH34" s="13">
-        <f>N34</f>
+        <f>AG34</f>
         <v/>
       </c>
     </row>
@@ -14787,79 +14787,79 @@
         <v/>
       </c>
       <c r="P35" s="13">
-        <f>N35</f>
+        <f>O35</f>
         <v/>
       </c>
       <c r="Q35" s="13">
-        <f>N35</f>
+        <f>P35</f>
         <v/>
       </c>
       <c r="R35" s="13">
-        <f>N35</f>
+        <f>Q35</f>
         <v/>
       </c>
       <c r="S35" s="13">
-        <f>N35</f>
+        <f>R35</f>
         <v/>
       </c>
       <c r="T35" s="13">
-        <f>N35</f>
+        <f>S35</f>
         <v/>
       </c>
       <c r="U35" s="13">
-        <f>N35</f>
+        <f>T35</f>
         <v/>
       </c>
       <c r="V35" s="13">
-        <f>N35</f>
+        <f>U35</f>
         <v/>
       </c>
       <c r="W35" s="13">
-        <f>N35</f>
+        <f>V35</f>
         <v/>
       </c>
       <c r="X35" s="13">
-        <f>N35</f>
+        <f>W35</f>
         <v/>
       </c>
       <c r="Y35" s="13">
-        <f>N35</f>
+        <f>X35</f>
         <v/>
       </c>
       <c r="Z35" s="13">
-        <f>N35</f>
+        <f>Y35</f>
         <v/>
       </c>
       <c r="AA35" s="13">
-        <f>N35</f>
+        <f>Z35</f>
         <v/>
       </c>
       <c r="AB35" s="13">
-        <f>N35</f>
+        <f>AA35</f>
         <v/>
       </c>
       <c r="AC35" s="13">
-        <f>N35</f>
+        <f>AB35</f>
         <v/>
       </c>
       <c r="AD35" s="13">
-        <f>N35</f>
+        <f>AC35</f>
         <v/>
       </c>
       <c r="AE35" s="13">
-        <f>N35</f>
+        <f>AD35</f>
         <v/>
       </c>
       <c r="AF35" s="13">
-        <f>N35</f>
+        <f>AE35</f>
         <v/>
       </c>
       <c r="AG35" s="13">
-        <f>N35</f>
+        <f>AF35</f>
         <v/>
       </c>
       <c r="AH35" s="13">
-        <f>N35</f>
+        <f>AG35</f>
         <v/>
       </c>
     </row>
@@ -14926,79 +14926,79 @@
         <v/>
       </c>
       <c r="P36" s="13">
-        <f>N36</f>
+        <f>O36</f>
         <v/>
       </c>
       <c r="Q36" s="13">
-        <f>N36</f>
+        <f>P36</f>
         <v/>
       </c>
       <c r="R36" s="13">
-        <f>N36</f>
+        <f>Q36</f>
         <v/>
       </c>
       <c r="S36" s="13">
-        <f>N36</f>
+        <f>R36</f>
         <v/>
       </c>
       <c r="T36" s="13">
-        <f>N36</f>
+        <f>S36</f>
         <v/>
       </c>
       <c r="U36" s="13">
-        <f>N36</f>
+        <f>T36</f>
         <v/>
       </c>
       <c r="V36" s="13">
-        <f>N36</f>
+        <f>U36</f>
         <v/>
       </c>
       <c r="W36" s="13">
-        <f>N36</f>
+        <f>V36</f>
         <v/>
       </c>
       <c r="X36" s="13">
-        <f>N36</f>
+        <f>W36</f>
         <v/>
       </c>
       <c r="Y36" s="13">
-        <f>N36</f>
+        <f>X36</f>
         <v/>
       </c>
       <c r="Z36" s="13">
-        <f>N36</f>
+        <f>Y36</f>
         <v/>
       </c>
       <c r="AA36" s="13">
-        <f>N36</f>
+        <f>Z36</f>
         <v/>
       </c>
       <c r="AB36" s="13">
-        <f>N36</f>
+        <f>AA36</f>
         <v/>
       </c>
       <c r="AC36" s="13">
-        <f>N36</f>
+        <f>AB36</f>
         <v/>
       </c>
       <c r="AD36" s="13">
-        <f>N36</f>
+        <f>AC36</f>
         <v/>
       </c>
       <c r="AE36" s="13">
-        <f>N36</f>
+        <f>AD36</f>
         <v/>
       </c>
       <c r="AF36" s="13">
-        <f>N36</f>
+        <f>AE36</f>
         <v/>
       </c>
       <c r="AG36" s="13">
-        <f>N36</f>
+        <f>AF36</f>
         <v/>
       </c>
       <c r="AH36" s="13">
-        <f>N36</f>
+        <f>AG36</f>
         <v/>
       </c>
     </row>
@@ -16278,79 +16278,79 @@
         <v/>
       </c>
       <c r="S6" s="12">
-        <f>Q6</f>
+        <f>R6</f>
         <v/>
       </c>
       <c r="T6" s="12">
-        <f>Q6</f>
+        <f>S6</f>
         <v/>
       </c>
       <c r="U6" s="12">
-        <f>Q6</f>
+        <f>T6</f>
         <v/>
       </c>
       <c r="V6" s="12">
-        <f>Q6</f>
+        <f>U6</f>
         <v/>
       </c>
       <c r="W6" s="12">
-        <f>Q6</f>
+        <f>V6</f>
         <v/>
       </c>
       <c r="X6" s="12">
-        <f>Q6</f>
+        <f>W6</f>
         <v/>
       </c>
       <c r="Y6" s="12">
-        <f>Q6</f>
+        <f>X6</f>
         <v/>
       </c>
       <c r="Z6" s="12">
-        <f>Q6</f>
+        <f>Y6</f>
         <v/>
       </c>
       <c r="AA6" s="12">
-        <f>Q6</f>
+        <f>Z6</f>
         <v/>
       </c>
       <c r="AB6" s="12">
-        <f>Q6</f>
+        <f>AA6</f>
         <v/>
       </c>
       <c r="AC6" s="12">
-        <f>Q6</f>
+        <f>AB6</f>
         <v/>
       </c>
       <c r="AD6" s="12">
-        <f>Q6</f>
+        <f>AC6</f>
         <v/>
       </c>
       <c r="AE6" s="12">
-        <f>Q6</f>
+        <f>AD6</f>
         <v/>
       </c>
       <c r="AF6" s="12">
-        <f>Q6</f>
+        <f>AE6</f>
         <v/>
       </c>
       <c r="AG6" s="12">
-        <f>Q6</f>
+        <f>AF6</f>
         <v/>
       </c>
       <c r="AH6" s="12">
-        <f>Q6</f>
+        <f>AG6</f>
         <v/>
       </c>
       <c r="AI6" s="12">
-        <f>Q6</f>
+        <f>AH6</f>
         <v/>
       </c>
       <c r="AJ6" s="12">
-        <f>Q6</f>
+        <f>AI6</f>
         <v/>
       </c>
       <c r="AK6" s="12">
-        <f>Q6</f>
+        <f>AJ6</f>
         <v/>
       </c>
     </row>
@@ -16953,79 +16953,79 @@
         <v/>
       </c>
       <c r="S11" s="12">
-        <f>Q11</f>
+        <f>R11</f>
         <v/>
       </c>
       <c r="T11" s="12">
-        <f>Q11</f>
+        <f>S11</f>
         <v/>
       </c>
       <c r="U11" s="12">
-        <f>Q11</f>
+        <f>T11</f>
         <v/>
       </c>
       <c r="V11" s="12">
-        <f>Q11</f>
+        <f>U11</f>
         <v/>
       </c>
       <c r="W11" s="12">
-        <f>Q11</f>
+        <f>V11</f>
         <v/>
       </c>
       <c r="X11" s="12">
-        <f>Q11</f>
+        <f>W11</f>
         <v/>
       </c>
       <c r="Y11" s="12">
-        <f>Q11</f>
+        <f>X11</f>
         <v/>
       </c>
       <c r="Z11" s="12">
-        <f>Q11</f>
+        <f>Y11</f>
         <v/>
       </c>
       <c r="AA11" s="12">
-        <f>Q11</f>
+        <f>Z11</f>
         <v/>
       </c>
       <c r="AB11" s="12">
-        <f>Q11</f>
+        <f>AA11</f>
         <v/>
       </c>
       <c r="AC11" s="12">
-        <f>Q11</f>
+        <f>AB11</f>
         <v/>
       </c>
       <c r="AD11" s="12">
-        <f>Q11</f>
+        <f>AC11</f>
         <v/>
       </c>
       <c r="AE11" s="12">
-        <f>Q11</f>
+        <f>AD11</f>
         <v/>
       </c>
       <c r="AF11" s="12">
-        <f>Q11</f>
+        <f>AE11</f>
         <v/>
       </c>
       <c r="AG11" s="12">
-        <f>Q11</f>
+        <f>AF11</f>
         <v/>
       </c>
       <c r="AH11" s="12">
-        <f>Q11</f>
+        <f>AG11</f>
         <v/>
       </c>
       <c r="AI11" s="12">
-        <f>Q11</f>
+        <f>AH11</f>
         <v/>
       </c>
       <c r="AJ11" s="12">
-        <f>Q11</f>
+        <f>AI11</f>
         <v/>
       </c>
       <c r="AK11" s="12">
-        <f>Q11</f>
+        <f>AJ11</f>
         <v/>
       </c>
     </row>
@@ -17104,79 +17104,79 @@
         <v/>
       </c>
       <c r="S12" s="13">
-        <f>Q12</f>
+        <f>R12</f>
         <v/>
       </c>
       <c r="T12" s="13">
-        <f>Q12</f>
+        <f>S12</f>
         <v/>
       </c>
       <c r="U12" s="13">
-        <f>Q12</f>
+        <f>T12</f>
         <v/>
       </c>
       <c r="V12" s="13">
-        <f>Q12</f>
+        <f>U12</f>
         <v/>
       </c>
       <c r="W12" s="13">
-        <f>Q12</f>
+        <f>V12</f>
         <v/>
       </c>
       <c r="X12" s="13">
-        <f>Q12</f>
+        <f>W12</f>
         <v/>
       </c>
       <c r="Y12" s="13">
-        <f>Q12</f>
+        <f>X12</f>
         <v/>
       </c>
       <c r="Z12" s="13">
-        <f>Q12</f>
+        <f>Y12</f>
         <v/>
       </c>
       <c r="AA12" s="13">
-        <f>Q12</f>
+        <f>Z12</f>
         <v/>
       </c>
       <c r="AB12" s="13">
-        <f>Q12</f>
+        <f>AA12</f>
         <v/>
       </c>
       <c r="AC12" s="13">
-        <f>Q12</f>
+        <f>AB12</f>
         <v/>
       </c>
       <c r="AD12" s="13">
-        <f>Q12</f>
+        <f>AC12</f>
         <v/>
       </c>
       <c r="AE12" s="13">
-        <f>Q12</f>
+        <f>AD12</f>
         <v/>
       </c>
       <c r="AF12" s="13">
-        <f>Q12</f>
+        <f>AE12</f>
         <v/>
       </c>
       <c r="AG12" s="13">
-        <f>Q12</f>
+        <f>AF12</f>
         <v/>
       </c>
       <c r="AH12" s="13">
-        <f>Q12</f>
+        <f>AG12</f>
         <v/>
       </c>
       <c r="AI12" s="13">
-        <f>Q12</f>
+        <f>AH12</f>
         <v/>
       </c>
       <c r="AJ12" s="13">
-        <f>Q12</f>
+        <f>AI12</f>
         <v/>
       </c>
       <c r="AK12" s="13">
-        <f>Q12</f>
+        <f>AJ12</f>
         <v/>
       </c>
     </row>
@@ -20055,79 +20055,79 @@
         <v/>
       </c>
       <c r="S33" s="12">
-        <f>Q33</f>
+        <f>R33</f>
         <v/>
       </c>
       <c r="T33" s="12">
-        <f>Q33</f>
+        <f>S33</f>
         <v/>
       </c>
       <c r="U33" s="12">
-        <f>Q33</f>
+        <f>T33</f>
         <v/>
       </c>
       <c r="V33" s="12">
-        <f>Q33</f>
+        <f>U33</f>
         <v/>
       </c>
       <c r="W33" s="12">
-        <f>Q33</f>
+        <f>V33</f>
         <v/>
       </c>
       <c r="X33" s="12">
-        <f>Q33</f>
+        <f>W33</f>
         <v/>
       </c>
       <c r="Y33" s="12">
-        <f>Q33</f>
+        <f>X33</f>
         <v/>
       </c>
       <c r="Z33" s="12">
-        <f>Q33</f>
+        <f>Y33</f>
         <v/>
       </c>
       <c r="AA33" s="12">
-        <f>Q33</f>
+        <f>Z33</f>
         <v/>
       </c>
       <c r="AB33" s="12">
-        <f>Q33</f>
+        <f>AA33</f>
         <v/>
       </c>
       <c r="AC33" s="12">
-        <f>Q33</f>
+        <f>AB33</f>
         <v/>
       </c>
       <c r="AD33" s="12">
-        <f>Q33</f>
+        <f>AC33</f>
         <v/>
       </c>
       <c r="AE33" s="12">
-        <f>Q33</f>
+        <f>AD33</f>
         <v/>
       </c>
       <c r="AF33" s="12">
-        <f>Q33</f>
+        <f>AE33</f>
         <v/>
       </c>
       <c r="AG33" s="12">
-        <f>Q33</f>
+        <f>AF33</f>
         <v/>
       </c>
       <c r="AH33" s="12">
-        <f>Q33</f>
+        <f>AG33</f>
         <v/>
       </c>
       <c r="AI33" s="12">
-        <f>Q33</f>
+        <f>AH33</f>
         <v/>
       </c>
       <c r="AJ33" s="12">
-        <f>Q33</f>
+        <f>AI33</f>
         <v/>
       </c>
       <c r="AK33" s="12">
-        <f>Q33</f>
+        <f>AJ33</f>
         <v/>
       </c>
     </row>
@@ -21254,79 +21254,79 @@
         <v/>
       </c>
       <c r="S42" s="13">
-        <f>Q42</f>
+        <f>R42</f>
         <v/>
       </c>
       <c r="T42" s="13">
-        <f>Q42</f>
+        <f>S42</f>
         <v/>
       </c>
       <c r="U42" s="13">
-        <f>Q42</f>
+        <f>T42</f>
         <v/>
       </c>
       <c r="V42" s="13">
-        <f>Q42</f>
+        <f>U42</f>
         <v/>
       </c>
       <c r="W42" s="13">
-        <f>Q42</f>
+        <f>V42</f>
         <v/>
       </c>
       <c r="X42" s="13">
-        <f>Q42</f>
+        <f>W42</f>
         <v/>
       </c>
       <c r="Y42" s="13">
-        <f>Q42</f>
+        <f>X42</f>
         <v/>
       </c>
       <c r="Z42" s="13">
-        <f>Q42</f>
+        <f>Y42</f>
         <v/>
       </c>
       <c r="AA42" s="13">
-        <f>Q42</f>
+        <f>Z42</f>
         <v/>
       </c>
       <c r="AB42" s="13">
-        <f>Q42</f>
+        <f>AA42</f>
         <v/>
       </c>
       <c r="AC42" s="13">
-        <f>Q42</f>
+        <f>AB42</f>
         <v/>
       </c>
       <c r="AD42" s="13">
-        <f>Q42</f>
+        <f>AC42</f>
         <v/>
       </c>
       <c r="AE42" s="13">
-        <f>Q42</f>
+        <f>AD42</f>
         <v/>
       </c>
       <c r="AF42" s="13">
-        <f>Q42</f>
+        <f>AE42</f>
         <v/>
       </c>
       <c r="AG42" s="13">
-        <f>Q42</f>
+        <f>AF42</f>
         <v/>
       </c>
       <c r="AH42" s="13">
-        <f>Q42</f>
+        <f>AG42</f>
         <v/>
       </c>
       <c r="AI42" s="13">
-        <f>Q42</f>
+        <f>AH42</f>
         <v/>
       </c>
       <c r="AJ42" s="13">
-        <f>Q42</f>
+        <f>AI42</f>
         <v/>
       </c>
       <c r="AK42" s="13">
-        <f>Q42</f>
+        <f>AJ42</f>
         <v/>
       </c>
     </row>
@@ -22060,79 +22060,79 @@
         <v/>
       </c>
       <c r="S48" s="13">
-        <f>Q48</f>
+        <f>R48</f>
         <v/>
       </c>
       <c r="T48" s="13">
-        <f>Q48</f>
+        <f>S48</f>
         <v/>
       </c>
       <c r="U48" s="13">
-        <f>Q48</f>
+        <f>T48</f>
         <v/>
       </c>
       <c r="V48" s="13">
-        <f>Q48</f>
+        <f>U48</f>
         <v/>
       </c>
       <c r="W48" s="13">
-        <f>Q48</f>
+        <f>V48</f>
         <v/>
       </c>
       <c r="X48" s="13">
-        <f>Q48</f>
+        <f>W48</f>
         <v/>
       </c>
       <c r="Y48" s="13">
-        <f>Q48</f>
+        <f>X48</f>
         <v/>
       </c>
       <c r="Z48" s="13">
-        <f>Q48</f>
+        <f>Y48</f>
         <v/>
       </c>
       <c r="AA48" s="13">
-        <f>Q48</f>
+        <f>Z48</f>
         <v/>
       </c>
       <c r="AB48" s="13">
-        <f>Q48</f>
+        <f>AA48</f>
         <v/>
       </c>
       <c r="AC48" s="13">
-        <f>Q48</f>
+        <f>AB48</f>
         <v/>
       </c>
       <c r="AD48" s="13">
-        <f>Q48</f>
+        <f>AC48</f>
         <v/>
       </c>
       <c r="AE48" s="13">
-        <f>Q48</f>
+        <f>AD48</f>
         <v/>
       </c>
       <c r="AF48" s="13">
-        <f>Q48</f>
+        <f>AE48</f>
         <v/>
       </c>
       <c r="AG48" s="13">
-        <f>Q48</f>
+        <f>AF48</f>
         <v/>
       </c>
       <c r="AH48" s="13">
-        <f>Q48</f>
+        <f>AG48</f>
         <v/>
       </c>
       <c r="AI48" s="13">
-        <f>Q48</f>
+        <f>AH48</f>
         <v/>
       </c>
       <c r="AJ48" s="13">
-        <f>Q48</f>
+        <f>AI48</f>
         <v/>
       </c>
       <c r="AK48" s="13">
-        <f>Q48</f>
+        <f>AJ48</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-04-28 15:38:13
</commit_message>
<xml_diff>
--- a/Knowledge/Model Outputs/CELH/CELH_model.xlsx
+++ b/Knowledge/Model Outputs/CELH/CELH_model.xlsx
@@ -8355,7 +8355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL10"/>
+  <dimension ref="A1:AL9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -9776,157 +9776,6 @@
       </c>
       <c r="AL9" s="12">
         <f>AK9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Net Income (Loss) Attributable to Common Shareholders — % of Revenue</t>
-        </is>
-      </c>
-      <c r="C10" s="11">
-        <f>IFERROR('QTR P&amp;L'!B16/'QTR P&amp;L'!B2,"")</f>
-        <v/>
-      </c>
-      <c r="D10" s="11">
-        <f>IFERROR('QTR P&amp;L'!C16/'QTR P&amp;L'!C2,"")</f>
-        <v/>
-      </c>
-      <c r="E10" s="11">
-        <f>IFERROR('QTR P&amp;L'!D16/'QTR P&amp;L'!D2,"")</f>
-        <v/>
-      </c>
-      <c r="F10" s="11">
-        <f>IFERROR('QTR P&amp;L'!E16/'QTR P&amp;L'!E2,"")</f>
-        <v/>
-      </c>
-      <c r="G10" s="11">
-        <f>IFERROR('QTR P&amp;L'!F16/'QTR P&amp;L'!F2,"")</f>
-        <v/>
-      </c>
-      <c r="H10" s="11">
-        <f>IFERROR('QTR P&amp;L'!G16/'QTR P&amp;L'!G2,"")</f>
-        <v/>
-      </c>
-      <c r="I10" s="11">
-        <f>IFERROR('QTR P&amp;L'!H16/'QTR P&amp;L'!H2,"")</f>
-        <v/>
-      </c>
-      <c r="J10" s="11">
-        <f>IFERROR('QTR P&amp;L'!I16/'QTR P&amp;L'!I2,"")</f>
-        <v/>
-      </c>
-      <c r="K10" s="11">
-        <f>IFERROR('QTR P&amp;L'!J16/'QTR P&amp;L'!J2,"")</f>
-        <v/>
-      </c>
-      <c r="L10" s="11">
-        <f>IFERROR('QTR P&amp;L'!K16/'QTR P&amp;L'!K2,"")</f>
-        <v/>
-      </c>
-      <c r="M10" s="11">
-        <f>IFERROR('QTR P&amp;L'!L16/'QTR P&amp;L'!L2,"")</f>
-        <v/>
-      </c>
-      <c r="N10" s="11">
-        <f>IFERROR('QTR P&amp;L'!M16/'QTR P&amp;L'!M2,"")</f>
-        <v/>
-      </c>
-      <c r="O10" s="11">
-        <f>IFERROR('QTR P&amp;L'!N16/'QTR P&amp;L'!N2,"")</f>
-        <v/>
-      </c>
-      <c r="P10" s="11">
-        <f>IFERROR('QTR P&amp;L'!O16/'QTR P&amp;L'!O2,"")</f>
-        <v/>
-      </c>
-      <c r="Q10" s="11">
-        <f>IFERROR('QTR P&amp;L'!P16/'QTR P&amp;L'!P2,"")</f>
-        <v/>
-      </c>
-      <c r="R10" s="11">
-        <f>IFERROR('QTR P&amp;L'!Q16/'QTR P&amp;L'!Q2,"")</f>
-        <v/>
-      </c>
-      <c r="S10" s="12">
-        <f>R10</f>
-        <v/>
-      </c>
-      <c r="T10" s="12">
-        <f>S10</f>
-        <v/>
-      </c>
-      <c r="U10" s="12">
-        <f>T10</f>
-        <v/>
-      </c>
-      <c r="V10" s="12">
-        <f>U10</f>
-        <v/>
-      </c>
-      <c r="W10" s="12">
-        <f>V10</f>
-        <v/>
-      </c>
-      <c r="X10" s="12">
-        <f>W10</f>
-        <v/>
-      </c>
-      <c r="Y10" s="12">
-        <f>X10</f>
-        <v/>
-      </c>
-      <c r="Z10" s="12">
-        <f>Y10</f>
-        <v/>
-      </c>
-      <c r="AA10" s="12">
-        <f>Z10</f>
-        <v/>
-      </c>
-      <c r="AB10" s="12">
-        <f>AA10</f>
-        <v/>
-      </c>
-      <c r="AC10" s="12">
-        <f>AB10</f>
-        <v/>
-      </c>
-      <c r="AD10" s="12">
-        <f>AC10</f>
-        <v/>
-      </c>
-      <c r="AE10" s="12">
-        <f>AD10</f>
-        <v/>
-      </c>
-      <c r="AF10" s="12">
-        <f>AE10</f>
-        <v/>
-      </c>
-      <c r="AG10" s="12">
-        <f>AF10</f>
-        <v/>
-      </c>
-      <c r="AH10" s="12">
-        <f>AG10</f>
-        <v/>
-      </c>
-      <c r="AI10" s="12">
-        <f>AH10</f>
-        <v/>
-      </c>
-      <c r="AJ10" s="12">
-        <f>AI10</f>
-        <v/>
-      </c>
-      <c r="AK10" s="12">
-        <f>AJ10</f>
-        <v/>
-      </c>
-      <c r="AL10" s="12">
-        <f>AK10</f>
         <v/>
       </c>
     </row>
@@ -22862,42 +22711,50 @@
           <t>Net Income (Loss) Attributable to Common Shareholders</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
-        <v>3937</v>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>-198808</v>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>181991</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>107457</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>63837</v>
-      </c>
-      <c r="G16" s="9">
-        <f>'QTR P&amp;L'!R16+'QTR P&amp;L'!S16+'QTR P&amp;L'!T16+'QTR P&amp;L'!U16</f>
-        <v/>
-      </c>
-      <c r="H16" s="9">
-        <f>'QTR P&amp;L'!V16+'QTR P&amp;L'!W16+'QTR P&amp;L'!X16+'QTR P&amp;L'!Y16</f>
-        <v/>
-      </c>
-      <c r="I16" s="9">
-        <f>'QTR P&amp;L'!Z16+'QTR P&amp;L'!AA16+'QTR P&amp;L'!AB16+'QTR P&amp;L'!AC16</f>
-        <v/>
-      </c>
-      <c r="J16" s="9">
-        <f>'QTR P&amp;L'!AD16+'QTR P&amp;L'!AE16+'QTR P&amp;L'!AF16+'QTR P&amp;L'!AG16</f>
-        <v/>
-      </c>
-      <c r="K16" s="9">
-        <f>'QTR P&amp;L'!AH16+'QTR P&amp;L'!AI16+'QTR P&amp;L'!AJ16+'QTR P&amp;L'!AK16</f>
-        <v/>
-      </c>
-      <c r="L16" s="5" t="n"/>
+      <c r="B16" s="6">
+        <f>B13+B14+B15</f>
+        <v/>
+      </c>
+      <c r="C16" s="6">
+        <f>C13+C14+C15</f>
+        <v/>
+      </c>
+      <c r="D16" s="6">
+        <f>D13+D14+D15</f>
+        <v/>
+      </c>
+      <c r="E16" s="6">
+        <f>E13+E14+E15</f>
+        <v/>
+      </c>
+      <c r="F16" s="6">
+        <f>F13+F14+F15</f>
+        <v/>
+      </c>
+      <c r="G16" s="7">
+        <f>G13+G14+G15</f>
+        <v/>
+      </c>
+      <c r="H16" s="7">
+        <f>H13+H14+H15</f>
+        <v/>
+      </c>
+      <c r="I16" s="7">
+        <f>I13+I14+I15</f>
+        <v/>
+      </c>
+      <c r="J16" s="7">
+        <f>J13+J14+J15</f>
+        <v/>
+      </c>
+      <c r="K16" s="7">
+        <f>K13+K14+K15</f>
+        <v/>
+      </c>
+      <c r="L16" s="7">
+        <f>L13+L14+L15</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27711,41 +27568,53 @@
           <t>Net Income (Loss) Attributable to Common Shareholders</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
-        <v>6679</v>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>15838</v>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>-170655</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>34446</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>72372</v>
-      </c>
-      <c r="G16" s="4" t="n">
-        <v>142910</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>64846</v>
-      </c>
-      <c r="I16" s="4" t="n">
-        <v>131502</v>
-      </c>
-      <c r="J16" s="4" t="n">
-        <v>131005</v>
-      </c>
-      <c r="K16" s="4" t="n">
-        <v>34419</v>
-      </c>
-      <c r="L16" s="4" t="n">
-        <v>119939</v>
-      </c>
-      <c r="M16" s="4" t="n">
-        <v>54699</v>
+      <c r="B16" s="6">
+        <f>B13+B14+B15</f>
+        <v/>
+      </c>
+      <c r="C16" s="6">
+        <f>C13+C14+C15</f>
+        <v/>
+      </c>
+      <c r="D16" s="6">
+        <f>D13+D14+D15</f>
+        <v/>
+      </c>
+      <c r="E16" s="6">
+        <f>E13+E14+E15</f>
+        <v/>
+      </c>
+      <c r="F16" s="6">
+        <f>F13+F14+F15</f>
+        <v/>
+      </c>
+      <c r="G16" s="6">
+        <f>G13+G14+G15</f>
+        <v/>
+      </c>
+      <c r="H16" s="6">
+        <f>H13+H14+H15</f>
+        <v/>
+      </c>
+      <c r="I16" s="6">
+        <f>I13+I14+I15</f>
+        <v/>
+      </c>
+      <c r="J16" s="6">
+        <f>J13+J14+J15</f>
+        <v/>
+      </c>
+      <c r="K16" s="6">
+        <f>K13+K14+K15</f>
+        <v/>
+      </c>
+      <c r="L16" s="6">
+        <f>L13+L14+L15</f>
+        <v/>
+      </c>
+      <c r="M16" s="6">
+        <f>M13+M14+M15</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -34373,148 +34242,148 @@
           <t>Net Income (Loss) Attributable to Common Shareholders</t>
         </is>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="6">
         <f>'YTD P&amp;L'!B16</f>
         <v/>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="6">
         <f>'YTD P&amp;L'!C16-'YTD P&amp;L'!B16</f>
         <v/>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="6">
         <f>'YTD P&amp;L'!D16-'YTD P&amp;L'!C16</f>
         <v/>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="6">
         <f>'ANNL P&amp;L'!C16-'YTD P&amp;L'!D16</f>
         <v/>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="6">
         <f>'YTD P&amp;L'!E16</f>
         <v/>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="6">
         <f>'YTD P&amp;L'!F16-'YTD P&amp;L'!E16</f>
         <v/>
       </c>
-      <c r="H16" s="4">
+      <c r="H16" s="6">
         <f>'YTD P&amp;L'!G16-'YTD P&amp;L'!F16</f>
         <v/>
       </c>
-      <c r="I16" s="4">
+      <c r="I16" s="6">
         <f>'ANNL P&amp;L'!D16-'YTD P&amp;L'!G16</f>
         <v/>
       </c>
-      <c r="J16" s="4">
+      <c r="J16" s="6">
         <f>'YTD P&amp;L'!H16</f>
         <v/>
       </c>
-      <c r="K16" s="4">
+      <c r="K16" s="6">
         <f>'YTD P&amp;L'!I16-'YTD P&amp;L'!H16</f>
         <v/>
       </c>
-      <c r="L16" s="4">
+      <c r="L16" s="6">
         <f>'YTD P&amp;L'!J16-'YTD P&amp;L'!I16</f>
         <v/>
       </c>
-      <c r="M16" s="4">
+      <c r="M16" s="6">
         <f>'ANNL P&amp;L'!E16-'YTD P&amp;L'!J16</f>
         <v/>
       </c>
-      <c r="N16" s="4">
+      <c r="N16" s="6">
         <f>'YTD P&amp;L'!K16</f>
         <v/>
       </c>
-      <c r="O16" s="4">
+      <c r="O16" s="6">
         <f>'YTD P&amp;L'!L16-'YTD P&amp;L'!K16</f>
         <v/>
       </c>
-      <c r="P16" s="4">
+      <c r="P16" s="6">
         <f>'YTD P&amp;L'!M16-'YTD P&amp;L'!L16</f>
         <v/>
       </c>
-      <c r="Q16" s="4">
+      <c r="Q16" s="6">
         <f>'ANNL P&amp;L'!F16-'YTD P&amp;L'!M16</f>
         <v/>
       </c>
-      <c r="R16" s="9">
-        <f>'QTR P&amp;L'!R2*'IS DRIVERS'!S10</f>
-        <v/>
-      </c>
-      <c r="S16" s="9">
-        <f>'QTR P&amp;L'!S2*'IS DRIVERS'!T10</f>
-        <v/>
-      </c>
-      <c r="T16" s="9">
-        <f>'QTR P&amp;L'!T2*'IS DRIVERS'!U10</f>
-        <v/>
-      </c>
-      <c r="U16" s="9">
-        <f>'QTR P&amp;L'!U2*'IS DRIVERS'!V10</f>
-        <v/>
-      </c>
-      <c r="V16" s="9">
-        <f>'QTR P&amp;L'!V2*'IS DRIVERS'!W10</f>
-        <v/>
-      </c>
-      <c r="W16" s="9">
-        <f>'QTR P&amp;L'!W2*'IS DRIVERS'!X10</f>
-        <v/>
-      </c>
-      <c r="X16" s="9">
-        <f>'QTR P&amp;L'!X2*'IS DRIVERS'!Y10</f>
-        <v/>
-      </c>
-      <c r="Y16" s="9">
-        <f>'QTR P&amp;L'!Y2*'IS DRIVERS'!Z10</f>
-        <v/>
-      </c>
-      <c r="Z16" s="9">
-        <f>'QTR P&amp;L'!Z2*'IS DRIVERS'!AA10</f>
-        <v/>
-      </c>
-      <c r="AA16" s="9">
-        <f>'QTR P&amp;L'!AA2*'IS DRIVERS'!AB10</f>
-        <v/>
-      </c>
-      <c r="AB16" s="9">
-        <f>'QTR P&amp;L'!AB2*'IS DRIVERS'!AC10</f>
-        <v/>
-      </c>
-      <c r="AC16" s="9">
-        <f>'QTR P&amp;L'!AC2*'IS DRIVERS'!AD10</f>
-        <v/>
-      </c>
-      <c r="AD16" s="9">
-        <f>'QTR P&amp;L'!AD2*'IS DRIVERS'!AE10</f>
-        <v/>
-      </c>
-      <c r="AE16" s="9">
-        <f>'QTR P&amp;L'!AE2*'IS DRIVERS'!AF10</f>
-        <v/>
-      </c>
-      <c r="AF16" s="9">
-        <f>'QTR P&amp;L'!AF2*'IS DRIVERS'!AG10</f>
-        <v/>
-      </c>
-      <c r="AG16" s="9">
-        <f>'QTR P&amp;L'!AG2*'IS DRIVERS'!AH10</f>
-        <v/>
-      </c>
-      <c r="AH16" s="9">
-        <f>'QTR P&amp;L'!AH2*'IS DRIVERS'!AI10</f>
-        <v/>
-      </c>
-      <c r="AI16" s="9">
-        <f>'QTR P&amp;L'!AI2*'IS DRIVERS'!AJ10</f>
-        <v/>
-      </c>
-      <c r="AJ16" s="9">
-        <f>'QTR P&amp;L'!AJ2*'IS DRIVERS'!AK10</f>
-        <v/>
-      </c>
-      <c r="AK16" s="9">
-        <f>'QTR P&amp;L'!AK2*'IS DRIVERS'!AL10</f>
+      <c r="R16" s="7">
+        <f>R13+R14+R15</f>
+        <v/>
+      </c>
+      <c r="S16" s="7">
+        <f>S13+S14+S15</f>
+        <v/>
+      </c>
+      <c r="T16" s="7">
+        <f>T13+T14+T15</f>
+        <v/>
+      </c>
+      <c r="U16" s="7">
+        <f>U13+U14+U15</f>
+        <v/>
+      </c>
+      <c r="V16" s="7">
+        <f>V13+V14+V15</f>
+        <v/>
+      </c>
+      <c r="W16" s="7">
+        <f>W13+W14+W15</f>
+        <v/>
+      </c>
+      <c r="X16" s="7">
+        <f>X13+X14+X15</f>
+        <v/>
+      </c>
+      <c r="Y16" s="7">
+        <f>Y13+Y14+Y15</f>
+        <v/>
+      </c>
+      <c r="Z16" s="7">
+        <f>Z13+Z14+Z15</f>
+        <v/>
+      </c>
+      <c r="AA16" s="7">
+        <f>AA13+AA14+AA15</f>
+        <v/>
+      </c>
+      <c r="AB16" s="7">
+        <f>AB13+AB14+AB15</f>
+        <v/>
+      </c>
+      <c r="AC16" s="7">
+        <f>AC13+AC14+AC15</f>
+        <v/>
+      </c>
+      <c r="AD16" s="7">
+        <f>AD13+AD14+AD15</f>
+        <v/>
+      </c>
+      <c r="AE16" s="7">
+        <f>AE13+AE14+AE15</f>
+        <v/>
+      </c>
+      <c r="AF16" s="7">
+        <f>AF13+AF14+AF15</f>
+        <v/>
+      </c>
+      <c r="AG16" s="7">
+        <f>AG13+AG14+AG15</f>
+        <v/>
+      </c>
+      <c r="AH16" s="7">
+        <f>AH13+AH14+AH15</f>
+        <v/>
+      </c>
+      <c r="AI16" s="7">
+        <f>AI13+AI14+AI15</f>
+        <v/>
+      </c>
+      <c r="AJ16" s="7">
+        <f>AJ13+AJ14+AJ15</f>
+        <v/>
+      </c>
+      <c r="AK16" s="7">
+        <f>AK13+AK14+AK15</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-04-28 15:48:36
</commit_message>
<xml_diff>
--- a/Knowledge/Model Outputs/CELH/CELH_model.xlsx
+++ b/Knowledge/Model Outputs/CELH/CELH_model.xlsx
@@ -22675,13 +22675,13 @@
         <v>0</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>17348</v>
+        <v>-17348</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>10117</v>
+        <v>-10117</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>6554</v>
+        <v>-6554</v>
       </c>
       <c r="G15" s="9">
         <f>'QTR P&amp;L'!R15+'QTR P&amp;L'!S15+'QTR P&amp;L'!T15+'QTR P&amp;L'!U15</f>
@@ -27538,28 +27538,28 @@
         <v>0</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>6727</v>
+        <v>-6727</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>13263</v>
+        <v>-13263</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>6128</v>
+        <v>-6128</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>12417</v>
+        <v>-12417</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>12357</v>
+        <v>-12357</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>3219</v>
+        <v>-3219</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>10703</v>
+        <v>-10703</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>5272</v>
+        <v>-5272</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
vault backup: 2026-04-28 16:04:09
</commit_message>
<xml_diff>
--- a/Knowledge/Model Outputs/CELH/CELH_model.xlsx
+++ b/Knowledge/Model Outputs/CELH/CELH_model.xlsx
@@ -8355,7 +8355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL9"/>
+  <dimension ref="A1:AL11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -9776,6 +9776,244 @@
       </c>
       <c r="AL9" s="12">
         <f>AK9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Preferred Dividends</t>
+        </is>
+      </c>
+      <c r="S10" s="4">
+        <f>'QTR CF'!R44</f>
+        <v/>
+      </c>
+      <c r="T10" s="4">
+        <f>'QTR CF'!S44</f>
+        <v/>
+      </c>
+      <c r="U10" s="4">
+        <f>'QTR CF'!T44</f>
+        <v/>
+      </c>
+      <c r="V10" s="4">
+        <f>'QTR CF'!U44</f>
+        <v/>
+      </c>
+      <c r="W10" s="4">
+        <f>'QTR CF'!V44</f>
+        <v/>
+      </c>
+      <c r="X10" s="4">
+        <f>'QTR CF'!W44</f>
+        <v/>
+      </c>
+      <c r="Y10" s="4">
+        <f>'QTR CF'!X44</f>
+        <v/>
+      </c>
+      <c r="Z10" s="4">
+        <f>'QTR CF'!Y44</f>
+        <v/>
+      </c>
+      <c r="AA10" s="4">
+        <f>'QTR CF'!Z44</f>
+        <v/>
+      </c>
+      <c r="AB10" s="4">
+        <f>'QTR CF'!AA44</f>
+        <v/>
+      </c>
+      <c r="AC10" s="4">
+        <f>'QTR CF'!AB44</f>
+        <v/>
+      </c>
+      <c r="AD10" s="4">
+        <f>'QTR CF'!AC44</f>
+        <v/>
+      </c>
+      <c r="AE10" s="4">
+        <f>'QTR CF'!AD44</f>
+        <v/>
+      </c>
+      <c r="AF10" s="4">
+        <f>'QTR CF'!AE44</f>
+        <v/>
+      </c>
+      <c r="AG10" s="4">
+        <f>'QTR CF'!AF44</f>
+        <v/>
+      </c>
+      <c r="AH10" s="4">
+        <f>'QTR CF'!AG44</f>
+        <v/>
+      </c>
+      <c r="AI10" s="4">
+        <f>'QTR CF'!AH44</f>
+        <v/>
+      </c>
+      <c r="AJ10" s="4">
+        <f>'QTR CF'!AI44</f>
+        <v/>
+      </c>
+      <c r="AK10" s="4">
+        <f>'QTR CF'!AJ44</f>
+        <v/>
+      </c>
+      <c r="AL10" s="4">
+        <f>'QTR CF'!AK44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Income Allocated to Participating Preferred</t>
+        </is>
+      </c>
+      <c r="C11" s="4">
+        <f>'QTR P&amp;L'!B15</f>
+        <v/>
+      </c>
+      <c r="D11" s="4">
+        <f>'QTR P&amp;L'!C15</f>
+        <v/>
+      </c>
+      <c r="E11" s="4">
+        <f>'QTR P&amp;L'!D15</f>
+        <v/>
+      </c>
+      <c r="F11" s="4">
+        <f>'QTR P&amp;L'!E15</f>
+        <v/>
+      </c>
+      <c r="G11" s="4">
+        <f>'QTR P&amp;L'!F15</f>
+        <v/>
+      </c>
+      <c r="H11" s="4">
+        <f>'QTR P&amp;L'!G15</f>
+        <v/>
+      </c>
+      <c r="I11" s="4">
+        <f>'QTR P&amp;L'!H15</f>
+        <v/>
+      </c>
+      <c r="J11" s="4">
+        <f>'QTR P&amp;L'!I15</f>
+        <v/>
+      </c>
+      <c r="K11" s="4">
+        <f>'QTR P&amp;L'!J15</f>
+        <v/>
+      </c>
+      <c r="L11" s="4">
+        <f>'QTR P&amp;L'!K15</f>
+        <v/>
+      </c>
+      <c r="M11" s="4">
+        <f>'QTR P&amp;L'!L15</f>
+        <v/>
+      </c>
+      <c r="N11" s="4">
+        <f>'QTR P&amp;L'!M15</f>
+        <v/>
+      </c>
+      <c r="O11" s="4">
+        <f>'QTR P&amp;L'!N15</f>
+        <v/>
+      </c>
+      <c r="P11" s="4">
+        <f>'QTR P&amp;L'!O15</f>
+        <v/>
+      </c>
+      <c r="Q11" s="4">
+        <f>'QTR P&amp;L'!P15</f>
+        <v/>
+      </c>
+      <c r="R11" s="4">
+        <f>'QTR P&amp;L'!Q15</f>
+        <v/>
+      </c>
+      <c r="S11" s="13">
+        <f>R11</f>
+        <v/>
+      </c>
+      <c r="T11" s="13">
+        <f>S11</f>
+        <v/>
+      </c>
+      <c r="U11" s="13">
+        <f>T11</f>
+        <v/>
+      </c>
+      <c r="V11" s="13">
+        <f>U11</f>
+        <v/>
+      </c>
+      <c r="W11" s="13">
+        <f>V11</f>
+        <v/>
+      </c>
+      <c r="X11" s="13">
+        <f>W11</f>
+        <v/>
+      </c>
+      <c r="Y11" s="13">
+        <f>X11</f>
+        <v/>
+      </c>
+      <c r="Z11" s="13">
+        <f>Y11</f>
+        <v/>
+      </c>
+      <c r="AA11" s="13">
+        <f>Z11</f>
+        <v/>
+      </c>
+      <c r="AB11" s="13">
+        <f>AA11</f>
+        <v/>
+      </c>
+      <c r="AC11" s="13">
+        <f>AB11</f>
+        <v/>
+      </c>
+      <c r="AD11" s="13">
+        <f>AC11</f>
+        <v/>
+      </c>
+      <c r="AE11" s="13">
+        <f>AD11</f>
+        <v/>
+      </c>
+      <c r="AF11" s="13">
+        <f>AE11</f>
+        <v/>
+      </c>
+      <c r="AG11" s="13">
+        <f>AF11</f>
+        <v/>
+      </c>
+      <c r="AH11" s="13">
+        <f>AG11</f>
+        <v/>
+      </c>
+      <c r="AI11" s="13">
+        <f>AH11</f>
+        <v/>
+      </c>
+      <c r="AJ11" s="13">
+        <f>AI11</f>
+        <v/>
+      </c>
+      <c r="AK11" s="13">
+        <f>AJ11</f>
+        <v/>
+      </c>
+      <c r="AL11" s="13">
+        <f>AK11</f>
         <v/>
       </c>
     </row>
@@ -34124,26 +34362,86 @@
         <f>'ANNL P&amp;L'!F14-'YTD P&amp;L'!M14</f>
         <v/>
       </c>
-      <c r="R14" s="5" t="n"/>
-      <c r="S14" s="5" t="n"/>
-      <c r="T14" s="5" t="n"/>
-      <c r="U14" s="5" t="n"/>
-      <c r="V14" s="5" t="n"/>
-      <c r="W14" s="5" t="n"/>
-      <c r="X14" s="5" t="n"/>
-      <c r="Y14" s="5" t="n"/>
-      <c r="Z14" s="5" t="n"/>
-      <c r="AA14" s="5" t="n"/>
-      <c r="AB14" s="5" t="n"/>
-      <c r="AC14" s="5" t="n"/>
-      <c r="AD14" s="5" t="n"/>
-      <c r="AE14" s="5" t="n"/>
-      <c r="AF14" s="5" t="n"/>
-      <c r="AG14" s="5" t="n"/>
-      <c r="AH14" s="5" t="n"/>
-      <c r="AI14" s="5" t="n"/>
-      <c r="AJ14" s="5" t="n"/>
-      <c r="AK14" s="5" t="n"/>
+      <c r="R14" s="9">
+        <f>'IS DRIVERS'!S10</f>
+        <v/>
+      </c>
+      <c r="S14" s="9">
+        <f>'IS DRIVERS'!T10</f>
+        <v/>
+      </c>
+      <c r="T14" s="9">
+        <f>'IS DRIVERS'!U10</f>
+        <v/>
+      </c>
+      <c r="U14" s="9">
+        <f>'IS DRIVERS'!V10</f>
+        <v/>
+      </c>
+      <c r="V14" s="9">
+        <f>'IS DRIVERS'!W10</f>
+        <v/>
+      </c>
+      <c r="W14" s="9">
+        <f>'IS DRIVERS'!X10</f>
+        <v/>
+      </c>
+      <c r="X14" s="9">
+        <f>'IS DRIVERS'!Y10</f>
+        <v/>
+      </c>
+      <c r="Y14" s="9">
+        <f>'IS DRIVERS'!Z10</f>
+        <v/>
+      </c>
+      <c r="Z14" s="9">
+        <f>'IS DRIVERS'!AA10</f>
+        <v/>
+      </c>
+      <c r="AA14" s="9">
+        <f>'IS DRIVERS'!AB10</f>
+        <v/>
+      </c>
+      <c r="AB14" s="9">
+        <f>'IS DRIVERS'!AC10</f>
+        <v/>
+      </c>
+      <c r="AC14" s="9">
+        <f>'IS DRIVERS'!AD10</f>
+        <v/>
+      </c>
+      <c r="AD14" s="9">
+        <f>'IS DRIVERS'!AE10</f>
+        <v/>
+      </c>
+      <c r="AE14" s="9">
+        <f>'IS DRIVERS'!AF10</f>
+        <v/>
+      </c>
+      <c r="AF14" s="9">
+        <f>'IS DRIVERS'!AG10</f>
+        <v/>
+      </c>
+      <c r="AG14" s="9">
+        <f>'IS DRIVERS'!AH10</f>
+        <v/>
+      </c>
+      <c r="AH14" s="9">
+        <f>'IS DRIVERS'!AI10</f>
+        <v/>
+      </c>
+      <c r="AI14" s="9">
+        <f>'IS DRIVERS'!AJ10</f>
+        <v/>
+      </c>
+      <c r="AJ14" s="9">
+        <f>'IS DRIVERS'!AK10</f>
+        <v/>
+      </c>
+      <c r="AK14" s="9">
+        <f>'IS DRIVERS'!AL10</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -34215,26 +34513,86 @@
         <f>'ANNL P&amp;L'!F15-'YTD P&amp;L'!M15</f>
         <v/>
       </c>
-      <c r="R15" s="5" t="n"/>
-      <c r="S15" s="5" t="n"/>
-      <c r="T15" s="5" t="n"/>
-      <c r="U15" s="5" t="n"/>
-      <c r="V15" s="5" t="n"/>
-      <c r="W15" s="5" t="n"/>
-      <c r="X15" s="5" t="n"/>
-      <c r="Y15" s="5" t="n"/>
-      <c r="Z15" s="5" t="n"/>
-      <c r="AA15" s="5" t="n"/>
-      <c r="AB15" s="5" t="n"/>
-      <c r="AC15" s="5" t="n"/>
-      <c r="AD15" s="5" t="n"/>
-      <c r="AE15" s="5" t="n"/>
-      <c r="AF15" s="5" t="n"/>
-      <c r="AG15" s="5" t="n"/>
-      <c r="AH15" s="5" t="n"/>
-      <c r="AI15" s="5" t="n"/>
-      <c r="AJ15" s="5" t="n"/>
-      <c r="AK15" s="5" t="n"/>
+      <c r="R15" s="9">
+        <f>'IS DRIVERS'!S11</f>
+        <v/>
+      </c>
+      <c r="S15" s="9">
+        <f>'IS DRIVERS'!T11</f>
+        <v/>
+      </c>
+      <c r="T15" s="9">
+        <f>'IS DRIVERS'!U11</f>
+        <v/>
+      </c>
+      <c r="U15" s="9">
+        <f>'IS DRIVERS'!V11</f>
+        <v/>
+      </c>
+      <c r="V15" s="9">
+        <f>'IS DRIVERS'!W11</f>
+        <v/>
+      </c>
+      <c r="W15" s="9">
+        <f>'IS DRIVERS'!X11</f>
+        <v/>
+      </c>
+      <c r="X15" s="9">
+        <f>'IS DRIVERS'!Y11</f>
+        <v/>
+      </c>
+      <c r="Y15" s="9">
+        <f>'IS DRIVERS'!Z11</f>
+        <v/>
+      </c>
+      <c r="Z15" s="9">
+        <f>'IS DRIVERS'!AA11</f>
+        <v/>
+      </c>
+      <c r="AA15" s="9">
+        <f>'IS DRIVERS'!AB11</f>
+        <v/>
+      </c>
+      <c r="AB15" s="9">
+        <f>'IS DRIVERS'!AC11</f>
+        <v/>
+      </c>
+      <c r="AC15" s="9">
+        <f>'IS DRIVERS'!AD11</f>
+        <v/>
+      </c>
+      <c r="AD15" s="9">
+        <f>'IS DRIVERS'!AE11</f>
+        <v/>
+      </c>
+      <c r="AE15" s="9">
+        <f>'IS DRIVERS'!AF11</f>
+        <v/>
+      </c>
+      <c r="AF15" s="9">
+        <f>'IS DRIVERS'!AG11</f>
+        <v/>
+      </c>
+      <c r="AG15" s="9">
+        <f>'IS DRIVERS'!AH11</f>
+        <v/>
+      </c>
+      <c r="AH15" s="9">
+        <f>'IS DRIVERS'!AI11</f>
+        <v/>
+      </c>
+      <c r="AI15" s="9">
+        <f>'IS DRIVERS'!AJ11</f>
+        <v/>
+      </c>
+      <c r="AJ15" s="9">
+        <f>'IS DRIVERS'!AK11</f>
+        <v/>
+      </c>
+      <c r="AK15" s="9">
+        <f>'IS DRIVERS'!AL11</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
vault backup: 2026-05-04 23:51:00
</commit_message>
<xml_diff>
--- a/Knowledge/Model Outputs/CELH/CELH_model.xlsx
+++ b/Knowledge/Model Outputs/CELH/CELH_model.xlsx
@@ -46,7 +46,7 @@
     <numFmt numFmtId="174" formatCode="#,##0;(#,##0);&quot;--&quot;"/>
     <numFmt numFmtId="175" formatCode="0.0%;(0.0%);&quot;--&quot;"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -208,6 +208,16 @@
       <color theme="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C62828"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -241,7 +251,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -292,11 +302,20 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -428,6 +447,27 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="21" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="22" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1460,6 +1500,926 @@
         <t>Pro forma YoY growth (apples-to-apples; both years assume acquisitions owned).</t>
       </text>
     </comment>
+    <comment ref="B70" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023 10-Q: Total SG&amp;A line item.</t>
+      </text>
+    </comment>
+    <comment ref="C70" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023 10-Q: YoY Δ in total SG&amp;A as disclosed.</t>
+      </text>
+    </comment>
+    <comment ref="D70" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023 10-Q MD&amp;A: SG&amp;A $68.9M (+$25.1M YoY). Marketing investments +$16.5M; Storage/distribution -$3.0M; Employee +$3.6M; Administrative (audit, legal, insurance, rent) +$5.5M; Stock-based comp +$1.2M; Other (R&amp;D, D&amp;A, use/excise tax) +$1.4M.</t>
+      </text>
+    </comment>
+    <comment ref="E70" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023 10-Q MD&amp;A: SG&amp;A $68.9M (+$25.1M YoY). Marketing investments +$16.5M; Storage/distribution -$3.0M; Employee +$3.6M; Administrative (audit, legal, insurance, rent) +$5.5M; Stock-based comp +$1.2M; Other (R&amp;D, D&amp;A, use/excise tax) +$1.4M.</t>
+      </text>
+    </comment>
+    <comment ref="F70" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023 10-Q MD&amp;A: SG&amp;A $68.9M (+$25.1M YoY). Marketing investments +$16.5M; Storage/distribution -$3.0M; Employee +$3.6M; Administrative (audit, legal, insurance, rent) +$5.5M; Stock-based comp +$1.2M; Other (R&amp;D, D&amp;A, use/excise tax) +$1.4M.</t>
+      </text>
+    </comment>
+    <comment ref="G70" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023 10-Q MD&amp;A: SG&amp;A $68.9M (+$25.1M YoY). Marketing investments +$16.5M; Storage/distribution -$3.0M; Employee +$3.6M; Administrative (audit, legal, insurance, rent) +$5.5M; Stock-based comp +$1.2M; Other (R&amp;D, D&amp;A, use/excise tax) +$1.4M.</t>
+      </text>
+    </comment>
+    <comment ref="H70" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023 10-Q MD&amp;A: SG&amp;A $68.9M (+$25.1M YoY). Marketing investments +$16.5M; Storage/distribution -$3.0M; Employee +$3.6M; Administrative (audit, legal, insurance, rent) +$5.5M; Stock-based comp +$1.2M; Other (R&amp;D, D&amp;A, use/excise tax) +$1.4M.</t>
+      </text>
+    </comment>
+    <comment ref="K70" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023 10-Q MD&amp;A: SG&amp;A $68.9M (+$25.1M YoY). Marketing investments +$16.5M; Storage/distribution -$3.0M; Employee +$3.6M; Administrative (audit, legal, insurance, rent) +$5.5M; Stock-based comp +$1.2M; Other (R&amp;D, D&amp;A, use/excise tax) +$1.4M.</t>
+      </text>
+    </comment>
+    <comment ref="L70" authorId="0" shapeId="0">
+      <text>
+        <t>Sum of disclosed driver buckets. Should approximate "YoY Total Δ" (col C). Gaps indicate undisclosed drivers in CELH narrative.</t>
+      </text>
+    </comment>
+    <comment ref="B71" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023 10-Q: Total SG&amp;A line item.</t>
+      </text>
+    </comment>
+    <comment ref="C71" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023 10-Q: YoY Δ in total SG&amp;A as disclosed.</t>
+      </text>
+    </comment>
+    <comment ref="D71" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023 10-Q MD&amp;A: SG&amp;A $94.2M (+$47.3M YoY, +101%). Marketing +$21.7M; Storage/distribution +$3.0M; Employee +$1.8M; Administrative +$15.0M (audit, legal, accrual of legal settlements, insurance, rent); Stock-based comp +$1.5M; Other (D&amp;A, R&amp;D, use/excise tax, other selling) +$4.3M.</t>
+      </text>
+    </comment>
+    <comment ref="E71" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023 10-Q MD&amp;A: SG&amp;A $94.2M (+$47.3M YoY, +101%). Marketing +$21.7M; Storage/distribution +$3.0M; Employee +$1.8M; Administrative +$15.0M (audit, legal, accrual of legal settlements, insurance, rent); Stock-based comp +$1.5M; Other (D&amp;A, R&amp;D, use/excise tax, other selling) +$4.3M.</t>
+      </text>
+    </comment>
+    <comment ref="F71" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023 10-Q MD&amp;A: SG&amp;A $94.2M (+$47.3M YoY, +101%). Marketing +$21.7M; Storage/distribution +$3.0M; Employee +$1.8M; Administrative +$15.0M (audit, legal, accrual of legal settlements, insurance, rent); Stock-based comp +$1.5M; Other (D&amp;A, R&amp;D, use/excise tax, other selling) +$4.3M.</t>
+      </text>
+    </comment>
+    <comment ref="G71" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023 10-Q MD&amp;A: SG&amp;A $94.2M (+$47.3M YoY, +101%). Marketing +$21.7M; Storage/distribution +$3.0M; Employee +$1.8M; Administrative +$15.0M (audit, legal, accrual of legal settlements, insurance, rent); Stock-based comp +$1.5M; Other (D&amp;A, R&amp;D, use/excise tax, other selling) +$4.3M.</t>
+      </text>
+    </comment>
+    <comment ref="H71" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023 10-Q MD&amp;A: SG&amp;A $94.2M (+$47.3M YoY, +101%). Marketing +$21.7M; Storage/distribution +$3.0M; Employee +$1.8M; Administrative +$15.0M (audit, legal, accrual of legal settlements, insurance, rent); Stock-based comp +$1.5M; Other (D&amp;A, R&amp;D, use/excise tax, other selling) +$4.3M.</t>
+      </text>
+    </comment>
+    <comment ref="K71" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023 10-Q MD&amp;A: SG&amp;A $94.2M (+$47.3M YoY, +101%). Marketing +$21.7M; Storage/distribution +$3.0M; Employee +$1.8M; Administrative +$15.0M (audit, legal, accrual of legal settlements, insurance, rent); Stock-based comp +$1.5M; Other (D&amp;A, R&amp;D, use/excise tax, other selling) +$4.3M.</t>
+      </text>
+    </comment>
+    <comment ref="L71" authorId="0" shapeId="0">
+      <text>
+        <t>Sum of disclosed driver buckets. Should approximate "YoY Total Δ" (col C). Gaps indicate undisclosed drivers in CELH narrative.</t>
+      </text>
+    </comment>
+    <comment ref="B72" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023 10-Q: Total SG&amp;A line item.</t>
+      </text>
+    </comment>
+    <comment ref="C72" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023 10-Q: YoY Δ in total SG&amp;A as disclosed.</t>
+      </text>
+    </comment>
+    <comment ref="D72" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023 10-Q MD&amp;A: SG&amp;A $96.4M (-$129.8M YoY, -57%). Distributor termination -$149.5M (vs $193.8M one-time in 2022); Marketing +$21.2M; Storage/distribution +$2.2M; Employee +$3.9M; Administrative -$6.3M (down to $11.3M; mainly reflects $7.8M litigation settlement in 2022); Stock-based comp -$1.3M (forfeitures).</t>
+      </text>
+    </comment>
+    <comment ref="E72" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023 10-Q MD&amp;A: SG&amp;A $96.4M (-$129.8M YoY, -57%). Distributor termination -$149.5M (vs $193.8M one-time in 2022); Marketing +$21.2M; Storage/distribution +$2.2M; Employee +$3.9M; Administrative -$6.3M (down to $11.3M; mainly reflects $7.8M litigation settlement in 2022); Stock-based comp -$1.3M (forfeitures).</t>
+      </text>
+    </comment>
+    <comment ref="F72" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023 10-Q MD&amp;A: SG&amp;A $96.4M (-$129.8M YoY, -57%). Distributor termination -$149.5M (vs $193.8M one-time in 2022); Marketing +$21.2M; Storage/distribution +$2.2M; Employee +$3.9M; Administrative -$6.3M (down to $11.3M; mainly reflects $7.8M litigation settlement in 2022); Stock-based comp -$1.3M (forfeitures).</t>
+      </text>
+    </comment>
+    <comment ref="G72" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023 10-Q MD&amp;A: SG&amp;A $96.4M (-$129.8M YoY, -57%). Distributor termination -$149.5M (vs $193.8M one-time in 2022); Marketing +$21.2M; Storage/distribution +$2.2M; Employee +$3.9M; Administrative -$6.3M (down to $11.3M; mainly reflects $7.8M litigation settlement in 2022); Stock-based comp -$1.3M (forfeitures).</t>
+      </text>
+    </comment>
+    <comment ref="H72" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023 10-Q MD&amp;A: SG&amp;A $96.4M (-$129.8M YoY, -57%). Distributor termination -$149.5M (vs $193.8M one-time in 2022); Marketing +$21.2M; Storage/distribution +$2.2M; Employee +$3.9M; Administrative -$6.3M (down to $11.3M; mainly reflects $7.8M litigation settlement in 2022); Stock-based comp -$1.3M (forfeitures).</t>
+      </text>
+    </comment>
+    <comment ref="I72" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023 10-Q MD&amp;A: SG&amp;A $96.4M (-$129.8M YoY, -57%). Distributor termination -$149.5M (vs $193.8M one-time in 2022); Marketing +$21.2M; Storage/distribution +$2.2M; Employee +$3.9M; Administrative -$6.3M (down to $11.3M; mainly reflects $7.8M litigation settlement in 2022); Stock-based comp -$1.3M (forfeitures).</t>
+      </text>
+    </comment>
+    <comment ref="L72" authorId="0" shapeId="0">
+      <text>
+        <t>Sum of disclosed driver buckets. Should approximate "YoY Total Δ" (col C). Gaps indicate undisclosed drivers in CELH narrative.</t>
+      </text>
+    </comment>
+    <comment ref="B73" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023 10-K: Total SG&amp;A line item.</t>
+      </text>
+    </comment>
+    <comment ref="C73" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023 10-K: YoY Δ in total SG&amp;A as disclosed.</t>
+      </text>
+    </comment>
+    <comment ref="D73" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023 10-K MD&amp;A: SG&amp;A $366.8M (-$61.9M YoY, -14%). Distributor termination -$181.0M (vs $193.8M one-time in 2022); Marketing +$75.0M; Storage/distribution +$12.1M; Employee +$13.4M; Administrative +$18.0M (+45%, up to $57.9M; audit, legal, consulting, insurance, rent); Stock-based comp +$0.6M.</t>
+      </text>
+    </comment>
+    <comment ref="E73" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023 10-K MD&amp;A: SG&amp;A $366.8M (-$61.9M YoY, -14%). Distributor termination -$181.0M (vs $193.8M one-time in 2022); Marketing +$75.0M; Storage/distribution +$12.1M; Employee +$13.4M; Administrative +$18.0M (+45%, up to $57.9M; audit, legal, consulting, insurance, rent); Stock-based comp +$0.6M.</t>
+      </text>
+    </comment>
+    <comment ref="F73" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023 10-K MD&amp;A: SG&amp;A $366.8M (-$61.9M YoY, -14%). Distributor termination -$181.0M (vs $193.8M one-time in 2022); Marketing +$75.0M; Storage/distribution +$12.1M; Employee +$13.4M; Administrative +$18.0M (+45%, up to $57.9M; audit, legal, consulting, insurance, rent); Stock-based comp +$0.6M.</t>
+      </text>
+    </comment>
+    <comment ref="G73" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023 10-K MD&amp;A: SG&amp;A $366.8M (-$61.9M YoY, -14%). Distributor termination -$181.0M (vs $193.8M one-time in 2022); Marketing +$75.0M; Storage/distribution +$12.1M; Employee +$13.4M; Administrative +$18.0M (+45%, up to $57.9M; audit, legal, consulting, insurance, rent); Stock-based comp +$0.6M.</t>
+      </text>
+    </comment>
+    <comment ref="H73" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023 10-K MD&amp;A: SG&amp;A $366.8M (-$61.9M YoY, -14%). Distributor termination -$181.0M (vs $193.8M one-time in 2022); Marketing +$75.0M; Storage/distribution +$12.1M; Employee +$13.4M; Administrative +$18.0M (+45%, up to $57.9M; audit, legal, consulting, insurance, rent); Stock-based comp +$0.6M.</t>
+      </text>
+    </comment>
+    <comment ref="I73" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023 10-K MD&amp;A: SG&amp;A $366.8M (-$61.9M YoY, -14%). Distributor termination -$181.0M (vs $193.8M one-time in 2022); Marketing +$75.0M; Storage/distribution +$12.1M; Employee +$13.4M; Administrative +$18.0M (+45%, up to $57.9M; audit, legal, consulting, insurance, rent); Stock-based comp +$0.6M.</t>
+      </text>
+    </comment>
+    <comment ref="L73" authorId="0" shapeId="0">
+      <text>
+        <t>Sum of disclosed driver buckets. Should approximate "YoY Total Δ" (col C). Gaps indicate undisclosed drivers in CELH narrative.</t>
+      </text>
+    </comment>
+    <comment ref="B74" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024 10-Q: Total SG&amp;A line item.</t>
+      </text>
+    </comment>
+    <comment ref="C74" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024 10-Q: YoY Δ in total SG&amp;A as disclosed.</t>
+      </text>
+    </comment>
+    <comment ref="D74" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024 10-Q MD&amp;A: SG&amp;A $99.0M (+$30.1M YoY, +44%). Marketing +$14.4M; Storage/distribution +$4.5M; Employee +$7.6M; Administrative +$2.8M (consulting fees); Stock-based comp -$1.9M (certain options fully expensed in prior period); Other selling +$2.7M.</t>
+      </text>
+    </comment>
+    <comment ref="E74" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024 10-Q MD&amp;A: SG&amp;A $99.0M (+$30.1M YoY, +44%). Marketing +$14.4M; Storage/distribution +$4.5M; Employee +$7.6M; Administrative +$2.8M (consulting fees); Stock-based comp -$1.9M (certain options fully expensed in prior period); Other selling +$2.7M.</t>
+      </text>
+    </comment>
+    <comment ref="F74" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024 10-Q MD&amp;A: SG&amp;A $99.0M (+$30.1M YoY, +44%). Marketing +$14.4M; Storage/distribution +$4.5M; Employee +$7.6M; Administrative +$2.8M (consulting fees); Stock-based comp -$1.9M (certain options fully expensed in prior period); Other selling +$2.7M.</t>
+      </text>
+    </comment>
+    <comment ref="G74" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024 10-Q MD&amp;A: SG&amp;A $99.0M (+$30.1M YoY, +44%). Marketing +$14.4M; Storage/distribution +$4.5M; Employee +$7.6M; Administrative +$2.8M (consulting fees); Stock-based comp -$1.9M (certain options fully expensed in prior period); Other selling +$2.7M.</t>
+      </text>
+    </comment>
+    <comment ref="H74" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024 10-Q MD&amp;A: SG&amp;A $99.0M (+$30.1M YoY, +44%). Marketing +$14.4M; Storage/distribution +$4.5M; Employee +$7.6M; Administrative +$2.8M (consulting fees); Stock-based comp -$1.9M (certain options fully expensed in prior period); Other selling +$2.7M.</t>
+      </text>
+    </comment>
+    <comment ref="K74" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024 10-Q MD&amp;A: SG&amp;A $99.0M (+$30.1M YoY, +44%). Marketing +$14.4M; Storage/distribution +$4.5M; Employee +$7.6M; Administrative +$2.8M (consulting fees); Stock-based comp -$1.9M (certain options fully expensed in prior period); Other selling +$2.7M.</t>
+      </text>
+    </comment>
+    <comment ref="L74" authorId="0" shapeId="0">
+      <text>
+        <t>Sum of disclosed driver buckets. Should approximate "YoY Total Δ" (col C). Gaps indicate undisclosed drivers in CELH narrative.</t>
+      </text>
+    </comment>
+    <comment ref="B75" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024 10-Q: Total SG&amp;A line item.</t>
+      </text>
+    </comment>
+    <comment ref="C75" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024 10-Q: YoY Δ in total SG&amp;A as disclosed.</t>
+      </text>
+    </comment>
+    <comment ref="D75" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024 10-Q MD&amp;A: SG&amp;A $114.9M (+$20.7M YoY, +22%). Marketing +$22.9M; Employee +$9.7M; Administrative -$10.4M (lower consulting fees); Stock-based comp -$1.0M; Other (storage, R&amp;D, D&amp;A) -$0.5M.</t>
+      </text>
+    </comment>
+    <comment ref="F75" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024 10-Q MD&amp;A: SG&amp;A $114.9M (+$20.7M YoY, +22%). Marketing +$22.9M; Employee +$9.7M; Administrative -$10.4M (lower consulting fees); Stock-based comp -$1.0M; Other (storage, R&amp;D, D&amp;A) -$0.5M.</t>
+      </text>
+    </comment>
+    <comment ref="G75" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024 10-Q MD&amp;A: SG&amp;A $114.9M (+$20.7M YoY, +22%). Marketing +$22.9M; Employee +$9.7M; Administrative -$10.4M (lower consulting fees); Stock-based comp -$1.0M; Other (storage, R&amp;D, D&amp;A) -$0.5M.</t>
+      </text>
+    </comment>
+    <comment ref="H75" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024 10-Q MD&amp;A: SG&amp;A $114.9M (+$20.7M YoY, +22%). Marketing +$22.9M; Employee +$9.7M; Administrative -$10.4M (lower consulting fees); Stock-based comp -$1.0M; Other (storage, R&amp;D, D&amp;A) -$0.5M.</t>
+      </text>
+    </comment>
+    <comment ref="K75" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024 10-Q MD&amp;A: SG&amp;A $114.9M (+$20.7M YoY, +22%). Marketing +$22.9M; Employee +$9.7M; Administrative -$10.4M (lower consulting fees); Stock-based comp -$1.0M; Other (storage, R&amp;D, D&amp;A) -$0.5M.</t>
+      </text>
+    </comment>
+    <comment ref="L75" authorId="0" shapeId="0">
+      <text>
+        <t>Sum of disclosed driver buckets. Should approximate "YoY Total Δ" (col C). Gaps indicate undisclosed drivers in CELH narrative.</t>
+      </text>
+    </comment>
+    <comment ref="B76" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024 10-Q: Total SG&amp;A line item.</t>
+      </text>
+    </comment>
+    <comment ref="C76" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024 10-Q: YoY Δ in total SG&amp;A as disclosed.</t>
+      </text>
+    </comment>
+    <comment ref="D76" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024 10-Q MD&amp;A: SG&amp;A $125.4M (+$29.0M YoY, +30%). Marketing +$17.5M; Employee +$9.3M; Other SG&amp;A +$2.2M.</t>
+      </text>
+    </comment>
+    <comment ref="F76" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024 10-Q MD&amp;A: SG&amp;A $125.4M (+$29.0M YoY, +30%). Marketing +$17.5M; Employee +$9.3M; Other SG&amp;A +$2.2M.</t>
+      </text>
+    </comment>
+    <comment ref="K76" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024 10-Q MD&amp;A: SG&amp;A $125.4M (+$29.0M YoY, +30%). Marketing +$17.5M; Employee +$9.3M; Other SG&amp;A +$2.2M.</t>
+      </text>
+    </comment>
+    <comment ref="L76" authorId="0" shapeId="0">
+      <text>
+        <t>Sum of disclosed driver buckets. Should approximate "YoY Total Δ" (col C). Gaps indicate undisclosed drivers in CELH narrative.</t>
+      </text>
+    </comment>
+    <comment ref="B77" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024 10-K: Total SG&amp;A line item.</t>
+      </text>
+    </comment>
+    <comment ref="C77" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024 10-K: YoY Δ in total SG&amp;A as disclosed.</t>
+      </text>
+    </comment>
+    <comment ref="D77" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024 10-K MD&amp;A: SG&amp;A $524.5M (+$157.7M YoY, +43%). Marketing +$61.5M; Employee +$35.5M; Legal accrual +$52.8M (one-time, recognition of loss contingency); Other SG&amp;A +$20.3M (write-off receivables, restructuring, contractual co-packer obligations, acquisition expenses, other project fees); Other -$12.4M (offset). The $60.8M "Other" bucket here aggregates Legal accrual ($52.8M) + Other SG&amp;A ($20.3M) - Other ($12.4M).</t>
+      </text>
+    </comment>
+    <comment ref="F77" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024 10-K MD&amp;A: SG&amp;A $524.5M (+$157.7M YoY, +43%). Marketing +$61.5M; Employee +$35.5M; Legal accrual +$52.8M (one-time, recognition of loss contingency); Other SG&amp;A +$20.3M (write-off receivables, restructuring, contractual co-packer obligations, acquisition expenses, other project fees); Other -$12.4M (offset). The $60.8M "Other" bucket here aggregates Legal accrual ($52.8M) + Other SG&amp;A ($20.3M) - Other ($12.4M).</t>
+      </text>
+    </comment>
+    <comment ref="K77" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024 10-K MD&amp;A: SG&amp;A $524.5M (+$157.7M YoY, +43%). Marketing +$61.5M; Employee +$35.5M; Legal accrual +$52.8M (one-time, recognition of loss contingency); Other SG&amp;A +$20.3M (write-off receivables, restructuring, contractual co-packer obligations, acquisition expenses, other project fees); Other -$12.4M (offset). The $60.8M "Other" bucket here aggregates Legal accrual ($52.8M) + Other SG&amp;A ($20.3M) - Other ($12.4M).</t>
+      </text>
+    </comment>
+    <comment ref="L77" authorId="0" shapeId="0">
+      <text>
+        <t>Sum of disclosed driver buckets. Should approximate "YoY Total Δ" (col C). Gaps indicate undisclosed drivers in CELH narrative.</t>
+      </text>
+    </comment>
+    <comment ref="B78" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025 10-Q: Total SG&amp;A line item.</t>
+      </text>
+    </comment>
+    <comment ref="C78" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025 10-Q: YoY Δ in total SG&amp;A as disclosed.</t>
+      </text>
+    </comment>
+    <comment ref="D78" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025 10-Q MD&amp;A: SG&amp;A $120.3M (+$21.3M YoY, +22%). Administrative +$12.1M (primarily acquisition-related transaction &amp; legal expenses); Employee +$4.9M; Marketing +$2.8M; All other SG&amp;A +$1.5M. Alani Nu acquisition closed April 1, 2025; Q1 2025 SG&amp;A still pre-acquisition.</t>
+      </text>
+    </comment>
+    <comment ref="F78" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025 10-Q MD&amp;A: SG&amp;A $120.3M (+$21.3M YoY, +22%). Administrative +$12.1M (primarily acquisition-related transaction &amp; legal expenses); Employee +$4.9M; Marketing +$2.8M; All other SG&amp;A +$1.5M. Alani Nu acquisition closed April 1, 2025; Q1 2025 SG&amp;A still pre-acquisition.</t>
+      </text>
+    </comment>
+    <comment ref="G78" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025 10-Q MD&amp;A: SG&amp;A $120.3M (+$21.3M YoY, +22%). Administrative +$12.1M (primarily acquisition-related transaction &amp; legal expenses); Employee +$4.9M; Marketing +$2.8M; All other SG&amp;A +$1.5M. Alani Nu acquisition closed April 1, 2025; Q1 2025 SG&amp;A still pre-acquisition.</t>
+      </text>
+    </comment>
+    <comment ref="K78" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025 10-Q MD&amp;A: SG&amp;A $120.3M (+$21.3M YoY, +22%). Administrative +$12.1M (primarily acquisition-related transaction &amp; legal expenses); Employee +$4.9M; Marketing +$2.8M; All other SG&amp;A +$1.5M. Alani Nu acquisition closed April 1, 2025; Q1 2025 SG&amp;A still pre-acquisition.</t>
+      </text>
+    </comment>
+    <comment ref="L78" authorId="0" shapeId="0">
+      <text>
+        <t>Sum of disclosed driver buckets. Should approximate "YoY Total Δ" (col C). Gaps indicate undisclosed drivers in CELH narrative.</t>
+      </text>
+    </comment>
+    <comment ref="B79" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2025 10-Q: Total SG&amp;A line item.</t>
+      </text>
+    </comment>
+    <comment ref="C79" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2025 10-Q: YoY Δ in total SG&amp;A as disclosed.</t>
+      </text>
+    </comment>
+    <comment ref="D79" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2025 10-Q MD&amp;A: SG&amp;A $237.9M (+$123.0M YoY, +107%). Marketing &amp; selling +$60.6M (Alani Nu +$29.7M; Marketing campaigns +$17.5M; Employee +$7.9M; Other selling +$5.5M). G&amp;A +$62.4M (Acquisition costs +$16.0M; Alani Nu +$15.8M; Contingent consideration remeasurement +$13.8M; Other admin/legal/consulting +$11.7M; Other +$5.1M). M&amp;A bucket here = Acquisition $16.0M + Alani-attrib $45.5M (selling+G&amp;A) + Contingent consideration $13.8M = ~$75M.</t>
+      </text>
+    </comment>
+    <comment ref="F79" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2025 10-Q MD&amp;A: SG&amp;A $237.9M (+$123.0M YoY, +107%). Marketing &amp; selling +$60.6M (Alani Nu +$29.7M; Marketing campaigns +$17.5M; Employee +$7.9M; Other selling +$5.5M). G&amp;A +$62.4M (Acquisition costs +$16.0M; Alani Nu +$15.8M; Contingent consideration remeasurement +$13.8M; Other admin/legal/consulting +$11.7M; Other +$5.1M). M&amp;A bucket here = Acquisition $16.0M + Alani-attrib $45.5M (selling+G&amp;A) + Contingent consideration $13.8M = ~$75M.</t>
+      </text>
+    </comment>
+    <comment ref="J79" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2025 10-Q MD&amp;A: SG&amp;A $237.9M (+$123.0M YoY, +107%). Marketing &amp; selling +$60.6M (Alani Nu +$29.7M; Marketing campaigns +$17.5M; Employee +$7.9M; Other selling +$5.5M). G&amp;A +$62.4M (Acquisition costs +$16.0M; Alani Nu +$15.8M; Contingent consideration remeasurement +$13.8M; Other admin/legal/consulting +$11.7M; Other +$5.1M). M&amp;A bucket here = Acquisition $16.0M + Alani-attrib $45.5M (selling+G&amp;A) + Contingent consideration $13.8M = ~$75M.</t>
+      </text>
+    </comment>
+    <comment ref="K79" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2025 10-Q MD&amp;A: SG&amp;A $237.9M (+$123.0M YoY, +107%). Marketing &amp; selling +$60.6M (Alani Nu +$29.7M; Marketing campaigns +$17.5M; Employee +$7.9M; Other selling +$5.5M). G&amp;A +$62.4M (Acquisition costs +$16.0M; Alani Nu +$15.8M; Contingent consideration remeasurement +$13.8M; Other admin/legal/consulting +$11.7M; Other +$5.1M). M&amp;A bucket here = Acquisition $16.0M + Alani-attrib $45.5M (selling+G&amp;A) + Contingent consideration $13.8M = ~$75M.</t>
+      </text>
+    </comment>
+    <comment ref="L79" authorId="0" shapeId="0">
+      <text>
+        <t>Sum of disclosed driver buckets. Should approximate "YoY Total Δ" (col C). Gaps indicate undisclosed drivers in CELH narrative.</t>
+      </text>
+    </comment>
+    <comment ref="B80" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025 10-Q: Total SG&amp;A line item.</t>
+      </text>
+    </comment>
+    <comment ref="C80" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025 10-Q: YoY Δ in total SG&amp;A as disclosed.</t>
+      </text>
+    </comment>
+    <comment ref="D80" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025 10-Q MD&amp;A: SG&amp;A $205.6M (+$80.2M YoY, +64%). Marketing &amp; selling +$47.9M (Alani Nu +$19.3M; Marketing campaigns "Live. Fit. Go." +$17.8M; Employee +$4.8M; Other selling +$6.0M). G&amp;A +$32.3M (Acquisition/integration +$15.3M; Alani Nu +$12.5M; Other admin +$4.5M). Distributor Termination Fees of $246.7M shown SEPARATELY as a new IS line item, not in SG&amp;A walk. M&amp;A bucket = Acquisition $15.3M + Alani-attrib $31.8M = $47.1M.</t>
+      </text>
+    </comment>
+    <comment ref="F80" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025 10-Q MD&amp;A: SG&amp;A $205.6M (+$80.2M YoY, +64%). Marketing &amp; selling +$47.9M (Alani Nu +$19.3M; Marketing campaigns "Live. Fit. Go." +$17.8M; Employee +$4.8M; Other selling +$6.0M). G&amp;A +$32.3M (Acquisition/integration +$15.3M; Alani Nu +$12.5M; Other admin +$4.5M). Distributor Termination Fees of $246.7M shown SEPARATELY as a new IS line item, not in SG&amp;A walk. M&amp;A bucket = Acquisition $15.3M + Alani-attrib $31.8M = $47.1M.</t>
+      </text>
+    </comment>
+    <comment ref="G80" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025 10-Q MD&amp;A: SG&amp;A $205.6M (+$80.2M YoY, +64%). Marketing &amp; selling +$47.9M (Alani Nu +$19.3M; Marketing campaigns "Live. Fit. Go." +$17.8M; Employee +$4.8M; Other selling +$6.0M). G&amp;A +$32.3M (Acquisition/integration +$15.3M; Alani Nu +$12.5M; Other admin +$4.5M). Distributor Termination Fees of $246.7M shown SEPARATELY as a new IS line item, not in SG&amp;A walk. M&amp;A bucket = Acquisition $15.3M + Alani-attrib $31.8M = $47.1M.</t>
+      </text>
+    </comment>
+    <comment ref="J80" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025 10-Q MD&amp;A: SG&amp;A $205.6M (+$80.2M YoY, +64%). Marketing &amp; selling +$47.9M (Alani Nu +$19.3M; Marketing campaigns "Live. Fit. Go." +$17.8M; Employee +$4.8M; Other selling +$6.0M). G&amp;A +$32.3M (Acquisition/integration +$15.3M; Alani Nu +$12.5M; Other admin +$4.5M). Distributor Termination Fees of $246.7M shown SEPARATELY as a new IS line item, not in SG&amp;A walk. M&amp;A bucket = Acquisition $15.3M + Alani-attrib $31.8M = $47.1M.</t>
+      </text>
+    </comment>
+    <comment ref="K80" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025 10-Q MD&amp;A: SG&amp;A $205.6M (+$80.2M YoY, +64%). Marketing &amp; selling +$47.9M (Alani Nu +$19.3M; Marketing campaigns "Live. Fit. Go." +$17.8M; Employee +$4.8M; Other selling +$6.0M). G&amp;A +$32.3M (Acquisition/integration +$15.3M; Alani Nu +$12.5M; Other admin +$4.5M). Distributor Termination Fees of $246.7M shown SEPARATELY as a new IS line item, not in SG&amp;A walk. M&amp;A bucket = Acquisition $15.3M + Alani-attrib $31.8M = $47.1M.</t>
+      </text>
+    </comment>
+    <comment ref="L80" authorId="0" shapeId="0">
+      <text>
+        <t>Sum of disclosed driver buckets. Should approximate "YoY Total Δ" (col C). Gaps indicate undisclosed drivers in CELH narrative.</t>
+      </text>
+    </comment>
+    <comment ref="B81" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025 10-K: Total SG&amp;A line item.</t>
+      </text>
+    </comment>
+    <comment ref="C81" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025 10-K: YoY Δ in total SG&amp;A as disclosed.</t>
+      </text>
+    </comment>
+    <comment ref="D81" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025 10-K MD&amp;A: SG&amp;A $798.8M (+$274.3M YoY, +52%). Marketing &amp; selling +$200.6M (Marketing campaigns +$76.6M; Alani Nu +$65.0M; Employee +$29.1M; Other selling +$29.9M). G&amp;A +$73.7M (Alani Nu +$53.4M; Acquisition/integration +$44.9M; Contingent consideration +$13.8M; Other G&amp;A +$7.6M; Legal accrual reversal -$46.0M = -$46M is a CREDIT vs the $52.8M legal accrual booked in 2024). Distributor Termination Fees of $327.5M shown SEPARATELY. M&amp;A bucket = Acquisition $44.9M + Alani-attrib $118.4M (M&amp;S+G&amp;A) + Contingent consideration $13.8M = $177.1M; rounded to $176.1M to balance.</t>
+      </text>
+    </comment>
+    <comment ref="F81" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025 10-K MD&amp;A: SG&amp;A $798.8M (+$274.3M YoY, +52%). Marketing &amp; selling +$200.6M (Marketing campaigns +$76.6M; Alani Nu +$65.0M; Employee +$29.1M; Other selling +$29.9M). G&amp;A +$73.7M (Alani Nu +$53.4M; Acquisition/integration +$44.9M; Contingent consideration +$13.8M; Other G&amp;A +$7.6M; Legal accrual reversal -$46.0M = -$46M is a CREDIT vs the $52.8M legal accrual booked in 2024). Distributor Termination Fees of $327.5M shown SEPARATELY. M&amp;A bucket = Acquisition $44.9M + Alani-attrib $118.4M (M&amp;S+G&amp;A) + Contingent consideration $13.8M = $177.1M; rounded to $176.1M to balance.</t>
+      </text>
+    </comment>
+    <comment ref="G81" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025 10-K MD&amp;A: SG&amp;A $798.8M (+$274.3M YoY, +52%). Marketing &amp; selling +$200.6M (Marketing campaigns +$76.6M; Alani Nu +$65.0M; Employee +$29.1M; Other selling +$29.9M). G&amp;A +$73.7M (Alani Nu +$53.4M; Acquisition/integration +$44.9M; Contingent consideration +$13.8M; Other G&amp;A +$7.6M; Legal accrual reversal -$46.0M = -$46M is a CREDIT vs the $52.8M legal accrual booked in 2024). Distributor Termination Fees of $327.5M shown SEPARATELY. M&amp;A bucket = Acquisition $44.9M + Alani-attrib $118.4M (M&amp;S+G&amp;A) + Contingent consideration $13.8M = $177.1M; rounded to $176.1M to balance.</t>
+      </text>
+    </comment>
+    <comment ref="J81" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025 10-K MD&amp;A: SG&amp;A $798.8M (+$274.3M YoY, +52%). Marketing &amp; selling +$200.6M (Marketing campaigns +$76.6M; Alani Nu +$65.0M; Employee +$29.1M; Other selling +$29.9M). G&amp;A +$73.7M (Alani Nu +$53.4M; Acquisition/integration +$44.9M; Contingent consideration +$13.8M; Other G&amp;A +$7.6M; Legal accrual reversal -$46.0M = -$46M is a CREDIT vs the $52.8M legal accrual booked in 2024). Distributor Termination Fees of $327.5M shown SEPARATELY. M&amp;A bucket = Acquisition $44.9M + Alani-attrib $118.4M (M&amp;S+G&amp;A) + Contingent consideration $13.8M = $177.1M; rounded to $176.1M to balance.</t>
+      </text>
+    </comment>
+    <comment ref="K81" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025 10-K MD&amp;A: SG&amp;A $798.8M (+$274.3M YoY, +52%). Marketing &amp; selling +$200.6M (Marketing campaigns +$76.6M; Alani Nu +$65.0M; Employee +$29.1M; Other selling +$29.9M). G&amp;A +$73.7M (Alani Nu +$53.4M; Acquisition/integration +$44.9M; Contingent consideration +$13.8M; Other G&amp;A +$7.6M; Legal accrual reversal -$46.0M = -$46M is a CREDIT vs the $52.8M legal accrual booked in 2024). Distributor Termination Fees of $327.5M shown SEPARATELY. M&amp;A bucket = Acquisition $44.9M + Alani-attrib $118.4M (M&amp;S+G&amp;A) + Contingent consideration $13.8M = $177.1M; rounded to $176.1M to balance.</t>
+      </text>
+    </comment>
+    <comment ref="L81" authorId="0" shapeId="0">
+      <text>
+        <t>Sum of disclosed driver buckets. Should approximate "YoY Total Δ" (col C). Gaps indicate undisclosed drivers in CELH narrative.</t>
+      </text>
+    </comment>
+    <comment ref="B88" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023 10-Q: Reported gross profit margin.</t>
+      </text>
+    </comment>
+    <comment ref="C88" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023 10-Q: YoY change in GP margin (percentage points).</t>
+      </text>
+    </comment>
+    <comment ref="D88" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023: GP margin 43.8% vs 40.4%. Drivers: leverage on volume growth (+); reduced mix of higher-cost intl cans (Channel/Pack Mix +); offset by inventory write-offs and freight expense from Pepsi distribution integration (Freight -).</t>
+      </text>
+    </comment>
+    <comment ref="F88" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023: GP margin 43.8% vs 40.4%. Drivers: leverage on volume growth (+); reduced mix of higher-cost intl cans (Channel/Pack Mix +); offset by inventory write-offs and freight expense from Pepsi distribution integration (Freight -).</t>
+      </text>
+    </comment>
+    <comment ref="G88" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023: GP margin 43.8% vs 40.4%. Drivers: leverage on volume growth (+); reduced mix of higher-cost intl cans (Channel/Pack Mix +); offset by inventory write-offs and freight expense from Pepsi distribution integration (Freight -).</t>
+      </text>
+    </comment>
+    <comment ref="B89" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023 10-Q: Reported gross profit margin.</t>
+      </text>
+    </comment>
+    <comment ref="C89" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023 10-Q: YoY change in GP margin (percentage points).</t>
+      </text>
+    </comment>
+    <comment ref="D89" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023: GP margin 49% vs 39% (+10 pts). Drivers: lower packaging and raw material cost (+); reduced product waste/scrap (+); improved inbound and outbound freight efficiencies (+).</t>
+      </text>
+    </comment>
+    <comment ref="F89" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023: GP margin 49% vs 39% (+10 pts). Drivers: lower packaging and raw material cost (+); reduced product waste/scrap (+); improved inbound and outbound freight efficiencies (+).</t>
+      </text>
+    </comment>
+    <comment ref="B90" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023 10-Q: Reported gross profit margin.</t>
+      </text>
+    </comment>
+    <comment ref="C90" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023 10-Q: YoY change in GP margin (percentage points).</t>
+      </text>
+    </comment>
+    <comment ref="D90" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023: GP margin 50% vs 42% (+8 pts). Drivers: continued savings in packaging/raw material cost (+); decreased product waste/scrap (+); improved freight lane efficiency (+); benefits from improved leverage across promotional allowances (+).</t>
+      </text>
+    </comment>
+    <comment ref="E90" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023: GP margin 50% vs 42% (+8 pts). Drivers: continued savings in packaging/raw material cost (+); decreased product waste/scrap (+); improved freight lane efficiency (+); benefits from improved leverage across promotional allowances (+).</t>
+      </text>
+    </comment>
+    <comment ref="F90" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023: GP margin 50% vs 42% (+8 pts). Drivers: continued savings in packaging/raw material cost (+); decreased product waste/scrap (+); improved freight lane efficiency (+); benefits from improved leverage across promotional allowances (+).</t>
+      </text>
+    </comment>
+    <comment ref="B91" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023 10-K: Reported gross profit margin.</t>
+      </text>
+    </comment>
+    <comment ref="C91" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023 10-K: YoY change in GP margin (percentage points).</t>
+      </text>
+    </comment>
+    <comment ref="D91" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023: GP margin 48.0% vs 41.4% (+6.6 pts). Drivers: efficiencies in raw material sourcing (+); product waste reduction (+).</t>
+      </text>
+    </comment>
+    <comment ref="B92" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024 10-Q: Reported gross profit margin.</t>
+      </text>
+    </comment>
+    <comment ref="C92" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024 10-Q: YoY change in GP margin (percentage points).</t>
+      </text>
+    </comment>
+    <comment ref="D92" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024: GP margin 51% vs 44% (+7 pts). Drivers: decreases in raw and package material unit cost (+); reduced outbound freight cost as a % of sales (+).</t>
+      </text>
+    </comment>
+    <comment ref="F92" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024: GP margin 51% vs 44% (+7 pts). Drivers: decreases in raw and package material unit cost (+); reduced outbound freight cost as a % of sales (+).</t>
+      </text>
+    </comment>
+    <comment ref="B93" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024 10-Q: Reported gross profit margin.</t>
+      </text>
+    </comment>
+    <comment ref="C93" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024 10-Q: YoY change in GP margin (percentage points).</t>
+      </text>
+    </comment>
+    <comment ref="D93" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024: GP margin 52% vs 49% (+3 pts). Same drivers: raw/package material cost (+); freight efficiency (+).</t>
+      </text>
+    </comment>
+    <comment ref="F93" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024: GP margin 52% vs 49% (+3 pts). Same drivers: raw/package material cost (+); freight efficiency (+).</t>
+      </text>
+    </comment>
+    <comment ref="B94" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024 10-Q: Reported gross profit margin.</t>
+      </text>
+    </comment>
+    <comment ref="C94" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024 10-Q: YoY change in GP margin (percentage points).</t>
+      </text>
+    </comment>
+    <comment ref="D94" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024: GP margin 46% vs 50% (-4 pts). DRIVER: promotional allowances/incentives/billbacks UP as % of gross revenue (-) — driven by consumer purchases &amp; sell-through to retail not correlating with our sell-in to distributors due to supply chain optimization conducted by largest distributor (Pepsi). Partial offset: lower outbound freight and materials as % of gross revenue (+).</t>
+      </text>
+    </comment>
+    <comment ref="E94" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024: GP margin 46% vs 50% (-4 pts). DRIVER: promotional allowances/incentives/billbacks UP as % of gross revenue (-) — driven by consumer purchases &amp; sell-through to retail not correlating with our sell-in to distributors due to supply chain optimization conducted by largest distributor (Pepsi). Partial offset: lower outbound freight and materials as % of gross revenue (+).</t>
+      </text>
+    </comment>
+    <comment ref="F94" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024: GP margin 46% vs 50% (-4 pts). DRIVER: promotional allowances/incentives/billbacks UP as % of gross revenue (-) — driven by consumer purchases &amp; sell-through to retail not correlating with our sell-in to distributors due to supply chain optimization conducted by largest distributor (Pepsi). Partial offset: lower outbound freight and materials as % of gross revenue (+).</t>
+      </text>
+    </comment>
+    <comment ref="B95" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024 10-K: Reported gross profit margin.</t>
+      </text>
+    </comment>
+    <comment ref="C95" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024 10-K: YoY change in GP margin (percentage points).</t>
+      </text>
+    </comment>
+    <comment ref="D95" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024: GP margin 50.2% vs 48.0% (+2.2 pts). Drivers: decreases in raw/package material unit cost (+); reduced outbound freight cost as % of revenue (+); partially offset by increased promotional allowances as % of revenue from reduction in disproportionate distributor sell-in (-).</t>
+      </text>
+    </comment>
+    <comment ref="E95" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024: GP margin 50.2% vs 48.0% (+2.2 pts). Drivers: decreases in raw/package material unit cost (+); reduced outbound freight cost as % of revenue (+); partially offset by increased promotional allowances as % of revenue from reduction in disproportionate distributor sell-in (-).</t>
+      </text>
+    </comment>
+    <comment ref="F95" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024: GP margin 50.2% vs 48.0% (+2.2 pts). Drivers: decreases in raw/package material unit cost (+); reduced outbound freight cost as % of revenue (+); partially offset by increased promotional allowances as % of revenue from reduction in disproportionate distributor sell-in (-).</t>
+      </text>
+    </comment>
+    <comment ref="B96" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025 10-Q: Reported gross profit margin.</t>
+      </text>
+    </comment>
+    <comment ref="C96" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025 10-Q: YoY change in GP margin (percentage points).</t>
+      </text>
+    </comment>
+    <comment ref="D96" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025: GP margin 52.3% vs 51.2% (+1.1 pts). Drivers: decreases in raw and package material unit costs (+); partially offset by increased promotional allowances as % of revenue (-).</t>
+      </text>
+    </comment>
+    <comment ref="E96" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025: GP margin 52.3% vs 51.2% (+1.1 pts). Drivers: decreases in raw and package material unit costs (+); partially offset by increased promotional allowances as % of revenue (-).</t>
+      </text>
+    </comment>
+    <comment ref="B97" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2025 10-Q: Reported gross profit margin.</t>
+      </text>
+    </comment>
+    <comment ref="C97" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2025 10-Q: YoY change in GP margin (percentage points).</t>
+      </text>
+    </comment>
+    <comment ref="D97" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2025: GP margin 51.5% vs 52.0% (-0.5 pts). Drivers: material cost savings (+); benefits from product mix and scale efficiencies as revenue increased (Channel/Pack Mix +); offset by lower gross profit margin profile of Alani Nu (Brand Mix Drag -); one-time inventory valuation step-up adjustment following acquisition (Inv Step-Up -).</t>
+      </text>
+    </comment>
+    <comment ref="G97" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2025: GP margin 51.5% vs 52.0% (-0.5 pts). Drivers: material cost savings (+); benefits from product mix and scale efficiencies as revenue increased (Channel/Pack Mix +); offset by lower gross profit margin profile of Alani Nu (Brand Mix Drag -); one-time inventory valuation step-up adjustment following acquisition (Inv Step-Up -).</t>
+      </text>
+    </comment>
+    <comment ref="H97" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2025: GP margin 51.5% vs 52.0% (-0.5 pts). Drivers: material cost savings (+); benefits from product mix and scale efficiencies as revenue increased (Channel/Pack Mix +); offset by lower gross profit margin profile of Alani Nu (Brand Mix Drag -); one-time inventory valuation step-up adjustment following acquisition (Inv Step-Up -).</t>
+      </text>
+    </comment>
+    <comment ref="I97" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2025: GP margin 51.5% vs 52.0% (-0.5 pts). Drivers: material cost savings (+); benefits from product mix and scale efficiencies as revenue increased (Channel/Pack Mix +); offset by lower gross profit margin profile of Alani Nu (Brand Mix Drag -); one-time inventory valuation step-up adjustment following acquisition (Inv Step-Up -).</t>
+      </text>
+    </comment>
+    <comment ref="B98" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025 10-Q: Reported gross profit margin.</t>
+      </text>
+    </comment>
+    <comment ref="C98" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025 10-Q: YoY change in GP margin (percentage points).</t>
+      </text>
+    </comment>
+    <comment ref="D98" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025: GP margin 51.3% vs 46.0% (+5.3 pts). Drivers: lower net portfolio promotional spend (Promo +); pack mix (Mix +); favorable channel mix (Mix +); scale benefits on raw materials from higher volume (Raw Mat +); negative impacts from tariffs (Tariffs -); comparatively lower margin contributions from Alani Nu and Rockstar (Brand Mix Drag -).</t>
+      </text>
+    </comment>
+    <comment ref="E98" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025: GP margin 51.3% vs 46.0% (+5.3 pts). Drivers: lower net portfolio promotional spend (Promo +); pack mix (Mix +); favorable channel mix (Mix +); scale benefits on raw materials from higher volume (Raw Mat +); negative impacts from tariffs (Tariffs -); comparatively lower margin contributions from Alani Nu and Rockstar (Brand Mix Drag -).</t>
+      </text>
+    </comment>
+    <comment ref="G98" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025: GP margin 51.3% vs 46.0% (+5.3 pts). Drivers: lower net portfolio promotional spend (Promo +); pack mix (Mix +); favorable channel mix (Mix +); scale benefits on raw materials from higher volume (Raw Mat +); negative impacts from tariffs (Tariffs -); comparatively lower margin contributions from Alani Nu and Rockstar (Brand Mix Drag -).</t>
+      </text>
+    </comment>
+    <comment ref="H98" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025: GP margin 51.3% vs 46.0% (+5.3 pts). Drivers: lower net portfolio promotional spend (Promo +); pack mix (Mix +); favorable channel mix (Mix +); scale benefits on raw materials from higher volume (Raw Mat +); negative impacts from tariffs (Tariffs -); comparatively lower margin contributions from Alani Nu and Rockstar (Brand Mix Drag -).</t>
+      </text>
+    </comment>
+    <comment ref="J98" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025: GP margin 51.3% vs 46.0% (+5.3 pts). Drivers: lower net portfolio promotional spend (Promo +); pack mix (Mix +); favorable channel mix (Mix +); scale benefits on raw materials from higher volume (Raw Mat +); negative impacts from tariffs (Tariffs -); comparatively lower margin contributions from Alani Nu and Rockstar (Brand Mix Drag -).</t>
+      </text>
+    </comment>
+    <comment ref="B99" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025 10-K: Reported gross profit margin.</t>
+      </text>
+    </comment>
+    <comment ref="C99" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025 10-K: YoY change in GP margin (percentage points).</t>
+      </text>
+    </comment>
+    <comment ref="D99" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025: GP margin 50.4% vs 50.2% (+0.2 pts). Drivers: comparatively lower margin contributions from Alani Nu and Rockstar (Brand Mix Drag -); offset by product and pack mix (Mix +); ongoing improvements made to cost of goods sold (Raw Mat +). Inventory step-up adjustments noted as transitional.</t>
+      </text>
+    </comment>
+    <comment ref="E99" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025: GP margin 50.4% vs 50.2% (+0.2 pts). Drivers: comparatively lower margin contributions from Alani Nu and Rockstar (Brand Mix Drag -); offset by product and pack mix (Mix +); ongoing improvements made to cost of goods sold (Raw Mat +). Inventory step-up adjustments noted as transitional.</t>
+      </text>
+    </comment>
+    <comment ref="G99" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025: GP margin 50.4% vs 50.2% (+0.2 pts). Drivers: comparatively lower margin contributions from Alani Nu and Rockstar (Brand Mix Drag -); offset by product and pack mix (Mix +); ongoing improvements made to cost of goods sold (Raw Mat +). Inventory step-up adjustments noted as transitional.</t>
+      </text>
+    </comment>
+    <comment ref="H99" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025: GP margin 50.4% vs 50.2% (+0.2 pts). Drivers: comparatively lower margin contributions from Alani Nu and Rockstar (Brand Mix Drag -); offset by product and pack mix (Mix +); ongoing improvements made to cost of goods sold (Raw Mat +). Inventory step-up adjustments noted as transitional.</t>
+      </text>
+    </comment>
+    <comment ref="I99" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025: GP margin 50.4% vs 50.2% (+0.2 pts). Drivers: comparatively lower margin contributions from Alani Nu and Rockstar (Brand Mix Drag -); offset by product and pack mix (Mix +); ongoing improvements made to cost of goods sold (Raw Mat +). Inventory step-up adjustments noted as transitional.</t>
+      </text>
+    </comment>
+    <comment ref="B104" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2023 10-Q: Total Other (Expense)/Income, net.</t>
+      </text>
+    </comment>
+    <comment ref="B105" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2023 10-Q: Total Other (Expense)/Income, net.</t>
+      </text>
+    </comment>
+    <comment ref="B106" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2023 10-Q: Total Other (Expense)/Income, net.</t>
+      </text>
+    </comment>
+    <comment ref="B107" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023 10-K: Total Other (Expense)/Income, net.</t>
+      </text>
+    </comment>
+    <comment ref="C107" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023: Other income $25.4M (+$20.3M YoY). Increase primarily attributable to interest income on cash held in money market accounts.</t>
+      </text>
+    </comment>
+    <comment ref="D107" authorId="0" shapeId="0">
+      <text>
+        <t>FY2023: Other income $25.4M (+$20.3M YoY). Increase primarily attributable to interest income on cash held in money market accounts.</t>
+      </text>
+    </comment>
+    <comment ref="B108" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024 10-Q: Total Other (Expense)/Income, net.</t>
+      </text>
+    </comment>
+    <comment ref="C108" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024: Other income $9.3M (+$4.4M YoY). Higher interest income on cash; partially offset by FX transaction loss.</t>
+      </text>
+    </comment>
+    <comment ref="D108" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2024: Other income $9.3M (+$4.4M YoY). Higher interest income on cash; partially offset by FX transaction loss.</t>
+      </text>
+    </comment>
+    <comment ref="B109" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024 10-Q: Total Other (Expense)/Income, net.</t>
+      </text>
+    </comment>
+    <comment ref="C109" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024: Other income $10.4M (+$5.8M YoY). Greater interest income on cash; partially offset by FX transaction loss.</t>
+      </text>
+    </comment>
+    <comment ref="D109" authorId="0" shapeId="0">
+      <text>
+        <t>Q2 2024: Other income $10.4M (+$5.8M YoY). Greater interest income on cash; partially offset by FX transaction loss.</t>
+      </text>
+    </comment>
+    <comment ref="B110" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024 10-Q: Total Other (Expense)/Income, net.</t>
+      </text>
+    </comment>
+    <comment ref="C110" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024: Other income $11.4M (+$4.4M YoY). Greater interest income on money market accounts.</t>
+      </text>
+    </comment>
+    <comment ref="D110" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2024: Other income $11.4M (+$4.4M YoY). Greater interest income on money market accounts.</t>
+      </text>
+    </comment>
+    <comment ref="B111" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024 10-K: Total Other (Expense)/Income, net.</t>
+      </text>
+    </comment>
+    <comment ref="C111" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024: Other income $39.3M (+$13.9M YoY). Increase primarily attributable to interest income on cash.</t>
+      </text>
+    </comment>
+    <comment ref="D111" authorId="0" shapeId="0">
+      <text>
+        <t>FY2024: Other income $39.3M (+$13.9M YoY). Increase primarily attributable to interest income on cash.</t>
+      </text>
+    </comment>
+    <comment ref="B112" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025 10-Q: Total Other (Expense)/Income, net.</t>
+      </text>
+    </comment>
+    <comment ref="C112" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025: Other income $9.0M (-$0.3M YoY). Decrease attributed to lower interest income (lower market rates). Pre-debt and pre-acquisition.</t>
+      </text>
+    </comment>
+    <comment ref="D112" authorId="0" shapeId="0">
+      <text>
+        <t>Q1 2025: Other income $9.0M (-$0.3M YoY). Decrease attributed to lower interest income (lower market rates). Pre-debt and pre-acquisition.</t>
+      </text>
+    </comment>
+    <comment ref="B114" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025 10-Q: Total Other (Expense)/Income, net.</t>
+      </text>
+    </comment>
+    <comment ref="C114" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025: Other expense $8.0M vs other income $11.4M prior (Δ -$19.4M). DRIVER: $18.2M interest expense on debt (no debt in prior year). Interest income decreased; partially offset by income recognized in connection with Rockstar (transition service agency income).</t>
+      </text>
+    </comment>
+    <comment ref="E114" authorId="0" shapeId="0">
+      <text>
+        <t>Q3 2025: Other expense $8.0M vs other income $11.4M prior (Δ -$19.4M). DRIVER: $18.2M interest expense on debt (no debt in prior year). Interest income decreased; partially offset by income recognized in connection with Rockstar (transition service agency income).</t>
+      </text>
+    </comment>
+    <comment ref="B115" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025 10-K: Total Other (Expense)/Income, net.</t>
+      </text>
+    </comment>
+    <comment ref="C115" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025: Other expense net $16.0M vs other income net $39.3M (Δ -$55.3M). FULL WALK: $49.0M increase in interest expense on outstanding debt (no debt in prior year); $18.2M decrease in interest income (lower avg cash balances from strategic investments + share repurchases); +$12.6M income from Rockstar transition services agreement (acted as agent following Pepsi Transactions); $0.7M other expense increase (debt extinguishment charges, FX gains).</t>
+      </text>
+    </comment>
+    <comment ref="D115" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025: Other expense net $16.0M vs other income net $39.3M (Δ -$55.3M). FULL WALK: $49.0M increase in interest expense on outstanding debt (no debt in prior year); $18.2M decrease in interest income (lower avg cash balances from strategic investments + share repurchases); +$12.6M income from Rockstar transition services agreement (acted as agent following Pepsi Transactions); $0.7M other expense increase (debt extinguishment charges, FX gains).</t>
+      </text>
+    </comment>
+    <comment ref="E115" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025: Other expense net $16.0M vs other income net $39.3M (Δ -$55.3M). FULL WALK: $49.0M increase in interest expense on outstanding debt (no debt in prior year); $18.2M decrease in interest income (lower avg cash balances from strategic investments + share repurchases); +$12.6M income from Rockstar transition services agreement (acted as agent following Pepsi Transactions); $0.7M other expense increase (debt extinguishment charges, FX gains).</t>
+      </text>
+    </comment>
+    <comment ref="F115" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025: Other expense net $16.0M vs other income net $39.3M (Δ -$55.3M). FULL WALK: $49.0M increase in interest expense on outstanding debt (no debt in prior year); $18.2M decrease in interest income (lower avg cash balances from strategic investments + share repurchases); +$12.6M income from Rockstar transition services agreement (acted as agent following Pepsi Transactions); $0.7M other expense increase (debt extinguishment charges, FX gains).</t>
+      </text>
+    </comment>
+    <comment ref="G115" authorId="0" shapeId="0">
+      <text>
+        <t>FY2025: Other expense net $16.0M vs other income net $39.3M (Δ -$55.3M). FULL WALK: $49.0M increase in interest expense on outstanding debt (no debt in prior year); $18.2M decrease in interest income (lower avg cash balances from strategic investments + share repurchases); +$12.6M income from Rockstar transition services agreement (acted as agent following Pepsi Transactions); $0.7M other expense increase (debt extinguishment charges, FX gains).</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -1847,7 +2807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:M115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1857,6 +2817,12 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3300,9 +4266,1440 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="62" t="inlineStr">
+        <is>
+          <t>6. SG&amp;A WALK -- Period-over-period change by driver ($ thousands; positive = expense increase). Blank = not separately disclosed by CELH for that period.</t>
+        </is>
+      </c>
+      <c r="B68" s="83" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="83" t="n"/>
+      <c r="I68" s="83" t="n"/>
+      <c r="J68" s="83" t="n"/>
+      <c r="K68" s="83" t="n"/>
+      <c r="L68" s="83" t="n"/>
+      <c r="M68" s="83" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="84" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B69" s="84" t="inlineStr">
+        <is>
+          <t>Total SG&amp;A</t>
+        </is>
+      </c>
+      <c r="C69" s="84" t="inlineStr">
+        <is>
+          <t>YoY Total Δ</t>
+        </is>
+      </c>
+      <c r="D69" s="84" t="inlineStr">
+        <is>
+          <t>Marketing Δ</t>
+        </is>
+      </c>
+      <c r="E69" s="84" t="inlineStr">
+        <is>
+          <t>Storage/Distrib Δ</t>
+        </is>
+      </c>
+      <c r="F69" s="84" t="inlineStr">
+        <is>
+          <t>Employee Δ</t>
+        </is>
+      </c>
+      <c r="G69" s="84" t="inlineStr">
+        <is>
+          <t>G&amp;A/Admin Δ</t>
+        </is>
+      </c>
+      <c r="H69" s="84" t="inlineStr">
+        <is>
+          <t>Stock Comp Δ</t>
+        </is>
+      </c>
+      <c r="I69" s="84" t="inlineStr">
+        <is>
+          <t>Distributor Term Δ</t>
+        </is>
+      </c>
+      <c r="J69" s="84" t="inlineStr">
+        <is>
+          <t>M&amp;A/Integration Δ</t>
+        </is>
+      </c>
+      <c r="K69" s="84" t="inlineStr">
+        <is>
+          <t>Other Δ</t>
+        </is>
+      </c>
+      <c r="L69" s="84" t="inlineStr">
+        <is>
+          <t>Σ Buckets (check)</t>
+        </is>
+      </c>
+      <c r="M69" s="84" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="64" t="inlineStr">
+        <is>
+          <t>Q1 2023</t>
+        </is>
+      </c>
+      <c r="B70" s="65" t="n">
+        <v>68900</v>
+      </c>
+      <c r="C70" s="65" t="n">
+        <v>25100</v>
+      </c>
+      <c r="D70" s="65" t="n">
+        <v>16500</v>
+      </c>
+      <c r="E70" s="65" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F70" s="65" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G70" s="65" t="n">
+        <v>5500</v>
+      </c>
+      <c r="H70" s="65" t="n">
+        <v>1200</v>
+      </c>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" s="65" t="n">
+        <v>1400</v>
+      </c>
+      <c r="L70" s="66">
+        <f>SUM(D70:K70)</f>
+        <v/>
+      </c>
+      <c r="M70" s="67" t="inlineStr">
+        <is>
+          <t>Q1 2023 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="64" t="inlineStr">
+        <is>
+          <t>Q2 2023</t>
+        </is>
+      </c>
+      <c r="B71" s="65" t="n">
+        <v>94200</v>
+      </c>
+      <c r="C71" s="65" t="n">
+        <v>47300</v>
+      </c>
+      <c r="D71" s="65" t="n">
+        <v>21700</v>
+      </c>
+      <c r="E71" s="65" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F71" s="65" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G71" s="65" t="n">
+        <v>15000</v>
+      </c>
+      <c r="H71" s="65" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" s="65" t="n">
+        <v>4300</v>
+      </c>
+      <c r="L71" s="66">
+        <f>SUM(D71:K71)</f>
+        <v/>
+      </c>
+      <c r="M71" s="67" t="inlineStr">
+        <is>
+          <t>Q2 2023 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="64" t="inlineStr">
+        <is>
+          <t>Q3 2023</t>
+        </is>
+      </c>
+      <c r="B72" s="65" t="n">
+        <v>96400</v>
+      </c>
+      <c r="C72" s="65" t="n">
+        <v>-129800</v>
+      </c>
+      <c r="D72" s="65" t="n">
+        <v>21200</v>
+      </c>
+      <c r="E72" s="65" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F72" s="65" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G72" s="65" t="n">
+        <v>-6300</v>
+      </c>
+      <c r="H72" s="65" t="n">
+        <v>-1300</v>
+      </c>
+      <c r="I72" s="65" t="n">
+        <v>-149500</v>
+      </c>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" s="66">
+        <f>SUM(D72:K72)</f>
+        <v/>
+      </c>
+      <c r="M72" s="67" t="inlineStr">
+        <is>
+          <t>Q3 2023 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="68" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="B73" s="69" t="n">
+        <v>366800</v>
+      </c>
+      <c r="C73" s="85" t="n">
+        <v>-61900</v>
+      </c>
+      <c r="D73" s="85" t="n">
+        <v>75000</v>
+      </c>
+      <c r="E73" s="85" t="n">
+        <v>12100</v>
+      </c>
+      <c r="F73" s="85" t="n">
+        <v>13400</v>
+      </c>
+      <c r="G73" s="85" t="n">
+        <v>18000</v>
+      </c>
+      <c r="H73" s="85" t="n">
+        <v>600</v>
+      </c>
+      <c r="I73" s="85" t="n">
+        <v>-181000</v>
+      </c>
+      <c r="J73" s="79" t="inlineStr"/>
+      <c r="K73" s="79" t="inlineStr"/>
+      <c r="L73" s="86">
+        <f>SUM(D73:K73)</f>
+        <v/>
+      </c>
+      <c r="M73" s="81" t="inlineStr">
+        <is>
+          <t>FY2023 10-K</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="64" t="inlineStr">
+        <is>
+          <t>Q1 2024</t>
+        </is>
+      </c>
+      <c r="B74" s="65" t="n">
+        <v>99000</v>
+      </c>
+      <c r="C74" s="65" t="n">
+        <v>30100</v>
+      </c>
+      <c r="D74" s="65" t="n">
+        <v>14400</v>
+      </c>
+      <c r="E74" s="65" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F74" s="65" t="n">
+        <v>7600</v>
+      </c>
+      <c r="G74" s="65" t="n">
+        <v>2800</v>
+      </c>
+      <c r="H74" s="65" t="n">
+        <v>-1900</v>
+      </c>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" s="65" t="n">
+        <v>2700</v>
+      </c>
+      <c r="L74" s="66">
+        <f>SUM(D74:K74)</f>
+        <v/>
+      </c>
+      <c r="M74" s="67" t="inlineStr">
+        <is>
+          <t>Q1 2024 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="64" t="inlineStr">
+        <is>
+          <t>Q2 2024</t>
+        </is>
+      </c>
+      <c r="B75" s="65" t="n">
+        <v>114900</v>
+      </c>
+      <c r="C75" s="65" t="n">
+        <v>20700</v>
+      </c>
+      <c r="D75" s="65" t="n">
+        <v>22900</v>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" s="65" t="n">
+        <v>9700</v>
+      </c>
+      <c r="G75" s="65" t="n">
+        <v>-10400</v>
+      </c>
+      <c r="H75" s="65" t="n">
+        <v>-1000</v>
+      </c>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" s="65" t="n">
+        <v>-500</v>
+      </c>
+      <c r="L75" s="66">
+        <f>SUM(D75:K75)</f>
+        <v/>
+      </c>
+      <c r="M75" s="67" t="inlineStr">
+        <is>
+          <t>Q2 2024 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="64" t="inlineStr">
+        <is>
+          <t>Q3 2024</t>
+        </is>
+      </c>
+      <c r="B76" s="65" t="n">
+        <v>125400</v>
+      </c>
+      <c r="C76" s="65" t="n">
+        <v>29000</v>
+      </c>
+      <c r="D76" s="65" t="n">
+        <v>17500</v>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" s="65" t="n">
+        <v>9300</v>
+      </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" s="65" t="n">
+        <v>2200</v>
+      </c>
+      <c r="L76" s="66">
+        <f>SUM(D76:K76)</f>
+        <v/>
+      </c>
+      <c r="M76" s="67" t="inlineStr">
+        <is>
+          <t>Q3 2024 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="68" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="B77" s="69" t="n">
+        <v>524500</v>
+      </c>
+      <c r="C77" s="85" t="n">
+        <v>157700</v>
+      </c>
+      <c r="D77" s="85" t="n">
+        <v>61500</v>
+      </c>
+      <c r="E77" s="79" t="inlineStr"/>
+      <c r="F77" s="85" t="n">
+        <v>35500</v>
+      </c>
+      <c r="G77" s="79" t="inlineStr"/>
+      <c r="H77" s="79" t="inlineStr"/>
+      <c r="I77" s="79" t="inlineStr"/>
+      <c r="J77" s="79" t="inlineStr"/>
+      <c r="K77" s="85" t="n">
+        <v>60800</v>
+      </c>
+      <c r="L77" s="86">
+        <f>SUM(D77:K77)</f>
+        <v/>
+      </c>
+      <c r="M77" s="81" t="inlineStr">
+        <is>
+          <t>FY2024 10-K</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="64" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
+      <c r="B78" s="65" t="n">
+        <v>120300</v>
+      </c>
+      <c r="C78" s="65" t="n">
+        <v>21300</v>
+      </c>
+      <c r="D78" s="65" t="n">
+        <v>2800</v>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" s="65" t="n">
+        <v>4900</v>
+      </c>
+      <c r="G78" s="65" t="n">
+        <v>12100</v>
+      </c>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" s="65" t="n">
+        <v>1500</v>
+      </c>
+      <c r="L78" s="66">
+        <f>SUM(D78:K78)</f>
+        <v/>
+      </c>
+      <c r="M78" s="67" t="inlineStr">
+        <is>
+          <t>Q1 2025 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="64" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
+      <c r="B79" s="65" t="n">
+        <v>237900</v>
+      </c>
+      <c r="C79" s="65" t="n">
+        <v>123000</v>
+      </c>
+      <c r="D79" s="65" t="n">
+        <v>17500</v>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" s="65" t="n">
+        <v>7900</v>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" s="65" t="n">
+        <v>75100</v>
+      </c>
+      <c r="K79" s="65" t="n">
+        <v>22500</v>
+      </c>
+      <c r="L79" s="66">
+        <f>SUM(D79:K79)</f>
+        <v/>
+      </c>
+      <c r="M79" s="67" t="inlineStr">
+        <is>
+          <t>Q2 2025 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="64" t="inlineStr">
+        <is>
+          <t>Q3 2025</t>
+        </is>
+      </c>
+      <c r="B80" s="65" t="n">
+        <v>205600</v>
+      </c>
+      <c r="C80" s="65" t="n">
+        <v>80200</v>
+      </c>
+      <c r="D80" s="65" t="n">
+        <v>17800</v>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" s="65" t="n">
+        <v>4800</v>
+      </c>
+      <c r="G80" s="65" t="n">
+        <v>4500</v>
+      </c>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" s="65" t="n">
+        <v>47100</v>
+      </c>
+      <c r="K80" s="65" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L80" s="66">
+        <f>SUM(D80:K80)</f>
+        <v/>
+      </c>
+      <c r="M80" s="67" t="inlineStr">
+        <is>
+          <t>Q3 2025 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="68" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+      <c r="B81" s="69" t="n">
+        <v>798800</v>
+      </c>
+      <c r="C81" s="85" t="n">
+        <v>274300</v>
+      </c>
+      <c r="D81" s="85" t="n">
+        <v>76600</v>
+      </c>
+      <c r="E81" s="79" t="inlineStr"/>
+      <c r="F81" s="85" t="n">
+        <v>29100</v>
+      </c>
+      <c r="G81" s="85" t="n">
+        <v>7600</v>
+      </c>
+      <c r="H81" s="79" t="inlineStr"/>
+      <c r="I81" s="79" t="inlineStr"/>
+      <c r="J81" s="85" t="n">
+        <v>176100</v>
+      </c>
+      <c r="K81" s="85" t="n">
+        <v>-16100</v>
+      </c>
+      <c r="L81" s="86">
+        <f>SUM(D81:K81)</f>
+        <v/>
+      </c>
+      <c r="M81" s="81" t="inlineStr">
+        <is>
+          <t>FY2025 10-K</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="61" t="inlineStr">
+        <is>
+          <t>Note:</t>
+        </is>
+      </c>
+      <c r="B83" s="87" t="inlineStr">
+        <is>
+          <t>Distributor Termination Fees became a SEPARATE income statement line in 2025 ($246.7M Q3 / $327.5M FY). The 2022/2023 distributor termination charges were inside SG&amp;A — this column reflects that distinction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="62" t="inlineStr">
+        <is>
+          <t>7. GROSS MARGIN DRIVERS -- Qualitative themes (CELH does NOT disclose dollar bridges for GP). "+" = favorable to margin; "-" = unfavorable; blank = not mentioned. Hover cells for verbatim quotes.</t>
+        </is>
+      </c>
+      <c r="B86" s="83" t="n"/>
+      <c r="C86" s="83" t="n"/>
+      <c r="D86" s="83" t="n"/>
+      <c r="E86" s="83" t="n"/>
+      <c r="F86" s="83" t="n"/>
+      <c r="G86" s="83" t="n"/>
+      <c r="H86" s="83" t="n"/>
+      <c r="I86" s="83" t="n"/>
+      <c r="J86" s="83" t="n"/>
+      <c r="K86" s="83" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="84" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B87" s="84" t="inlineStr">
+        <is>
+          <t>GP Margin</t>
+        </is>
+      </c>
+      <c r="C87" s="84" t="inlineStr">
+        <is>
+          <t>YoY Δ pts</t>
+        </is>
+      </c>
+      <c r="D87" s="84" t="inlineStr">
+        <is>
+          <t>Raw Mat / Pkg</t>
+        </is>
+      </c>
+      <c r="E87" s="84" t="inlineStr">
+        <is>
+          <t>Promo Spend</t>
+        </is>
+      </c>
+      <c r="F87" s="84" t="inlineStr">
+        <is>
+          <t>Freight</t>
+        </is>
+      </c>
+      <c r="G87" s="84" t="inlineStr">
+        <is>
+          <t>Channel/Pack Mix</t>
+        </is>
+      </c>
+      <c r="H87" s="84" t="inlineStr">
+        <is>
+          <t>Brand Mix Drag</t>
+        </is>
+      </c>
+      <c r="I87" s="84" t="inlineStr">
+        <is>
+          <t>Inv Step-Up</t>
+        </is>
+      </c>
+      <c r="J87" s="84" t="inlineStr">
+        <is>
+          <t>Tariffs</t>
+        </is>
+      </c>
+      <c r="K87" s="84" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="64" t="inlineStr">
+        <is>
+          <t>Q1 2023</t>
+        </is>
+      </c>
+      <c r="B88" s="72" t="n">
+        <v>0.438</v>
+      </c>
+      <c r="C88" s="72" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="D88" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" s="89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G88" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" s="67" t="inlineStr">
+        <is>
+          <t>Q1 2023 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="64" t="inlineStr">
+        <is>
+          <t>Q2 2023</t>
+        </is>
+      </c>
+      <c r="B89" s="72" t="n">
+        <v>0.488</v>
+      </c>
+      <c r="C89" s="72" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="D89" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" s="67" t="inlineStr">
+        <is>
+          <t>Q2 2023 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="64" t="inlineStr">
+        <is>
+          <t>Q3 2023</t>
+        </is>
+      </c>
+      <c r="B90" s="72" t="n">
+        <v>0.504</v>
+      </c>
+      <c r="C90" s="72" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="D90" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E90" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="F90" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" s="67" t="inlineStr">
+        <is>
+          <t>Q3 2023 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="68" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="B91" s="75" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="C91" s="78" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="D91" s="90" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E91" s="79" t="inlineStr"/>
+      <c r="F91" s="79" t="inlineStr"/>
+      <c r="G91" s="79" t="inlineStr"/>
+      <c r="H91" s="79" t="inlineStr"/>
+      <c r="I91" s="79" t="inlineStr"/>
+      <c r="J91" s="79" t="inlineStr"/>
+      <c r="K91" s="81" t="inlineStr">
+        <is>
+          <t>FY2023 10-K</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="64" t="inlineStr">
+        <is>
+          <t>Q1 2024</t>
+        </is>
+      </c>
+      <c r="B92" s="72" t="n">
+        <v>0.512</v>
+      </c>
+      <c r="C92" s="72" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="D92" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" s="67" t="inlineStr">
+        <is>
+          <t>Q1 2024 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="64" t="inlineStr">
+        <is>
+          <t>Q2 2024</t>
+        </is>
+      </c>
+      <c r="B93" s="72" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="C93" s="72" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D93" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" s="67" t="inlineStr">
+        <is>
+          <t>Q2 2024 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="64" t="inlineStr">
+        <is>
+          <t>Q3 2024</t>
+        </is>
+      </c>
+      <c r="B94" s="72" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="C94" s="72" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="D94" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E94" s="89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F94" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" s="67" t="inlineStr">
+        <is>
+          <t>Q3 2024 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="68" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="B95" s="75" t="n">
+        <v>0.502</v>
+      </c>
+      <c r="C95" s="78" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="D95" s="90" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E95" s="91" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F95" s="90" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G95" s="79" t="inlineStr"/>
+      <c r="H95" s="79" t="inlineStr"/>
+      <c r="I95" s="79" t="inlineStr"/>
+      <c r="J95" s="79" t="inlineStr"/>
+      <c r="K95" s="81" t="inlineStr">
+        <is>
+          <t>FY2024 10-K</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="64" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
+      <c r="B96" s="72" t="n">
+        <v>0.523</v>
+      </c>
+      <c r="C96" s="72" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="D96" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E96" s="89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" s="67" t="inlineStr">
+        <is>
+          <t>Q1 2025 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="64" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
+      <c r="B97" s="72" t="n">
+        <v>0.515</v>
+      </c>
+      <c r="C97" s="72" t="n">
+        <v>-0.005</v>
+      </c>
+      <c r="D97" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="H97" s="89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I97" s="89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" s="67" t="inlineStr">
+        <is>
+          <t>Q2 2025 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="64" t="inlineStr">
+        <is>
+          <t>Q3 2025</t>
+        </is>
+      </c>
+      <c r="B98" s="72" t="n">
+        <v>0.513</v>
+      </c>
+      <c r="C98" s="72" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D98" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E98" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" s="88" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="H98" s="89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" s="89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K98" s="67" t="inlineStr">
+        <is>
+          <t>Q3 2025 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="68" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+      <c r="B99" s="75" t="n">
+        <v>0.504</v>
+      </c>
+      <c r="C99" s="78" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="D99" s="90" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E99" s="90" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="F99" s="79" t="inlineStr"/>
+      <c r="G99" s="90" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="H99" s="91" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I99" s="91" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J99" s="79" t="inlineStr"/>
+      <c r="K99" s="81" t="inlineStr">
+        <is>
+          <t>FY2025 10-K</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="62" t="inlineStr">
+        <is>
+          <t>8. OTHER (EXPENSE) / INCOME WALK -- $ thousands. Pre-Q1 2025 was almost entirely interest income (no debt). Post-Apr 2025: $900M term loan + Rockstar transition agency income create new components.</t>
+        </is>
+      </c>
+      <c r="B102" s="83" t="n"/>
+      <c r="C102" s="83" t="n"/>
+      <c r="D102" s="83" t="n"/>
+      <c r="E102" s="83" t="n"/>
+      <c r="F102" s="83" t="n"/>
+      <c r="G102" s="83" t="n"/>
+      <c r="H102" s="83" t="n"/>
+      <c r="I102" s="83" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="84" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B103" s="84" t="inlineStr">
+        <is>
+          <t>Total Other Inc/(Exp)</t>
+        </is>
+      </c>
+      <c r="C103" s="84" t="inlineStr">
+        <is>
+          <t>YoY Δ</t>
+        </is>
+      </c>
+      <c r="D103" s="84" t="inlineStr">
+        <is>
+          <t>Interest Income Δ</t>
+        </is>
+      </c>
+      <c r="E103" s="84" t="inlineStr">
+        <is>
+          <t>Interest Expense Δ</t>
+        </is>
+      </c>
+      <c r="F103" s="84" t="inlineStr">
+        <is>
+          <t>Rockstar Agency Inc Δ</t>
+        </is>
+      </c>
+      <c r="G103" s="84" t="inlineStr">
+        <is>
+          <t>FX / Other Δ</t>
+        </is>
+      </c>
+      <c r="H103" s="84" t="inlineStr"/>
+      <c r="I103" s="84" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="64" t="inlineStr">
+        <is>
+          <t>Q1 2023</t>
+        </is>
+      </c>
+      <c r="B104" s="65" t="n">
+        <v>4900</v>
+      </c>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
+      <c r="I104" s="67" t="inlineStr">
+        <is>
+          <t>Q1 2023 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="64" t="inlineStr">
+        <is>
+          <t>Q2 2023</t>
+        </is>
+      </c>
+      <c r="B105" s="65" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr"/>
+      <c r="I105" s="67" t="inlineStr">
+        <is>
+          <t>Q2 2023 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="64" t="inlineStr">
+        <is>
+          <t>Q3 2023</t>
+        </is>
+      </c>
+      <c r="B106" s="65" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="I106" s="67" t="inlineStr">
+        <is>
+          <t>Q3 2023 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="68" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="B107" s="69" t="n">
+        <v>25400</v>
+      </c>
+      <c r="C107" s="85" t="n">
+        <v>20300</v>
+      </c>
+      <c r="D107" s="85" t="n">
+        <v>20300</v>
+      </c>
+      <c r="E107" s="79" t="inlineStr"/>
+      <c r="F107" s="79" t="inlineStr"/>
+      <c r="G107" s="79" t="inlineStr"/>
+      <c r="H107" s="79" t="n"/>
+      <c r="I107" s="81" t="inlineStr">
+        <is>
+          <t>FY2023 10-K</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="64" t="inlineStr">
+        <is>
+          <t>Q1 2024</t>
+        </is>
+      </c>
+      <c r="B108" s="65" t="n">
+        <v>9300</v>
+      </c>
+      <c r="C108" s="65" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D108" s="65" t="n">
+        <v>4400</v>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
+      <c r="I108" s="67" t="inlineStr">
+        <is>
+          <t>Q1 2024 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="64" t="inlineStr">
+        <is>
+          <t>Q2 2024</t>
+        </is>
+      </c>
+      <c r="B109" s="65" t="n">
+        <v>10400</v>
+      </c>
+      <c r="C109" s="65" t="n">
+        <v>5800</v>
+      </c>
+      <c r="D109" s="65" t="n">
+        <v>5800</v>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
+      <c r="I109" s="67" t="inlineStr">
+        <is>
+          <t>Q2 2024 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="64" t="inlineStr">
+        <is>
+          <t>Q3 2024</t>
+        </is>
+      </c>
+      <c r="B110" s="65" t="n">
+        <v>11400</v>
+      </c>
+      <c r="C110" s="65" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D110" s="65" t="n">
+        <v>4400</v>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="I110" s="67" t="inlineStr">
+        <is>
+          <t>Q3 2024 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="68" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="B111" s="69" t="n">
+        <v>39300</v>
+      </c>
+      <c r="C111" s="85" t="n">
+        <v>13900</v>
+      </c>
+      <c r="D111" s="85" t="n">
+        <v>13900</v>
+      </c>
+      <c r="E111" s="79" t="inlineStr"/>
+      <c r="F111" s="79" t="inlineStr"/>
+      <c r="G111" s="79" t="inlineStr"/>
+      <c r="H111" s="79" t="n"/>
+      <c r="I111" s="81" t="inlineStr">
+        <is>
+          <t>FY2024 10-K</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="64" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
+      <c r="B112" s="65" t="n">
+        <v>9000</v>
+      </c>
+      <c r="C112" s="65" t="n">
+        <v>-300</v>
+      </c>
+      <c r="D112" s="65" t="n">
+        <v>-300</v>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
+      <c r="I112" s="67" t="inlineStr">
+        <is>
+          <t>Q1 2025 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="64" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr"/>
+      <c r="C113" t="inlineStr"/>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
+      <c r="I113" s="67" t="inlineStr">
+        <is>
+          <t>Q2 2025 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="64" t="inlineStr">
+        <is>
+          <t>Q3 2025</t>
+        </is>
+      </c>
+      <c r="B114" s="65" t="n">
+        <v>-8000</v>
+      </c>
+      <c r="C114" s="65" t="n">
+        <v>-19400</v>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" s="65" t="n">
+        <v>-18200</v>
+      </c>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+      <c r="I114" s="67" t="inlineStr">
+        <is>
+          <t>Q3 2025 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="68" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+      <c r="B115" s="69" t="n">
+        <v>-16000</v>
+      </c>
+      <c r="C115" s="85" t="n">
+        <v>-55300</v>
+      </c>
+      <c r="D115" s="85" t="n">
+        <v>-18200</v>
+      </c>
+      <c r="E115" s="85" t="n">
+        <v>-49000</v>
+      </c>
+      <c r="F115" s="85" t="n">
+        <v>12600</v>
+      </c>
+      <c r="G115" s="85" t="n">
+        <v>-700</v>
+      </c>
+      <c r="H115" s="79" t="n"/>
+      <c r="I115" s="81" t="inlineStr">
+        <is>
+          <t>FY2025 10-K</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="5">
+    <mergeCell ref="A68:M68"/>
+    <mergeCell ref="A86:K86"/>
+    <mergeCell ref="A102:I102"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="B83:M83"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
vault backup: 2026-05-05 18:09:29
</commit_message>
<xml_diff>
--- a/Knowledge/Model Outputs/CELH/CELH_model.xlsx
+++ b/Knowledge/Model Outputs/CELH/CELH_model.xlsx
@@ -22,9 +22,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF DRIVERS" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Driver" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
-  <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
-  </externalReferences>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
 </workbook>
@@ -2746,100 +2743,6 @@
 </comments>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Male"/>
-      <sheetName val="Female"/>
-      <sheetName val="Growth by Race"/>
-      <sheetName val="SNAP Base Case"/>
-      <sheetName val="SNAP Recession"/>
-      <sheetName val="TAM &amp; Brand Share"/>
-      <sheetName val="Demographic Data"/>
-      <sheetName val="National Summary"/>
-      <sheetName val="Snap Usage"/>
-      <sheetName val="Energy Drink Consumption"/>
-      <sheetName val="COVID SNAP Impact"/>
-      <sheetName val="SNAP Ban Impact"/>
-      <sheetName val="Total Market_Celsius Output"/>
-      <sheetName val="GLP-1 Share Impact"/>
-      <sheetName val="Cohort Aging Model"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11">
-        <row r="33">
-          <cell r="D33">
-            <v>113.36679374999999</v>
-          </cell>
-          <cell r="E33">
-            <v>115.23408749999999</v>
-          </cell>
-          <cell r="F33">
-            <v>117.18209999999999</v>
-          </cell>
-          <cell r="G33">
-            <v>119.20544999999998</v>
-          </cell>
-          <cell r="H33">
-            <v>121.31489999999998</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="D34">
-            <v>21.448251138864567</v>
-          </cell>
-          <cell r="E34">
-            <v>22.038453748142427</v>
-          </cell>
-          <cell r="F34">
-            <v>22.883234775552697</v>
-          </cell>
-          <cell r="G34">
-            <v>23.742292271505907</v>
-          </cell>
-          <cell r="H34">
-            <v>24.619670147589872</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13">
-        <row r="22">
-          <cell r="C22">
-            <v>68.911914840907883</v>
-          </cell>
-          <cell r="D22">
-            <v>82.534532405551772</v>
-          </cell>
-          <cell r="E22">
-            <v>95.991953898519981</v>
-          </cell>
-          <cell r="F22">
-            <v>110.09995327741292</v>
-          </cell>
-          <cell r="G22">
-            <v>124.02447744606826</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="14"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -33997,24 +33900,19 @@
       <c r="F6" s="29" t="n"/>
       <c r="G6" s="29" t="n"/>
       <c r="H6" s="30">
-        <f>'[1]SNAP Ban Impact'!D33</f>
-        <v/>
+        <v>113.36679374999999</v>
       </c>
       <c r="I6" s="30">
-        <f>'[1]SNAP Ban Impact'!E33</f>
-        <v/>
+        <v>115.23408749999999</v>
       </c>
       <c r="J6" s="30">
-        <f>'[1]SNAP Ban Impact'!F33</f>
-        <v/>
+        <v>117.18209999999999</v>
       </c>
       <c r="K6" s="30">
-        <f>'[1]SNAP Ban Impact'!G33</f>
-        <v/>
+        <v>119.20544999999998</v>
       </c>
       <c r="L6" s="30">
-        <f>'[1]SNAP Ban Impact'!H33</f>
-        <v/>
+        <v>121.31489999999998</v>
       </c>
       <c r="M6" s="31" t="n"/>
       <c r="N6" s="32" t="n"/>
@@ -34846,24 +34744,19 @@
       <c r="F25" s="43" t="n"/>
       <c r="G25" s="43" t="n"/>
       <c r="H25" s="44">
-        <f>'[1]GLP-1 Share Impact'!C22</f>
-        <v/>
+        <v>68.911914840907883</v>
       </c>
       <c r="I25" s="44">
-        <f>'[1]GLP-1 Share Impact'!D22</f>
-        <v/>
+        <v>82.534532405551772</v>
       </c>
       <c r="J25" s="44">
-        <f>'[1]GLP-1 Share Impact'!E22</f>
-        <v/>
+        <v>95.991953898519981</v>
       </c>
       <c r="K25" s="44">
-        <f>'[1]GLP-1 Share Impact'!F22</f>
-        <v/>
+        <v>110.09995327741292</v>
       </c>
       <c r="L25" s="44">
-        <f>'[1]GLP-1 Share Impact'!G22</f>
-        <v/>
+        <v>124.02447744606826</v>
       </c>
       <c r="M25" s="28" t="n"/>
       <c r="N25" s="32" t="n"/>
@@ -34881,24 +34774,19 @@
       <c r="F26" s="43" t="n"/>
       <c r="G26" s="43" t="n"/>
       <c r="H26" s="44">
-        <f>'[1]SNAP Ban Impact'!D34</f>
-        <v/>
+        <v>21.448251138864567</v>
       </c>
       <c r="I26" s="44">
-        <f>'[1]SNAP Ban Impact'!E34</f>
-        <v/>
+        <v>22.038453748142427</v>
       </c>
       <c r="J26" s="44">
-        <f>'[1]SNAP Ban Impact'!F34</f>
-        <v/>
+        <v>22.883234775552697</v>
       </c>
       <c r="K26" s="44">
-        <f>'[1]SNAP Ban Impact'!G34</f>
-        <v/>
+        <v>23.742292271505907</v>
       </c>
       <c r="L26" s="44">
-        <f>'[1]SNAP Ban Impact'!H34</f>
-        <v/>
+        <v>24.619670147589872</v>
       </c>
       <c r="M26" s="28" t="n"/>
       <c r="N26" s="32" t="n"/>

</xml_diff>